<commit_message>
Added new Donate actions to turn Coins into Honor
with Court and Undermarket versions
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3352" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B4FEFF1-680E-49BA-B0DD-DB1965E21A14}"/>
+  <xr:revisionPtr revIDLastSave="3365" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3914F54C-9B9D-401F-A4C7-EB6EA0DFAF21}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="513">
   <si>
     <t>Standard Card</t>
   </si>
@@ -1574,6 +1574,15 @@
   </si>
   <si>
     <t>Send Troops up to Leader's Level to the Battlefield</t>
+  </si>
+  <si>
+    <t>Donate</t>
+  </si>
+  <si>
+    <t>Pay up to Leader's Level Coins to the Royal Bank and immediately gain half the Coins paid in Honor</t>
+  </si>
+  <si>
+    <t>Pay up to Leader's Level Coins to the Royal Bank and immediately gain half the Coins paid in Honor. Immediately demote the Leader used.</t>
   </si>
 </sst>
 </file>
@@ -3684,6 +3693,10 @@
 </FeaturePropertyBags>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -5117,7 +5130,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D195C1D-DB02-1743-BBD2-99104C1FFD33}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -5501,15 +5514,15 @@
       <c r="H16" s="42"/>
       <c r="I16" s="45"/>
     </row>
-    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>259</v>
+        <v>510</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>260</v>
+        <v>512</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
@@ -5518,12 +5531,12 @@
       <c r="H17" s="42"/>
       <c r="I17" s="45"/>
     </row>
-    <row r="18" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="37" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>261</v>
@@ -5535,12 +5548,12 @@
       <c r="H18" s="42"/>
       <c r="I18" s="45"/>
     </row>
-    <row r="19" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B19" s="35" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>261</v>
@@ -5554,10 +5567,10 @@
     </row>
     <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
-        <v>480</v>
+        <v>264</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>481</v>
+        <v>265</v>
       </c>
       <c r="C20" s="38" t="s">
         <v>261</v>
@@ -5571,10 +5584,10 @@
     </row>
     <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
-        <v>251</v>
+        <v>480</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>267</v>
+        <v>481</v>
       </c>
       <c r="C21" s="38" t="s">
         <v>261</v>
@@ -5588,10 +5601,10 @@
     </row>
     <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="37" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C22" s="38" t="s">
         <v>261</v>
@@ -5603,22 +5616,56 @@
       <c r="H22" s="42"/>
       <c r="I22" s="45"/>
     </row>
-    <row r="23" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="39" t="s">
+    <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>268</v>
+      </c>
+      <c r="C23" s="38" t="s">
+        <v>261</v>
+      </c>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="45"/>
+    </row>
+    <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="39" t="s">
         <v>257</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B24" s="40" t="s">
         <v>269</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C24" s="41" t="s">
         <v>261</v>
       </c>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="43"/>
-      <c r="I23" s="46"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="45"/>
+    </row>
+    <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="39" t="s">
+        <v>510</v>
+      </c>
+      <c r="B25" s="40" t="s">
+        <v>511</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>261</v>
+      </c>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="43"/>
+      <c r="I25" s="46"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7419,7 +7466,7 @@
         <v>Elite Troops</v>
       </c>
       <c r="BD1" s="80" t="str">
-        <f t="shared" ref="BD1:BM2" si="2">U1</f>
+        <f t="shared" ref="BD1:BI2" si="2">U1</f>
         <v>Bazaar</v>
       </c>
       <c r="BE1" s="78" t="str">

</xml_diff>

<commit_message>
Added investments and laws for new Donate action
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3365" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3914F54C-9B9D-401F-A4C7-EB6EA0DFAF21}"/>
+  <xr:revisionPtr revIDLastSave="3394" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BF81C7C-8420-4A84-91BD-B49F52503D96}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="520">
   <si>
     <t>Standard Card</t>
   </si>
@@ -1513,9 +1513,6 @@
     <t>Gain $L3 additional Coins from outside the Royal Bank when winning a Sue</t>
   </si>
   <si>
-    <t xml:space="preserve">   </t>
-  </si>
-  <si>
     <t>Move the Law $L6 additional places forward in the queue during Prioritize</t>
   </si>
   <si>
@@ -1583,6 +1580,30 @@
   </si>
   <si>
     <t>Pay up to Leader's Level Coins to the Royal Bank and immediately gain half the Coins paid in Honor. Immediately demote the Leader used.</t>
+  </si>
+  <si>
+    <t>Convert $L3 additional Coins during Court Donate</t>
+  </si>
+  <si>
+    <t>Convert $L3 additional Coins during Undermarket Donate</t>
+  </si>
+  <si>
+    <t>Abusive Power</t>
+  </si>
+  <si>
+    <t>Soup Kitchens</t>
+  </si>
+  <si>
+    <t>At least $L6 Players must use Deploy or all Players suffer sanctions on Donate</t>
+  </si>
+  <si>
+    <t>No more than $L6 Players may use Deploy or all Players suffer sanctions on Donate</t>
+  </si>
+  <si>
+    <t>Stalled Front</t>
+  </si>
+  <si>
+    <t>Quality Strength</t>
   </si>
 </sst>
 </file>
@@ -4094,7 +4115,7 @@
         <v>487</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>16</v>
@@ -4262,7 +4283,7 @@
         <v>55</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
@@ -4351,7 +4372,7 @@
         <v>74</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>488</v>
@@ -4389,7 +4410,7 @@
         <v>82</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>83</v>
@@ -4481,7 +4502,7 @@
         <v>104</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>106</v>
@@ -4496,7 +4517,7 @@
         <v>108</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
@@ -4518,9 +4539,7 @@
       <c r="E19" s="15" t="s">
         <v>458</v>
       </c>
-      <c r="F19" s="23" t="s">
-        <v>489</v>
-      </c>
+      <c r="F19" s="23"/>
       <c r="G19" s="25"/>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
@@ -4800,15 +4819,19 @@
       <c r="C32" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="D32" s="6"/>
-      <c r="E32" s="16"/>
+      <c r="D32" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>516</v>
+      </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
       <c r="H32" s="4"/>
       <c r="I32" s="3"/>
       <c r="J32" s="4"/>
     </row>
-    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>168</v>
       </c>
@@ -4818,8 +4841,12 @@
       <c r="C33" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="D33" s="6"/>
-      <c r="E33" s="16"/>
+      <c r="D33" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>517</v>
+      </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
       <c r="H33" s="4"/>
@@ -4834,7 +4861,7 @@
         <v>172</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="16"/>
@@ -4885,10 +4912,10 @@
         <v>177</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -4898,12 +4925,16 @@
       <c r="I37" s="3"/>
       <c r="J37" s="4"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="16"/>
+      <c r="B38" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>512</v>
+      </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
       <c r="F38" s="6"/>
@@ -4912,12 +4943,16 @@
       <c r="I38" s="3"/>
       <c r="J38" s="4"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="B39" s="6"/>
-      <c r="C39" s="16"/>
+      <c r="B39" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>513</v>
+      </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
       <c r="F39" s="6"/>
@@ -5178,7 +5213,7 @@
         <v>202</v>
       </c>
       <c r="B2" s="48" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C2" s="49" t="s">
         <v>203</v>
@@ -5248,7 +5283,7 @@
         <v>217</v>
       </c>
       <c r="F4" s="42" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="G4" s="42" t="s">
         <v>218</v>
@@ -5308,7 +5343,7 @@
         <v>451</v>
       </c>
       <c r="H6" s="42" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="I6" s="45"/>
     </row>
@@ -5323,7 +5358,7 @@
         <v>203</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E7" s="42" t="s">
         <v>331</v>
@@ -5394,7 +5429,7 @@
         <v>203</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="E10" s="42" t="s">
         <v>243</v>
@@ -5409,14 +5444,14 @@
         <v>244</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>203</v>
       </c>
       <c r="D11" s="42"/>
       <c r="E11" s="42" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F11" s="42"/>
       <c r="G11" s="42"/>
@@ -5516,10 +5551,10 @@
     </row>
     <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C17" s="38" t="s">
         <v>253</v>
@@ -5652,10 +5687,10 @@
     </row>
     <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39" t="s">
+        <v>509</v>
+      </c>
+      <c r="B25" s="40" t="s">
         <v>510</v>
-      </c>
-      <c r="B25" s="40" t="s">
-        <v>511</v>
       </c>
       <c r="C25" s="41" t="s">
         <v>261</v>
@@ -9049,10 +9084,10 @@
         <v>465</v>
       </c>
       <c r="F1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H1" t="s">
         <v>466</v>
@@ -9061,7 +9096,7 @@
         <v>467</v>
       </c>
       <c r="J1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="K1" t="s">
         <v>468</v>
@@ -9094,7 +9129,7 @@
         <v>477</v>
       </c>
       <c r="U1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added new Scheme cards to affect Queue more directly
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3394" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BF81C7C-8420-4A84-91BD-B49F52503D96}"/>
+  <xr:revisionPtr revIDLastSave="3399" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FD2E225-2670-451F-AA6F-E1868A59396C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="524">
   <si>
     <t>Standard Card</t>
   </si>
@@ -1604,6 +1604,18 @@
   </si>
   <si>
     <t>Quality Strength</t>
+  </si>
+  <si>
+    <t>Move one of your Laws $D6 spaces back in the Queue</t>
+  </si>
+  <si>
+    <t>Move $D6 of your Laws one space back in the Queue</t>
+  </si>
+  <si>
+    <t>Rallied Opposition</t>
+  </si>
+  <si>
+    <t>Waning Support</t>
   </si>
 </sst>
 </file>
@@ -4539,8 +4551,12 @@
       <c r="E19" s="15" t="s">
         <v>458</v>
       </c>
-      <c r="F19" s="23"/>
-      <c r="G19" s="25"/>
+      <c r="F19" s="23" t="s">
+        <v>522</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>520</v>
+      </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
       <c r="J19" s="4"/>
@@ -4561,8 +4577,12 @@
       <c r="E20" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="7"/>
+      <c r="F20" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>521</v>
+      </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
       <c r="J20" s="4"/>

</xml_diff>

<commit_message>
Changed all Laws to be $L6
The few that were $L3 didn't make sense to have such restrictions
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3399" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FD2E225-2670-451F-AA6F-E1868A59396C}"/>
+  <xr:revisionPtr revIDLastSave="3403" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5D1A1E9-6FEE-4738-94CE-64DDE07B3441}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -919,12 +919,6 @@
     <t>Persian</t>
   </si>
   <si>
-    <t>At least $L3 Players must use Court Actions or all Players suffer sanctions on Flatter</t>
-  </si>
-  <si>
-    <t>No more than $L3 Players may use Court Actions or all Players suffer sanctions on Flatter</t>
-  </si>
-  <si>
     <t>Law Cards</t>
   </si>
   <si>
@@ -1492,12 +1486,6 @@
     <t>Move a Law Leader's Level places forward in the queue, but never to become the Deliberated Law</t>
   </si>
   <si>
-    <t>At least $L3 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
-  </si>
-  <si>
-    <t>No more than $L3 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
-  </si>
-  <si>
     <t>Spend $L3 fewer Cards per Coin when Monetizing in the Undermarket</t>
   </si>
   <si>
@@ -1616,6 +1604,18 @@
   </si>
   <si>
     <t>Waning Support</t>
+  </si>
+  <si>
+    <t>At least $L6 Players must use Court Actions or all Players suffer sanctions on Flatter</t>
+  </si>
+  <si>
+    <t>No more than $L6 Players may use Court Actions or all Players suffer sanctions on Flatter</t>
+  </si>
+  <si>
+    <t>At least $L6 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
+  </si>
+  <si>
+    <t>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
   </si>
 </sst>
 </file>
@@ -4124,10 +4124,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>16</v>
@@ -4159,7 +4159,7 @@
         <v>23</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>24</v>
@@ -4185,7 +4185,7 @@
         <v>29</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>30</v>
@@ -4260,10 +4260,10 @@
         <v>48</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>49</v>
@@ -4289,13 +4289,13 @@
         <v>54</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>55</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
@@ -4312,10 +4312,10 @@
         <v>58</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>59</v>
@@ -4341,7 +4341,7 @@
         <v>64</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>65</v>
@@ -4384,10 +4384,10 @@
         <v>74</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>76</v>
@@ -4413,7 +4413,7 @@
         <v>80</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>81</v>
@@ -4422,7 +4422,7 @@
         <v>82</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>83</v>
@@ -4514,7 +4514,7 @@
         <v>104</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>106</v>
@@ -4523,13 +4523,13 @@
         <v>107</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>108</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
@@ -4549,13 +4549,13 @@
         <v>112</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
@@ -4578,10 +4578,10 @@
         <v>117</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
@@ -4623,7 +4623,7 @@
         <v>126</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="7"/>
@@ -4680,10 +4680,10 @@
         <v>137</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>139</v>
@@ -4702,16 +4702,16 @@
         <v>141</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>142</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>482</v>
+        <v>522</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4733,7 +4733,7 @@
         <v>146</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>483</v>
+        <v>523</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4755,7 +4755,7 @@
         <v>150</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>291</v>
+        <v>520</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4777,7 +4777,7 @@
         <v>154</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>292</v>
+        <v>521</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -4840,10 +4840,10 @@
         <v>167</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -4862,10 +4862,10 @@
         <v>170</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -4881,7 +4881,7 @@
         <v>172</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="16"/>
@@ -4914,10 +4914,10 @@
         <v>176</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -4932,10 +4932,10 @@
         <v>177</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -4950,10 +4950,10 @@
         <v>178</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -4968,10 +4968,10 @@
         <v>179</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -5219,7 +5219,7 @@
         <v>199</v>
       </c>
       <c r="G1" s="54" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="H1" s="54" t="s">
         <v>200</v>
@@ -5233,7 +5233,7 @@
         <v>202</v>
       </c>
       <c r="B2" s="48" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="C2" s="49" t="s">
         <v>203</v>
@@ -5259,16 +5259,16 @@
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C3" s="38" t="s">
         <v>203</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E3" s="42" t="s">
         <v>210</v>
@@ -5280,7 +5280,7 @@
         <v>212</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="I3" s="42" t="s">
         <v>213</v>
@@ -5303,7 +5303,7 @@
         <v>217</v>
       </c>
       <c r="F4" s="42" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="G4" s="42" t="s">
         <v>218</v>
@@ -5318,7 +5318,7 @@
         <v>220</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C5" s="38" t="s">
         <v>203</v>
@@ -5333,10 +5333,10 @@
         <v>223</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="I5" s="45"/>
     </row>
@@ -5360,10 +5360,10 @@
         <v>228</v>
       </c>
       <c r="G6" s="42" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="H6" s="42" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="I6" s="45"/>
     </row>
@@ -5378,13 +5378,13 @@
         <v>203</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G7" s="42" t="s">
         <v>231</v>
@@ -5406,7 +5406,7 @@
         <v>234</v>
       </c>
       <c r="E8" s="42" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F8" s="42" t="s">
         <v>235</v>
@@ -5449,7 +5449,7 @@
         <v>203</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="E10" s="42" t="s">
         <v>243</v>
@@ -5464,14 +5464,14 @@
         <v>244</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>203</v>
       </c>
       <c r="D11" s="42"/>
       <c r="E11" s="42" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="F11" s="42"/>
       <c r="G11" s="42"/>
@@ -5571,10 +5571,10 @@
     </row>
     <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="C17" s="38" t="s">
         <v>253</v>
@@ -5639,10 +5639,10 @@
     </row>
     <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C21" s="38" t="s">
         <v>261</v>
@@ -5707,10 +5707,10 @@
     </row>
     <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="B25" s="40" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="C25" s="41" t="s">
         <v>261</v>
@@ -5757,7 +5757,7 @@
         <v>275</v>
       </c>
       <c r="I1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -5783,7 +5783,7 @@
         <v>156</v>
       </c>
       <c r="I2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -5809,7 +5809,7 @@
         <v>169</v>
       </c>
       <c r="I3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -5835,7 +5835,7 @@
         <v>148</v>
       </c>
       <c r="I4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="I5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5887,7 +5887,7 @@
         <v>154</v>
       </c>
       <c r="I6" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5898,7 +5898,7 @@
         <v>282</v>
       </c>
       <c r="C7" s="74" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D7" t="s">
         <v>283</v>
@@ -5913,12 +5913,12 @@
         <v>201</v>
       </c>
       <c r="I7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="95" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B8" s="95" t="s">
         <v>273</v>
@@ -5939,12 +5939,12 @@
         <v>272</v>
       </c>
       <c r="I8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="63" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B9" s="63" t="s">
         <v>274</v>
@@ -5967,7 +5967,7 @@
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="96" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B10" s="96" t="s">
         <v>272</v>
@@ -5990,205 +5990,205 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>389</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -6196,111 +6196,111 @@
     </row>
     <row r="23" spans="1:9" ht="225" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>403</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="255" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="D24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>409</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="345" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="F26" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>418</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="255" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>428</v>
-      </c>
       <c r="F27" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>422</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="195" x14ac:dyDescent="0.25">
@@ -6308,63 +6308,63 @@
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>425</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>427</v>
       </c>
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>430</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>229</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>264</v>
       </c>
       <c r="I30" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -6376,65 +6376,65 @@
         <v>245</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>241</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>202</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="2"/>
       <c r="D34" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -6450,10 +6450,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>264</v>
@@ -6467,7 +6467,7 @@
     </row>
     <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>245</v>
@@ -6476,19 +6476,19 @@
         <v>241</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="I37" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -6506,35 +6506,35 @@
         <v>245</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="I38" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>248</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>245</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="I39" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -6542,14 +6542,14 @@
       <c r="B40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="G40" s="2"/>
       <c r="I40" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -6589,19 +6589,19 @@
     </row>
     <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>264</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>241</v>
@@ -6609,47 +6609,47 @@
     </row>
     <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>266</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>232</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="49" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>229</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="50" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2" t="s">
@@ -6668,16 +6668,16 @@
         <v>229</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>264</v>
@@ -6688,44 +6688,44 @@
         <v>241</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>241</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>245</v>
@@ -6734,20 +6734,20 @@
         <v>202</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
@@ -6763,22 +6763,22 @@
     </row>
     <row r="58" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>236</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
@@ -6789,16 +6789,16 @@
         <v>264</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>245</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
@@ -6812,28 +6812,28 @@
         <v>245</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>245</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B61" s="3"/>
       <c r="C61" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>248</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>245</v>
@@ -6902,7 +6902,7 @@
         <v>248</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D3" s="30" t="s">
         <v>244</v>
@@ -6954,7 +6954,7 @@
         <v>262</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D1" s="30" t="s">
         <v>264</v>
@@ -8133,19 +8133,19 @@
       </c>
       <c r="Y4" s="85" t="str">
         <f>Cards!E26</f>
-        <v>At least $L3 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
+        <v>At least $L6 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
       </c>
       <c r="Z4" s="83" t="str">
         <f>Cards!E27</f>
-        <v>No more than $L3 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
+        <v>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
       </c>
       <c r="AA4" s="85" t="str">
         <f>Cards!E28</f>
-        <v>At least $L3 Players must use Court Actions or all Players suffer sanctions on Flatter</v>
+        <v>At least $L6 Players must use Court Actions or all Players suffer sanctions on Flatter</v>
       </c>
       <c r="AB4" s="83" t="str">
         <f>Cards!E29</f>
-        <v>No more than $L3 Players may use Court Actions or all Players suffer sanctions on Flatter</v>
+        <v>No more than $L6 Players may use Court Actions or all Players suffer sanctions on Flatter</v>
       </c>
       <c r="AC4" s="85" t="str">
         <f>Cards!E30</f>
@@ -8253,19 +8253,19 @@
       </c>
       <c r="BC4" s="83" t="str">
         <f t="shared" ref="BC4" si="28">Y4</f>
-        <v>At least $L3 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
+        <v>At least $L6 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
       </c>
       <c r="BD4" s="85" t="str">
         <f t="shared" ref="BD4" si="29">Z4</f>
-        <v>No more than $L3 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
+        <v>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</v>
       </c>
       <c r="BE4" s="83" t="str">
         <f t="shared" ref="BE4" si="30">AA4</f>
-        <v>At least $L3 Players must use Court Actions or all Players suffer sanctions on Flatter</v>
+        <v>At least $L6 Players must use Court Actions or all Players suffer sanctions on Flatter</v>
       </c>
       <c r="BF4" s="85" t="str">
         <f t="shared" ref="BF4" si="31">AB4</f>
-        <v>No more than $L3 Players may use Court Actions or all Players suffer sanctions on Flatter</v>
+        <v>No more than $L6 Players may use Court Actions or all Players suffer sanctions on Flatter</v>
       </c>
       <c r="BG4" s="83" t="str">
         <f t="shared" ref="BG4" si="32">AC4</f>
@@ -8781,31 +8781,31 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C1" t="s">
+        <v>311</v>
+      </c>
+      <c r="D1" t="s">
         <v>312</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>313</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>314</v>
-      </c>
-      <c r="E1" t="s">
-        <v>315</v>
-      </c>
-      <c r="F1" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B2">
         <f>30*2</f>
         <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D2">
         <v>27.7</v>
@@ -8813,14 +8813,14 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B3">
         <f>34*2</f>
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D3">
         <v>27.7</v>
@@ -8828,14 +8828,14 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B4">
         <f>18*3</f>
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D4">
         <v>30.75</v>
@@ -8843,222 +8843,222 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B5">
         <f>2*6+6*6</f>
         <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B6">
         <f>1*6+10*6</f>
         <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B7">
         <f>10*6+10</f>
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E7" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B8">
         <f>2*8*6</f>
         <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B9">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B10">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E10" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B11">
         <f>(30*6-B10)/5</f>
         <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E11" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B12">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C12" t="s">
+        <v>316</v>
+      </c>
+      <c r="E12" t="s">
         <v>318</v>
-      </c>
-      <c r="E12" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B13">
         <f>(15*6-B12)/5</f>
         <v>12</v>
       </c>
       <c r="C13" t="s">
+        <v>316</v>
+      </c>
+      <c r="E13" t="s">
         <v>318</v>
-      </c>
-      <c r="E13" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B18">
         <f>10*6</f>
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B19">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B20">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -9089,67 +9089,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B1" t="s">
+        <v>460</v>
+      </c>
+      <c r="C1" t="s">
         <v>461</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>462</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>463</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>490</v>
+      </c>
+      <c r="G1" t="s">
+        <v>489</v>
+      </c>
+      <c r="H1" t="s">
         <v>464</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>465</v>
       </c>
-      <c r="F1" t="s">
-        <v>494</v>
-      </c>
-      <c r="G1" t="s">
-        <v>493</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
+        <v>487</v>
+      </c>
+      <c r="K1" t="s">
         <v>466</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>467</v>
       </c>
-      <c r="J1" t="s">
-        <v>491</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>468</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>469</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>470</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>471</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>472</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>473</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>474</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>475</v>
       </c>
-      <c r="S1" t="s">
-        <v>476</v>
-      </c>
-      <c r="T1" t="s">
-        <v>477</v>
-      </c>
       <c r="U1" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated cards and actions from playtest feedback
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3403" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5D1A1E9-6FEE-4738-94CE-64DDE07B3441}"/>
+  <xr:revisionPtr revIDLastSave="3436" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37185AFA-472E-4E99-AEE5-A6FF8A9012A1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="526">
   <si>
     <t>Standard Card</t>
   </si>
@@ -346,9 +346,6 @@
     <t>Undeniable Advisors</t>
   </si>
   <si>
-    <t>You may repeat Court Actions with level 7 - $L6 Leaders</t>
-  </si>
-  <si>
     <t>Chattering Windbags</t>
   </si>
   <si>
@@ -1549,18 +1546,12 @@
     <t>Exchange Alliance tokens with a Player of your choice. The chosen Player must place a Leader on this space. Both players then exchange up to the lowest LL tokens.</t>
   </si>
   <si>
-    <t>If Greeks are victorious, give remaining attacking Greeks to the player who deployed the fewest Troops (break ties with deployment order then with a Tie Trial or agreement). That player destroys 1 Troop per attacking Greek or 1 investment at level $D6 if they have no Troops.</t>
-  </si>
-  <si>
     <t>Add 1 Coin per Player to Royal Bank</t>
   </si>
   <si>
     <t>Give 1 Troop per Player to each player</t>
   </si>
   <si>
-    <t>Send Troops up to Leader's Level to the Battlefield</t>
-  </si>
-  <si>
     <t>Donate</t>
   </si>
   <si>
@@ -1616,6 +1607,21 @@
   </si>
   <si>
     <t>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You may repeat Court Actions with level 7 - $L6 (or higher) Leaders </t>
+  </si>
+  <si>
+    <t>Send Troops up to Leader's Level to the Battlefield and gain half Troops in Coins</t>
+  </si>
+  <si>
+    <t>You may repeat Undermarket Actions at double the penalty</t>
+  </si>
+  <si>
+    <t>Painful Progress</t>
+  </si>
+  <si>
+    <t>If Greeks are victorious, give remaining attacking Greeks to the player who deployed the fewest Troops (break ties with deployment order then with a Tie Trial or agreement). That player destroys 1 Troop per attacking Greek or downgrades 1 investment by $D6 levels if they have no Troops.</t>
   </si>
 </sst>
 </file>
@@ -2540,7 +2546,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2820,6 +2826,9 @@
       </extLst>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
@@ -4124,10 +4133,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>16</v>
@@ -4159,7 +4168,7 @@
         <v>23</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>24</v>
@@ -4185,7 +4194,7 @@
         <v>29</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>30</v>
@@ -4260,10 +4269,10 @@
         <v>48</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>49</v>
@@ -4289,13 +4298,13 @@
         <v>54</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>55</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
@@ -4312,10 +4321,10 @@
         <v>58</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>59</v>
@@ -4341,7 +4350,7 @@
         <v>64</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>65</v>
@@ -4384,10 +4393,10 @@
         <v>74</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>76</v>
@@ -4413,7 +4422,7 @@
         <v>80</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>81</v>
@@ -4422,7 +4431,7 @@
         <v>82</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>83</v>
@@ -4491,16 +4500,16 @@
         <v>99</v>
       </c>
       <c r="C17" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="F17" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>97</v>
@@ -4511,25 +4520,25 @@
     </row>
     <row r="18" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C18" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="15" t="s">
+        <v>454</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="E18" s="15" t="s">
-        <v>455</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="G18" s="7" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
@@ -4537,25 +4546,25 @@
     </row>
     <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="C19" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="D19" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="E19" s="15" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
@@ -4563,25 +4572,25 @@
     </row>
     <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="D20" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E20" s="15" t="s">
-        <v>117</v>
-      </c>
       <c r="F20" s="6" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
@@ -4589,19 +4598,19 @@
     </row>
     <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="D21" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="15" t="s">
         <v>121</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>122</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="7"/>
@@ -4611,19 +4620,19 @@
     </row>
     <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="C22" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="D22" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="E22" s="15" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="7"/>
@@ -4633,19 +4642,19 @@
     </row>
     <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="D23" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="15" t="s">
         <v>130</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>131</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="9"/>
@@ -4655,19 +4664,19 @@
     </row>
     <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="D24" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="15" t="s">
         <v>135</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>136</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="7"/>
@@ -4677,19 +4686,19 @@
     </row>
     <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D25" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E25" s="15" t="s">
         <v>139</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>140</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="7"/>
@@ -4699,19 +4708,19 @@
     </row>
     <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>458</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="E26" s="15" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4721,19 +4730,19 @@
     </row>
     <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="D27" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="E27" s="15" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4743,19 +4752,19 @@
     </row>
     <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="D28" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>150</v>
-      </c>
       <c r="E28" s="15" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4765,19 +4774,19 @@
     </row>
     <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="D29" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>154</v>
-      </c>
       <c r="E29" s="15" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -4787,19 +4796,19 @@
     </row>
     <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="D30" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="E30" s="15" t="s">
         <v>158</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>159</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="7"/>
@@ -4809,19 +4818,19 @@
     </row>
     <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="D31" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="15" t="s">
         <v>163</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>164</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="7"/>
@@ -4831,19 +4840,19 @@
     </row>
     <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B32" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="C32" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="C32" s="15" t="s">
-        <v>167</v>
-      </c>
       <c r="D32" s="8" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -4853,19 +4862,19 @@
     </row>
     <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="C33" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="C33" s="15" t="s">
-        <v>170</v>
-      </c>
       <c r="D33" s="6" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -4875,13 +4884,13 @@
     </row>
     <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>172</v>
-      </c>
       <c r="C34" s="15" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="16"/>
@@ -4893,13 +4902,13 @@
     </row>
     <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="C35" s="15" t="s">
         <v>174</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>175</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="16"/>
@@ -4911,13 +4920,13 @@
     </row>
     <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="C36" s="15" t="s">
         <v>481</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>482</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -4929,13 +4938,13 @@
     </row>
     <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -4947,13 +4956,13 @@
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -4965,13 +4974,13 @@
     </row>
     <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -4981,12 +4990,16 @@
       <c r="I39" s="3"/>
       <c r="J39" s="4"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="16"/>
+        <v>179</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>523</v>
+      </c>
       <c r="D40" s="6"/>
       <c r="E40" s="16"/>
       <c r="F40" s="6"/>
@@ -4997,7 +5010,7 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="16"/>
@@ -5011,7 +5024,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="16"/>
@@ -5025,7 +5038,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="16"/>
@@ -5039,7 +5052,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="16"/>
@@ -5053,7 +5066,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="16"/>
@@ -5067,7 +5080,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="16"/>
@@ -5081,7 +5094,7 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="16"/>
@@ -5095,7 +5108,7 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="16"/>
@@ -5109,7 +5122,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="16"/>
@@ -5123,7 +5136,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="16"/>
@@ -5137,7 +5150,7 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="16"/>
@@ -5151,7 +5164,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="16"/>
@@ -5165,7 +5178,7 @@
     </row>
     <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="17"/>
@@ -5201,215 +5214,215 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" s="52" t="s">
         <v>194</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="C1" s="53" t="s">
         <v>195</v>
       </c>
-      <c r="C1" s="53" t="s">
+      <c r="D1" s="54" t="s">
         <v>196</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="E1" s="54" t="s">
         <v>197</v>
       </c>
-      <c r="E1" s="54" t="s">
+      <c r="F1" s="54" t="s">
         <v>198</v>
       </c>
-      <c r="F1" s="54" t="s">
+      <c r="G1" s="54" t="s">
+        <v>449</v>
+      </c>
+      <c r="H1" s="54" t="s">
         <v>199</v>
       </c>
-      <c r="G1" s="54" t="s">
-        <v>450</v>
-      </c>
-      <c r="H1" s="54" t="s">
+      <c r="I1" s="55" t="s">
         <v>200</v>
-      </c>
-      <c r="I1" s="55" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="47" t="s">
+        <v>358</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>522</v>
+      </c>
+      <c r="C2" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="B2" s="48" t="s">
-        <v>504</v>
-      </c>
-      <c r="C2" s="49" t="s">
+      <c r="D2" s="50" t="s">
         <v>203</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="E2" s="50" t="s">
         <v>204</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="F2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>206</v>
       </c>
-      <c r="G2" s="50" t="s">
+      <c r="H2" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="H2" s="50" t="s">
+      <c r="I2" s="50" t="s">
         <v>208</v>
-      </c>
-      <c r="I2" s="50" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E3" s="42" t="s">
+        <v>209</v>
+      </c>
+      <c r="F3" s="42" t="s">
         <v>210</v>
       </c>
-      <c r="F3" s="42" t="s">
+      <c r="G3" s="42" t="s">
         <v>211</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="H3" s="42" t="s">
+        <v>324</v>
+      </c>
+      <c r="I3" s="42" t="s">
         <v>212</v>
-      </c>
-      <c r="H3" s="42" t="s">
-        <v>325</v>
-      </c>
-      <c r="I3" s="42" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
+        <v>213</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>214</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="C4" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D4" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D4" s="42" t="s">
+      <c r="E4" s="42" t="s">
         <v>216</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="F4" s="42" t="s">
+        <v>485</v>
+      </c>
+      <c r="G4" s="42" t="s">
         <v>217</v>
       </c>
-      <c r="F4" s="42" t="s">
-        <v>486</v>
-      </c>
-      <c r="G4" s="42" t="s">
+      <c r="H4" s="42" t="s">
         <v>218</v>
-      </c>
-      <c r="H4" s="42" t="s">
-        <v>219</v>
       </c>
       <c r="I4" s="45"/>
     </row>
     <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>330</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D5" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="B5" s="35" t="s">
-        <v>331</v>
-      </c>
-      <c r="C5" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D5" s="42" t="s">
+      <c r="E5" s="42" t="s">
         <v>221</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="F5" s="42" t="s">
         <v>222</v>
       </c>
-      <c r="F5" s="42" t="s">
-        <v>223</v>
-      </c>
       <c r="G5" s="42" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I5" s="45"/>
     </row>
     <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="B6" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="C6" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>225</v>
       </c>
-      <c r="C6" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D6" s="42" t="s">
+      <c r="E6" s="42" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="F6" s="42" t="s">
         <v>227</v>
       </c>
-      <c r="F6" s="42" t="s">
-        <v>228</v>
-      </c>
       <c r="G6" s="42" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H6" s="42" t="s">
-        <v>501</v>
+        <v>525</v>
       </c>
       <c r="I6" s="45"/>
     </row>
     <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
+        <v>228</v>
+      </c>
+      <c r="B7" s="36" t="s">
         <v>229</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="C7" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>491</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>328</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>363</v>
+      </c>
+      <c r="G7" s="42" t="s">
         <v>230</v>
-      </c>
-      <c r="C7" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>492</v>
-      </c>
-      <c r="E7" s="42" t="s">
-        <v>329</v>
-      </c>
-      <c r="F7" s="44" t="s">
-        <v>364</v>
-      </c>
-      <c r="G7" s="42" t="s">
-        <v>231</v>
       </c>
       <c r="H7" s="42"/>
       <c r="I7" s="45"/>
     </row>
     <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
+        <v>231</v>
+      </c>
+      <c r="B8" s="35" t="s">
         <v>232</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="C8" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>233</v>
       </c>
-      <c r="C8" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D8" s="42" t="s">
+      <c r="E8" s="42" t="s">
+        <v>329</v>
+      </c>
+      <c r="F8" s="42" t="s">
         <v>234</v>
-      </c>
-      <c r="E8" s="42" t="s">
-        <v>330</v>
-      </c>
-      <c r="F8" s="42" t="s">
-        <v>235</v>
       </c>
       <c r="G8" s="42"/>
       <c r="H8" s="42"/>
@@ -5417,22 +5430,22 @@
     </row>
     <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
+        <v>235</v>
+      </c>
+      <c r="B9" s="35" t="s">
         <v>236</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="C9" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D9" s="42" t="s">
         <v>237</v>
       </c>
-      <c r="C9" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D9" s="42" t="s">
+      <c r="E9" s="42" t="s">
         <v>238</v>
       </c>
-      <c r="E9" s="42" t="s">
+      <c r="F9" s="42" t="s">
         <v>239</v>
-      </c>
-      <c r="F9" s="42" t="s">
-        <v>240</v>
       </c>
       <c r="G9" s="42"/>
       <c r="H9" s="42"/>
@@ -5440,19 +5453,19 @@
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
+        <v>240</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>500</v>
+      </c>
+      <c r="E10" s="42" t="s">
         <v>242</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>203</v>
-      </c>
-      <c r="D10" s="42" t="s">
-        <v>502</v>
-      </c>
-      <c r="E10" s="42" t="s">
-        <v>243</v>
       </c>
       <c r="F10" s="42"/>
       <c r="G10" s="42"/>
@@ -5461,17 +5474,17 @@
     </row>
     <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D11" s="42"/>
       <c r="E11" s="42" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="F11" s="42"/>
       <c r="G11" s="42"/>
@@ -5480,17 +5493,17 @@
     </row>
     <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>245</v>
       </c>
-      <c r="B12" s="35" t="s">
-        <v>246</v>
-      </c>
       <c r="C12" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D12" s="42"/>
       <c r="E12" s="42" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F12" s="44"/>
       <c r="G12" s="42"/>
@@ -5499,17 +5512,17 @@
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
+        <v>247</v>
+      </c>
+      <c r="B13" s="35" t="s">
         <v>248</v>
       </c>
-      <c r="B13" s="35" t="s">
-        <v>249</v>
-      </c>
       <c r="C13" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D13" s="42"/>
       <c r="E13" s="42" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F13" s="44"/>
       <c r="G13" s="42"/>
@@ -5518,17 +5531,17 @@
     </row>
     <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
+        <v>250</v>
+      </c>
+      <c r="B14" s="35" t="s">
         <v>251</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="C14" s="38" t="s">
         <v>252</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>253</v>
       </c>
       <c r="D14" s="42"/>
       <c r="E14" s="42" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F14" s="44"/>
       <c r="G14" s="42"/>
@@ -5537,13 +5550,13 @@
     </row>
     <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="B15" s="35" t="s">
         <v>255</v>
       </c>
-      <c r="B15" s="35" t="s">
-        <v>256</v>
-      </c>
       <c r="C15" s="38" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="42"/>
@@ -5554,13 +5567,13 @@
     </row>
     <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="B16" s="35" t="s">
         <v>257</v>
       </c>
-      <c r="B16" s="35" t="s">
-        <v>258</v>
-      </c>
       <c r="C16" s="38" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D16" s="42"/>
       <c r="E16" s="42"/>
@@ -5571,13 +5584,13 @@
     </row>
     <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
@@ -5588,13 +5601,13 @@
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="37" t="s">
+        <v>258</v>
+      </c>
+      <c r="B18" s="35" t="s">
         <v>259</v>
       </c>
-      <c r="B18" s="35" t="s">
+      <c r="C18" s="38" t="s">
         <v>260</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>261</v>
       </c>
       <c r="D18" s="42"/>
       <c r="E18" s="42"/>
@@ -5605,13 +5618,13 @@
     </row>
     <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="B19" s="35" t="s">
         <v>262</v>
       </c>
-      <c r="B19" s="35" t="s">
-        <v>263</v>
-      </c>
       <c r="C19" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D19" s="42"/>
       <c r="E19" s="42"/>
@@ -5622,13 +5635,13 @@
     </row>
     <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="B20" s="35" t="s">
         <v>264</v>
       </c>
-      <c r="B20" s="35" t="s">
-        <v>265</v>
-      </c>
       <c r="C20" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D20" s="42"/>
       <c r="E20" s="42"/>
@@ -5639,13 +5652,13 @@
     </row>
     <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
+        <v>477</v>
+      </c>
+      <c r="B21" s="35" t="s">
         <v>478</v>
       </c>
-      <c r="B21" s="35" t="s">
-        <v>479</v>
-      </c>
       <c r="C21" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D21" s="42"/>
       <c r="E21" s="42"/>
@@ -5656,13 +5669,13 @@
     </row>
     <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="37" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D22" s="42"/>
       <c r="E22" s="42"/>
@@ -5673,13 +5686,13 @@
     </row>
     <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="37" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B23" s="35" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C23" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D23" s="42"/>
       <c r="E23" s="42"/>
@@ -5690,13 +5703,13 @@
     </row>
     <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="39" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C24" s="41" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D24" s="42"/>
       <c r="E24" s="42"/>
@@ -5707,13 +5720,13 @@
     </row>
     <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B25" s="40" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="C25" s="41" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D25" s="43"/>
       <c r="E25" s="43"/>
@@ -5739,33 +5752,33 @@
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="72"/>
       <c r="B1" s="65" t="s">
+        <v>269</v>
+      </c>
+      <c r="C1" s="65" t="s">
         <v>270</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="D1" s="64" t="s">
         <v>271</v>
       </c>
-      <c r="D1" s="64" t="s">
+      <c r="E1" s="64" t="s">
         <v>272</v>
       </c>
-      <c r="E1" s="64" t="s">
+      <c r="F1" s="64" t="s">
         <v>273</v>
       </c>
-      <c r="F1" s="64" t="s">
+      <c r="G1" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="G1" s="64" t="s">
-        <v>275</v>
-      </c>
       <c r="I1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="74" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B2" s="75" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C2" s="68" t="s">
         <v>92</v>
@@ -5774,21 +5787,21 @@
         <v>99</v>
       </c>
       <c r="E2" s="69" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F2" s="63" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G2" s="69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="74" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B3" s="76" t="s">
         <v>47</v>
@@ -5800,21 +5813,21 @@
         <v>15</v>
       </c>
       <c r="E3" s="66" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F3" s="63" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G3" s="66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="74" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B4" s="67" t="s">
         <v>85</v>
@@ -5823,27 +5836,27 @@
         <v>57</v>
       </c>
       <c r="D4" s="66" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E4" s="66" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F4" s="66" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G4" s="66" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I4" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B5" s="73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C5" s="73" t="s">
         <v>80</v>
@@ -5855,21 +5868,21 @@
         <v>75</v>
       </c>
       <c r="F5" s="70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G5" s="71" t="s">
         <v>27</v>
       </c>
       <c r="I5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B6" s="98" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C6" s="99" t="s">
         <v>42</v>
@@ -5878,317 +5891,317 @@
         <v>94</v>
       </c>
       <c r="E6" s="101" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F6" s="100" t="s">
         <v>81</v>
       </c>
       <c r="G6" s="102" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="77" t="s">
+        <v>280</v>
+      </c>
+      <c r="B7" s="77" t="s">
         <v>281</v>
       </c>
-      <c r="B7" s="77" t="s">
+      <c r="C7" s="74" t="s">
+        <v>382</v>
+      </c>
+      <c r="D7" t="s">
         <v>282</v>
       </c>
-      <c r="C7" s="74" t="s">
-        <v>383</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="E7" s="74" t="s">
         <v>283</v>
       </c>
-      <c r="E7" s="74" t="s">
+      <c r="F7" t="s">
         <v>284</v>
       </c>
-      <c r="F7" t="s">
-        <v>285</v>
-      </c>
       <c r="G7" s="74" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="95" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B8" s="95" t="s">
+        <v>272</v>
+      </c>
+      <c r="C8" s="91" t="s">
         <v>273</v>
       </c>
-      <c r="C8" s="91" t="s">
+      <c r="D8" s="95" t="s">
         <v>274</v>
       </c>
-      <c r="D8" s="95" t="s">
-        <v>275</v>
-      </c>
       <c r="E8" s="91" t="s">
+        <v>269</v>
+      </c>
+      <c r="F8" s="95" t="s">
         <v>270</v>
       </c>
-      <c r="F8" s="95" t="s">
+      <c r="G8" s="92" t="s">
         <v>271</v>
       </c>
-      <c r="G8" s="92" t="s">
-        <v>272</v>
-      </c>
       <c r="I8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="63" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B9" s="63" t="s">
+        <v>273</v>
+      </c>
+      <c r="C9" t="s">
+        <v>271</v>
+      </c>
+      <c r="D9" s="63" t="s">
+        <v>270</v>
+      </c>
+      <c r="E9" t="s">
         <v>274</v>
       </c>
-      <c r="C9" t="s">
+      <c r="F9" s="63" t="s">
+        <v>269</v>
+      </c>
+      <c r="G9" s="76" t="s">
         <v>272</v>
-      </c>
-      <c r="D9" s="63" t="s">
-        <v>271</v>
-      </c>
-      <c r="E9" t="s">
-        <v>275</v>
-      </c>
-      <c r="F9" s="63" t="s">
-        <v>270</v>
-      </c>
-      <c r="G9" s="76" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="96" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B10" s="96" t="s">
+        <v>271</v>
+      </c>
+      <c r="C10" s="93" t="s">
+        <v>274</v>
+      </c>
+      <c r="D10" s="96" t="s">
+        <v>269</v>
+      </c>
+      <c r="E10" s="93" t="s">
+        <v>273</v>
+      </c>
+      <c r="F10" s="96" t="s">
         <v>272</v>
       </c>
-      <c r="C10" s="93" t="s">
-        <v>275</v>
-      </c>
-      <c r="D10" s="96" t="s">
+      <c r="G10" s="94" t="s">
         <v>270</v>
-      </c>
-      <c r="E10" s="93" t="s">
-        <v>274</v>
-      </c>
-      <c r="F10" s="96" t="s">
-        <v>273</v>
-      </c>
-      <c r="G10" s="94" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>385</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>386</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>388</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>381</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>392</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -6196,111 +6209,111 @@
     </row>
     <row r="23" spans="1:9" ht="225" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>402</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="255" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>410</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="345" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>409</v>
-      </c>
       <c r="D25" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>413</v>
-      </c>
       <c r="F25" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>417</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="255" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>421</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="195" x14ac:dyDescent="0.25">
@@ -6308,133 +6321,133 @@
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>429</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>344</v>
-      </c>
       <c r="G30" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I30" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>340</v>
-      </c>
       <c r="G32" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="2"/>
       <c r="D34" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -6450,16 +6463,16 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
@@ -6467,74 +6480,74 @@
     </row>
     <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E37" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="F37" s="2" t="s">
-        <v>354</v>
-      </c>
       <c r="G37" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I37" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I38" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I39" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -6542,14 +6555,14 @@
       <c r="B40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G40" s="2"/>
       <c r="I40" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -6589,165 +6602,165 @@
     </row>
     <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C47" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>433</v>
-      </c>
       <c r="G47" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="49" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>437</v>
-      </c>
       <c r="F49" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="50" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G50" s="2"/>
     </row>
     <row r="52" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E52" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="F52" s="2" t="s">
-        <v>344</v>
-      </c>
       <c r="G52" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>340</v>
-      </c>
       <c r="G54" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="C55" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E55" s="2" t="s">
+      <c r="G55" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
@@ -6763,80 +6776,80 @@
     </row>
     <row r="58" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E58" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>354</v>
-      </c>
       <c r="G58" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B61" s="3"/>
       <c r="C61" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
@@ -6864,64 +6877,66 @@
   <sheetData>
     <row r="1" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" s="32" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C1" s="33" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D1" s="32" t="s">
+        <v>201</v>
+      </c>
+      <c r="E1" s="110" t="s">
         <v>202</v>
-      </c>
-      <c r="E1" s="109" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="31" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D2" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="E2" s="110"/>
+        <v>228</v>
+      </c>
+      <c r="E2" s="111"/>
     </row>
     <row r="3" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A3" s="30" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>244</v>
-      </c>
-      <c r="E3" s="110"/>
+        <v>243</v>
+      </c>
+      <c r="E3" s="111"/>
     </row>
     <row r="4" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A4" s="34" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>257</v>
-      </c>
-      <c r="D4" s="34"/>
+        <v>256</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>502</v>
+      </c>
       <c r="E4" s="62" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -6948,44 +6963,46 @@
   <sheetData>
     <row r="1" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>264</v>
-      </c>
-      <c r="E1" s="111" t="s">
-        <v>261</v>
+        <v>263</v>
+      </c>
+      <c r="E1" s="112" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="56" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B2" s="32" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C2" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="D2" s="55"/>
-      <c r="E2" s="112"/>
+        <v>256</v>
+      </c>
+      <c r="D2" s="109" t="s">
+        <v>502</v>
+      </c>
+      <c r="E2" s="113"/>
     </row>
     <row r="3" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="57" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3" s="114" t="s">
         <v>286</v>
       </c>
-      <c r="B3" s="113" t="s">
-        <v>287</v>
-      </c>
-      <c r="C3" s="114"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="116"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7055,20 +7072,20 @@
       <c r="A2" s="60">
         <v>39</v>
       </c>
-      <c r="B2" s="118" t="s">
-        <v>288</v>
-      </c>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
-      <c r="I2" s="119"/>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="119"/>
-      <c r="M2" s="119"/>
+      <c r="B2" s="119" t="s">
+        <v>287</v>
+      </c>
+      <c r="C2" s="120"/>
+      <c r="D2" s="120"/>
+      <c r="E2" s="120"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="120"/>
       <c r="N2" s="60">
         <v>14</v>
       </c>
@@ -7077,18 +7094,18 @@
       <c r="A3" s="60">
         <v>38</v>
       </c>
-      <c r="B3" s="120"/>
-      <c r="C3" s="121"/>
-      <c r="D3" s="121"/>
-      <c r="E3" s="121"/>
-      <c r="F3" s="121"/>
-      <c r="G3" s="121"/>
-      <c r="H3" s="121"/>
-      <c r="I3" s="121"/>
-      <c r="J3" s="121"/>
-      <c r="K3" s="121"/>
-      <c r="L3" s="121"/>
-      <c r="M3" s="121"/>
+      <c r="B3" s="121"/>
+      <c r="C3" s="122"/>
+      <c r="D3" s="122"/>
+      <c r="E3" s="122"/>
+      <c r="F3" s="122"/>
+      <c r="G3" s="122"/>
+      <c r="H3" s="122"/>
+      <c r="I3" s="122"/>
+      <c r="J3" s="122"/>
+      <c r="K3" s="122"/>
+      <c r="L3" s="122"/>
+      <c r="M3" s="122"/>
       <c r="N3" s="60">
         <v>15</v>
       </c>
@@ -7097,20 +7114,20 @@
       <c r="A4" s="60">
         <v>37</v>
       </c>
-      <c r="B4" s="116" t="s">
-        <v>289</v>
-      </c>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
-      <c r="L4" s="117"/>
-      <c r="M4" s="117"/>
+      <c r="B4" s="117" t="s">
+        <v>288</v>
+      </c>
+      <c r="C4" s="118"/>
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="118"/>
+      <c r="I4" s="118"/>
+      <c r="J4" s="118"/>
+      <c r="K4" s="118"/>
+      <c r="L4" s="118"/>
+      <c r="M4" s="118"/>
       <c r="N4" s="60">
         <v>16</v>
       </c>
@@ -7119,30 +7136,30 @@
       <c r="A5" s="60">
         <v>36</v>
       </c>
-      <c r="B5" s="122" t="s">
-        <v>290</v>
-      </c>
-      <c r="C5" s="123"/>
-      <c r="D5" s="126" t="s">
-        <v>290</v>
-      </c>
-      <c r="E5" s="127"/>
-      <c r="F5" s="126" t="s">
-        <v>290</v>
-      </c>
-      <c r="G5" s="127"/>
-      <c r="H5" s="126" t="s">
-        <v>290</v>
-      </c>
-      <c r="I5" s="127"/>
-      <c r="J5" s="126" t="s">
-        <v>290</v>
-      </c>
-      <c r="K5" s="127"/>
-      <c r="L5" s="126" t="s">
-        <v>290</v>
-      </c>
-      <c r="M5" s="130"/>
+      <c r="B5" s="123" t="s">
+        <v>289</v>
+      </c>
+      <c r="C5" s="124"/>
+      <c r="D5" s="127" t="s">
+        <v>289</v>
+      </c>
+      <c r="E5" s="128"/>
+      <c r="F5" s="127" t="s">
+        <v>289</v>
+      </c>
+      <c r="G5" s="128"/>
+      <c r="H5" s="127" t="s">
+        <v>289</v>
+      </c>
+      <c r="I5" s="128"/>
+      <c r="J5" s="127" t="s">
+        <v>289</v>
+      </c>
+      <c r="K5" s="128"/>
+      <c r="L5" s="127" t="s">
+        <v>289</v>
+      </c>
+      <c r="M5" s="131"/>
       <c r="N5" s="60">
         <v>17</v>
       </c>
@@ -7151,18 +7168,18 @@
       <c r="A6" s="60">
         <v>35</v>
       </c>
-      <c r="B6" s="122"/>
-      <c r="C6" s="123"/>
-      <c r="D6" s="122"/>
-      <c r="E6" s="128"/>
-      <c r="F6" s="122"/>
-      <c r="G6" s="128"/>
-      <c r="H6" s="122"/>
-      <c r="I6" s="128"/>
-      <c r="J6" s="122"/>
-      <c r="K6" s="128"/>
-      <c r="L6" s="122"/>
-      <c r="M6" s="123"/>
+      <c r="B6" s="123"/>
+      <c r="C6" s="124"/>
+      <c r="D6" s="123"/>
+      <c r="E6" s="129"/>
+      <c r="F6" s="123"/>
+      <c r="G6" s="129"/>
+      <c r="H6" s="123"/>
+      <c r="I6" s="129"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="129"/>
+      <c r="L6" s="123"/>
+      <c r="M6" s="124"/>
       <c r="N6" s="60">
         <v>18</v>
       </c>
@@ -7171,18 +7188,18 @@
       <c r="A7" s="60">
         <v>34</v>
       </c>
-      <c r="B7" s="124"/>
-      <c r="C7" s="125"/>
-      <c r="D7" s="124"/>
-      <c r="E7" s="129"/>
-      <c r="F7" s="124"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="124"/>
-      <c r="I7" s="129"/>
-      <c r="J7" s="124"/>
-      <c r="K7" s="129"/>
-      <c r="L7" s="124"/>
-      <c r="M7" s="125"/>
+      <c r="B7" s="125"/>
+      <c r="C7" s="126"/>
+      <c r="D7" s="125"/>
+      <c r="E7" s="130"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="130"/>
+      <c r="H7" s="125"/>
+      <c r="I7" s="130"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="130"/>
+      <c r="L7" s="125"/>
+      <c r="M7" s="126"/>
       <c r="N7" s="60">
         <v>19</v>
       </c>
@@ -7608,7 +7625,7 @@
       </c>
       <c r="P2" s="104" t="str">
         <f>Cards!C17</f>
-        <v>You may repeat Court Actions with level 7 - $L6 Leaders</v>
+        <v xml:space="preserve">You may repeat Court Actions with level 7 - $L6 (or higher) Leaders </v>
       </c>
       <c r="Q2" s="103" t="str">
         <f>Cards!C18</f>
@@ -7748,7 +7765,7 @@
       </c>
       <c r="AY2" s="104" t="str">
         <f t="shared" si="1"/>
-        <v>You may repeat Court Actions with level 7 - $L6 Leaders</v>
+        <v xml:space="preserve">You may repeat Court Actions with level 7 - $L6 (or higher) Leaders </v>
       </c>
       <c r="AZ2" s="103" t="str">
         <f t="shared" si="1"/>
@@ -8781,31 +8798,31 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C1" t="s">
         <v>310</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>311</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>312</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>313</v>
-      </c>
-      <c r="F1" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B2">
         <f>30*2</f>
         <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D2">
         <v>27.7</v>
@@ -8813,14 +8830,14 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B3">
         <f>34*2</f>
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D3">
         <v>27.7</v>
@@ -8828,14 +8845,14 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B4">
         <f>18*3</f>
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D4">
         <v>30.75</v>
@@ -8843,222 +8860,222 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B5">
         <f>2*6+6*6</f>
         <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B6">
         <f>1*6+10*6</f>
         <v>66</v>
       </c>
       <c r="C6" t="s">
+        <v>315</v>
+      </c>
+      <c r="E6" t="s">
         <v>316</v>
-      </c>
-      <c r="E6" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B7">
         <f>10*6+10</f>
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B8">
         <f>2*8*6</f>
         <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B9">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B10">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C10" t="s">
+        <v>315</v>
+      </c>
+      <c r="E10" t="s">
         <v>316</v>
-      </c>
-      <c r="E10" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B11">
         <f>(30*6-B10)/5</f>
         <v>30</v>
       </c>
       <c r="C11" t="s">
+        <v>315</v>
+      </c>
+      <c r="E11" t="s">
         <v>316</v>
-      </c>
-      <c r="E11" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B12">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B13">
         <f>(15*6-B12)/5</f>
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E13" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B18">
         <f>10*6</f>
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B19">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B20">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -9080,7 +9097,7 @@
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.28515625" style="108" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.42578125" style="108" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" style="108" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.42578125" style="108" bestFit="1" customWidth="1"/>
     <col min="12" max="19" width="11.85546875" style="108" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12.85546875" style="108" bestFit="1" customWidth="1"/>
@@ -9089,67 +9106,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B1" t="s">
         <v>459</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>460</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>461</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>462</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>489</v>
+      </c>
+      <c r="G1" t="s">
+        <v>488</v>
+      </c>
+      <c r="H1" t="s">
         <v>463</v>
       </c>
-      <c r="F1" t="s">
-        <v>490</v>
-      </c>
-      <c r="G1" t="s">
-        <v>489</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>464</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="108" t="s">
+        <v>486</v>
+      </c>
+      <c r="K1" t="s">
         <v>465</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
+        <v>466</v>
+      </c>
+      <c r="M1" t="s">
+        <v>467</v>
+      </c>
+      <c r="N1" t="s">
+        <v>468</v>
+      </c>
+      <c r="O1" t="s">
+        <v>469</v>
+      </c>
+      <c r="P1" t="s">
+        <v>470</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>471</v>
+      </c>
+      <c r="R1" t="s">
+        <v>472</v>
+      </c>
+      <c r="S1" t="s">
+        <v>473</v>
+      </c>
+      <c r="T1" t="s">
+        <v>474</v>
+      </c>
+      <c r="U1" t="s">
         <v>487</v>
-      </c>
-      <c r="K1" t="s">
-        <v>466</v>
-      </c>
-      <c r="L1" t="s">
-        <v>467</v>
-      </c>
-      <c r="M1" t="s">
-        <v>468</v>
-      </c>
-      <c r="N1" t="s">
-        <v>469</v>
-      </c>
-      <c r="O1" t="s">
-        <v>470</v>
-      </c>
-      <c r="P1" t="s">
-        <v>471</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>472</v>
-      </c>
-      <c r="R1" t="s">
-        <v>473</v>
-      </c>
-      <c r="S1" t="s">
-        <v>474</v>
-      </c>
-      <c r="T1" t="s">
-        <v>475</v>
-      </c>
-      <c r="U1" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
@@ -9253,11 +9270,53 @@
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A4" s="106">
+        <v>46105</v>
+      </c>
+      <c r="B4">
+        <v>6</v>
+      </c>
       <c r="C4" s="107" t="b">
         <v>0</v>
       </c>
       <c r="D4" s="107" t="b">
         <v>0</v>
+      </c>
+      <c r="E4">
+        <v>12</v>
+      </c>
+      <c r="F4">
+        <v>17</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+      <c r="H4" s="108">
+        <v>0.77500000000000002</v>
+      </c>
+      <c r="I4" s="108">
+        <v>0.92777777777777781</v>
+      </c>
+      <c r="J4" s="108">
+        <v>0.78472222222222221</v>
+      </c>
+      <c r="K4" s="108">
+        <v>0.79236111111111107</v>
+      </c>
+      <c r="L4" s="108">
+        <v>0.81111111111111112</v>
+      </c>
+      <c r="M4" s="108">
+        <v>0.83194444444444449</v>
+      </c>
+      <c r="N4" s="108">
+        <v>0.85277777777777775</v>
+      </c>
+      <c r="O4" s="108">
+        <v>0.88263888888888886</v>
+      </c>
+      <c r="P4" s="108">
+        <v>0.92083333333333328</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Renamed Player Shield to Player Screen
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3573" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE269E95-B60B-4888-B96D-B58BAF152290}"/>
+  <xr:revisionPtr revIDLastSave="3628" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38D428B6-DD5E-5BAD-A10B-A879336AE14B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2543,7 +2543,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2891,9 +2891,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3735,10 +3732,6 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -7563,7 +7556,7 @@
         <v>Elite Troops</v>
       </c>
       <c r="BH1" s="81" t="str">
-        <f t="shared" ref="BH1:BQ2" si="2">U1</f>
+        <f t="shared" ref="BH1:BP2" si="2">U1</f>
         <v>Bazaar</v>
       </c>
       <c r="BI1" s="78" t="str">
@@ -8416,7 +8409,7 @@
         <f>AF2</f>
         <v>Trade for up to $L3 additional Coins when Selling to the Undermarket</v>
       </c>
-      <c r="BP4" s="132" t="str">
+      <c r="BP4" s="103" t="str">
         <f>AD2</f>
         <v>Spend $L3 fewer Commodities per Coin when Selling to the Court</v>
       </c>

</xml_diff>

<commit_message>
Added last two training manuals
and simplified up the training section of the spreadsheet now that the info
has been offloaded to other documents.
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3984" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA427B99-EB21-4C0E-964D-00F6EEEB84D3}"/>
+  <xr:revisionPtr revIDLastSave="4020" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A4ADEB1-1B0B-4B21-8355-52A9DF4AA46E}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="472">
   <si>
     <t>Standard Card</t>
   </si>
@@ -553,9 +553,6 @@
     <t>Schemes</t>
   </si>
   <si>
-    <t>Deploy Troops</t>
-  </si>
-  <si>
     <t>Provincial</t>
   </si>
   <si>
@@ -742,9 +739,6 @@
     <t>Gain the King's Favor &amp; gain half Leader's Level Coins from the Royal Bank. Players holding the King's Favor may not Flatter</t>
   </si>
   <si>
-    <t>Prepare</t>
-  </si>
-  <si>
     <t>Exchange up to Leader Level Coins for Commodities with the Royal Bank at Market Rate then decrease the Market Rate by 1</t>
   </si>
   <si>
@@ -967,24 +961,9 @@
     <t>Undermarket Buy with 2 Coins</t>
   </si>
   <si>
-    <t>Court Buy</t>
-  </si>
-  <si>
-    <t>Court Buy with 4 Coins</t>
-  </si>
-  <si>
     <t>Upgrade Eager Laborers by 2 Levels</t>
   </si>
   <si>
-    <t>Court Sell for 3 Coins</t>
-  </si>
-  <si>
-    <t>Private Sell for 2 Coins</t>
-  </si>
-  <si>
-    <t>Infiltrate 2 Spies</t>
-  </si>
-  <si>
     <t>Postpone with Level 1 Leader</t>
   </si>
   <si>
@@ -994,18 +973,12 @@
     <t>Petition both Laws</t>
   </si>
   <si>
-    <t>Build Level 2 Investment</t>
-  </si>
-  <si>
     <t>Deploy 2 Troops with 1 extra</t>
   </si>
   <si>
     <t>Private Sell</t>
   </si>
   <si>
-    <t>Court Monetize with Law and Scheme cards for 2 Coins</t>
-  </si>
-  <si>
     <t>Undermarket Sell for 4 Coins</t>
   </si>
   <si>
@@ -1039,84 +1012,9 @@
     <t>Instructions</t>
   </si>
   <si>
-    <t>Setup</t>
-  </si>
-  <si>
-    <t>Find starting Investments and Law</t>
-  </si>
-  <si>
-    <t>Place 4 Greeks per player in the Greek Reserves of the Battlefield</t>
-  </si>
-  <si>
-    <t>Place 3 Coins plus 1 per player in the Royal Bank</t>
-  </si>
-  <si>
-    <t>Place a non-player die in the Market Rate with value 3</t>
-  </si>
-  <si>
-    <t>Place your Investments in front of your shield and place a non-player die on each showing level 2</t>
-  </si>
-  <si>
-    <t>Place four of your player dice in front of your shield showing level 2. These are your Leaders.</t>
-  </si>
-  <si>
-    <t>Mark your Law and place it facedown near the Court</t>
-  </si>
-  <si>
-    <t>Without looking at the player Laws, stack them facedown near the Court in turn order. Each player's mark should be visible in the stack. The Veteran's Law should be on top, and the Crime Lord's should be on the bottom.</t>
-  </si>
-  <si>
-    <t>Take the dice, favors, and card markers of your color</t>
-  </si>
-  <si>
-    <t>Place one of your favors on the scoretrack on the outside of the Battlefield</t>
-  </si>
-  <si>
-    <t>Take the King's Favor and place it in front of your shield</t>
-  </si>
-  <si>
-    <t>Give 4 Troops to each player. Tell them to keep Troops in front of their shield.</t>
-  </si>
-  <si>
-    <t>Give 1 Spy to each player. Tell them to keep Spies behind their shield.</t>
-  </si>
-  <si>
-    <t>Give 3 Coins to each player. Tell them to keep Coins behind their shield.</t>
-  </si>
-  <si>
     <t>Spies, cards</t>
   </si>
   <si>
-    <t>Place 2 markers from each Player in each Scheme envelope. Then, give each player an envelope and tell them to keep it behind their shield.</t>
-  </si>
-  <si>
-    <t>Take the Troops and put them near you in plain sight of all players</t>
-  </si>
-  <si>
-    <t>Take the Spies and put them near you in plain sight of all players</t>
-  </si>
-  <si>
-    <t>Take the Coins and Commodities and put them near you in plain sight of all players</t>
-  </si>
-  <si>
-    <t>Take the Battlefield and non-player dice and put them near you in plain sight of all players</t>
-  </si>
-  <si>
-    <t>Take the Scheme envelopes</t>
-  </si>
-  <si>
-    <t>Once all players have collected their starting cards, shuffle the three decks. Give each player 2 cards from each deck for their hand. Tell each player to keep the cards private.</t>
-  </si>
-  <si>
-    <t>Startup</t>
-  </si>
-  <si>
-    <t>Set your Law to 2 when the Chief Scribe asks you</t>
-  </si>
-  <si>
-    <t>Reveal the top card in the Law queue and have the Veteran set the value. Read the deliberated Law and tell players it is not currently active but will be at the end of the round.</t>
-  </si>
-  <si>
     <t>Round 1</t>
   </si>
   <si>
@@ -1126,132 +1024,18 @@
     <t>Round 3</t>
   </si>
   <si>
-    <t>Night</t>
-  </si>
-  <si>
-    <t>Take one of your unused leaders and place it on the Buy space of the Court. Explain you want some Commodities and will pay the Court 2 Coins in exchange for 3 Commodities per Coin. The number of Commodities is determined by the Market Rate. Place 2 Coins in the Royal Bank and take 6 Commodities. Explain that you will lower the Market Rate by 1 since Commodities are now a little more rare.</t>
-  </si>
-  <si>
-    <t>Take one of your unused leaders and place it on Flatter in the Court. Explain you would like the King's Favor since it is worth 1 Honor at the end of the game and that it breaks any tie during the game. Explain that the king also sends you home with some cash. Take 1 Coin (half your Leader's level) from the Royal Bank.</t>
-  </si>
-  <si>
-    <t>Take one of your unused leaders and place it on the Persian spaces of the Battlefield. Place 2 of your Troops in the same space. Explain you want to deploy 2 Troops to fight the Greeks. Since you are the player with the most Troops deployed, you will be the General at the end of the round and gain 1 Honor (Victory Point). Explain the king pays you for your Troops then take 1 Coin (half Troop count) from the Royal Bank.</t>
-  </si>
-  <si>
-    <t>Take one of your unused leaders and place it in a Persian space of the Battlefield. Explain you also want to deploy 2 Troops, but you have War Machines which allows you to purchase more and deploy them immediately. Pay 1 Coin to gain 1 Troop then deploy 3 Troops. Since you now have the most Troops, you will be the General at the end of the round. The king then pays you half your deployed Troops (rounded up), so take 2 Coins from the Royal Bank.</t>
-  </si>
-  <si>
-    <t>Take one of your unused Leaders and place it on Harvest in the Province. Explain you want to get some Commodities, but the Court Buy space is already taken, nor would it get you any more than Harvest. Explain only one player per round may take Court actions. Instead, you will gain 2 Commodities, one for each of your Leader's level.</t>
-  </si>
-  <si>
-    <t>Deploy an unused leader and 2 Troops into the Battlefield then take 1 Coin from the Royal Bank. Explain you have Elite Troops which gets you more Coins during deployment then take 2 more Coins from the Royal Bank.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Brainstorm in the Province. Explain you want more cards then take a card from each deck for each level of your Leader (2 cards from each deck).</t>
-  </si>
-  <si>
-    <t>Brainstorm and gain 2 cards from each deck. Explain your Genius Commanders also give you two more cards. Take 2 Investments in addition to your other cards.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Promote in the Province and immediately increase its level by 1. Explain you want a more powerful leader and are willing to spend an action to get it.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Monetize in the Court. Explain you want some Coins and don't want your cards. This action allows you to gain Coins in exchange for the opposite of the Market Rate in cards (7 - Market Rate). You also have Market Niche, so discard 3 non-Scheme cards and take 1 Coin from the Royal Bank. Explain you do not change the Market Rate for selling ideas.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Sell in the Province Undermarket. Explain you want Coins in exchange for your Commodities since the Market Rate is so low. Normally, the Undermarket would be worse than the Court, but you have Blood Pact which makes it better for you. Pay 2 Commodities for 2 Coins from outside the Royal Bank. Explain you are dealing with the Undermarket, not the king, so you aren't restricted by the Royal Bank. Increase the Market Rate by 1 since Commodities are now less rare.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Buy in the Province Undermarket. Explain you want Commodities but have to take a worse rate since the Court Buy has already been used. Exchange 2 Coins for 4 Commodities outside the Royal Bank. Decrease the Market Rate by 1.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Negotiate in the Province. Explain you want to form an alliance with the Crime Lord, and he must put one of his unused leaders on the same space. Both players then exchange 2 favors, one for each leader level. Explain favors are worth Honor at the end of the game.</t>
-  </si>
-  <si>
-    <t>You have a card that allows you to Monetize at a better rate, so place an unused leader on that card. Then, discard 3 Schemes and 3 Laws to gain 2 Coins outside the Royal Bank.</t>
-  </si>
-  <si>
-    <t>You have no more leaders left, so you must pass for the rest of the round.</t>
-  </si>
-  <si>
-    <t>Place an unused leader on Commission in the Province. Explain you want another leader, so take a leader from behind your shield and place it on the same space with half the level of the first leader.</t>
-  </si>
-  <si>
-    <t>Harvest 1 Commodity for each of your leader's levels.</t>
-  </si>
-  <si>
-    <t>All players are out of leaders, so the round ends and moves to the event phase.</t>
-  </si>
-  <si>
-    <t>1. Explain there are no active Laws, so no one has to pay Taxes. Since no one broke any Laws, the King's Favor stays where it is.</t>
-  </si>
-  <si>
-    <t>2. Now, we fight the Greeks. I deployed the most Troops, so I am the General and will gain 1 Honor now. I will roll 1 die for each player, cut each die value in half (rounded up) then total the result. This is how many Greeks we have to fight. Each Greek and Persian Troop in the battle will kill each other, and whichever side has remaining troops wins (we win ties). If we win, each player who deployed Troops will gain 1 Honor. If we lose, the remaining Greeks will attack our Provinces. See rulebook for Battle details.</t>
-  </si>
-  <si>
-    <t>3. After the battle, everyone collects their leaders from the board.</t>
-  </si>
-  <si>
-    <t>4. I will take everyone's Sheme envelopes, mix them up, then open them one by one. If there are any Schemes, we will resolve them. Then, I will return the reset envelopes to players.</t>
-  </si>
-  <si>
-    <t>5. Since no one postponed this deliberated Law, it becomes active. From now on, all players must obey it or their leaders will have one less level when taking the sanctioned action and pay a tax at the end of the round. I will also reveal the next Law for deliberation. It was sponsored by the Master of Lies, so they will choose its value. This Law is not active until the end of the next round.</t>
-  </si>
-  <si>
-    <t>5. Set your Law to 2 when the Chief Scribe asks you</t>
-  </si>
-  <si>
-    <t>6. There are still Greeks left, so we will play another round.</t>
-  </si>
-  <si>
-    <t>8. I have the King's Favor, so I will start the next round.</t>
-  </si>
-  <si>
-    <t>Scheme Instructions</t>
-  </si>
-  <si>
-    <t>You are doing great! Keep up the good work.</t>
-  </si>
-  <si>
     <t>Court Buy with 2 Coins</t>
   </si>
   <si>
-    <t>Deploy 2 Troops with 1 War Machine</t>
-  </si>
-  <si>
-    <t>Court Monetize with 3 non-scheme cards</t>
-  </si>
-  <si>
-    <t>Undermarket Sell for 2 Coins</t>
-  </si>
-  <si>
-    <t>Brainstorm with 2 extra Investments</t>
-  </si>
-  <si>
-    <t>Negotiate with Crime Lord</t>
-  </si>
-  <si>
-    <t>Monetize with 3 Schemes and 3 Laws</t>
-  </si>
-  <si>
     <t>Change the boundary of an active Law to $L6</t>
   </si>
   <si>
     <t>Irregular Partiality</t>
   </si>
   <si>
-    <t>Place an unused leader on Accuse in the Province. Explain you want to fight the Master of Lies, and they must place one of their unused leaders on the same space. Both players then put 1 Coin into the Royal Bank and roll dice to resolve the Accuse. Each Accuse has three rounds. The player who rolls more hits wins a round. The player who wins the best two out of three rounds wins the Accuse. Each die rolled higher than 3 counts as a hit. Tied rounds are repeated unless a player has the King's Favor to break the tie. You have Training Grounds which give you an automatic two hits each Roll. Perform the Accuse. Whoever wins takes two Coins from the Royal Bank and gains 1 Honor.</t>
-  </si>
-  <si>
-    <t>Accuse Crime Lord</t>
-  </si>
-  <si>
     <t>Accuse Veteran</t>
   </si>
   <si>
-    <t>Accuse Master of Lies</t>
-  </si>
-  <si>
     <t>Desperate Attorneys</t>
   </si>
   <si>
@@ -1519,15 +1303,6 @@
     <t>Court Sell for 2 Coins</t>
   </si>
   <si>
-    <t>7. The king has many other financial interests and has made some money. I will add 3 Coins to the Royal Bank and adjust the Market Rate by 1 in a random direction. See rulebook for Market Rate adjustment details. Roll until Market Rate increases to 3.</t>
-  </si>
-  <si>
-    <t>At some point during the next round, place a Spy into the Scheme envelope with Corporate Takeover. Place a marker for the Warmongerer in the top left corner of the card and a marker for one of your Allies in the bottom right corner.</t>
-  </si>
-  <si>
-    <t>At some point during the next round, place a Spy into the Scheme envelope with Intimidation. Place a marker for the Chief Scribe in the top left corner of the card.</t>
-  </si>
-  <si>
     <t>Private Sell for 3 Coins</t>
   </si>
   <si>
@@ -1537,9 +1312,6 @@
     <t>Infiltrate 3 Spies</t>
   </si>
   <si>
-    <t>Take one of your unused leaders and place it on the Recruit space of the Province. Explain you want to get some Troops, so you will pay  2 Coins to the people of your Province. Put 2 Coins in the pile, not the Royal Bank, and take 2 Troops + 1. Explain that the Coins do not go to the Royal Bank during Recruit.</t>
-  </si>
-  <si>
     <t>Deploy $L3 additional Troops during Deploy</t>
   </si>
   <si>
@@ -1655,6 +1427,39 @@
   </si>
   <si>
     <t>Build Level 2 Investment (Boasting Propaganda)</t>
+  </si>
+  <si>
+    <t>Recruit 3 Troops</t>
+  </si>
+  <si>
+    <t>Buy with 2 Coins</t>
+  </si>
+  <si>
+    <t>Harvest 4 Commodities</t>
+  </si>
+  <si>
+    <t>Monetize for 1 Coin</t>
+  </si>
+  <si>
+    <t>Brainstorm for 6 cards</t>
+  </si>
+  <si>
+    <t>Brainstorm for 8 cards</t>
+  </si>
+  <si>
+    <t>Negotiate with the Crime Lord</t>
+  </si>
+  <si>
+    <t>Sue the Master of Lies</t>
+  </si>
+  <si>
+    <t>Monetize Schemes and Laws for 2 Coins</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Sue Crime Lord</t>
   </si>
 </sst>
 </file>
@@ -2976,6 +2781,60 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2986,60 +2845,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4272,7 +4077,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>474</v>
+        <v>402</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="2"/>
@@ -4283,10 +4088,10 @@
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>435</v>
+        <v>363</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>436</v>
+        <v>364</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>14</v>
@@ -4295,10 +4100,10 @@
         <v>15</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>522</v>
+        <v>446</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>484</v>
+        <v>412</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="2"/>
@@ -4312,19 +4117,19 @@
         <v>17</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>502</v>
+        <v>426</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>473</v>
+        <v>401</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="3"/>
@@ -4344,13 +4149,13 @@
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>523</v>
+        <v>447</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="2"/>
@@ -4373,10 +4178,10 @@
         <v>29</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>519</v>
+        <v>443</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>476</v>
+        <v>404</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="3"/>
@@ -4399,10 +4204,10 @@
         <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>511</v>
+        <v>435</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>512</v>
+        <v>436</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="3"/>
@@ -4416,19 +4221,19 @@
         <v>41</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>510</v>
+        <v>434</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>397</v>
+        <v>328</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>513</v>
+        <v>437</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>514</v>
+        <v>438</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="2"/>
@@ -4439,7 +4244,7 @@
         <v>38</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>532</v>
+        <v>456</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>44</v>
@@ -4448,13 +4253,13 @@
         <v>39</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>396</v>
+        <v>327</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>515</v>
+        <v>439</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>516</v>
+        <v>440</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
@@ -4471,16 +4276,16 @@
         <v>49</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>526</v>
+        <v>450</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>530</v>
+        <v>454</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>517</v>
+        <v>441</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>518</v>
+        <v>442</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="2"/>
@@ -4491,22 +4296,22 @@
         <v>43</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>446</v>
+        <v>374</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>529</v>
+        <v>453</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>531</v>
+        <v>455</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>521</v>
+        <v>445</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>520</v>
+        <v>444</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="2"/>
@@ -4520,7 +4325,7 @@
         <v>57</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>432</v>
+        <v>360</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>50</v>
@@ -4532,7 +4337,7 @@
         <v>46</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>478</v>
+        <v>406</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="2"/>
@@ -4558,7 +4363,7 @@
         <v>52</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>477</v>
+        <v>405</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
@@ -4584,7 +4389,7 @@
         <v>42</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>477</v>
+        <v>405</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
@@ -4598,7 +4403,7 @@
         <v>71</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>468</v>
+        <v>396</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>63</v>
@@ -4610,7 +4415,7 @@
         <v>65</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>480</v>
+        <v>408</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="3"/>
@@ -4621,7 +4426,7 @@
         <v>66</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>445</v>
+        <v>373</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>76</v>
@@ -4630,13 +4435,13 @@
         <v>69</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>533</v>
+        <v>457</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>509</v>
+        <v>433</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>479</v>
+        <v>407</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="2"/>
@@ -4659,10 +4464,10 @@
         <v>73</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>483</v>
+        <v>411</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>479</v>
+        <v>407</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="2"/>
@@ -4682,13 +4487,13 @@
         <v>77</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>409</v>
+        <v>337</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>36</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>475</v>
+        <v>403</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
@@ -4708,13 +4513,13 @@
         <v>81</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>410</v>
+        <v>338</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>462</v>
+        <v>390</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>481</v>
+        <v>409</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
@@ -4737,10 +4542,10 @@
         <v>86</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>463</v>
+        <v>391</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>482</v>
+        <v>410</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
@@ -4763,10 +4568,10 @@
         <v>91</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>486</v>
+        <v>414</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>481</v>
+        <v>409</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="3"/>
@@ -4786,13 +4591,13 @@
         <v>95</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>429</v>
+        <v>357</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>485</v>
+        <v>413</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="3"/>
@@ -4803,10 +4608,10 @@
         <v>96</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>403</v>
+        <v>331</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>527</v>
+        <v>451</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>99</v>
@@ -4825,10 +4630,10 @@
         <v>101</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>402</v>
+        <v>330</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>528</v>
+        <v>452</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>104</v>
@@ -4872,13 +4677,13 @@
         <v>116</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>110</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>466</v>
+        <v>394</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4900,7 +4705,7 @@
         <v>114</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>467</v>
+        <v>395</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4922,7 +4727,7 @@
         <v>117</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>464</v>
+        <v>392</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4944,7 +4749,7 @@
         <v>121</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>465</v>
+        <v>393</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -5004,13 +4809,13 @@
         <v>139</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>443</v>
+        <v>371</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>460</v>
+        <v>388</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>458</v>
+        <v>386</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -5029,10 +4834,10 @@
         <v>142</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>461</v>
+        <v>389</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>459</v>
+        <v>387</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -5045,10 +4850,10 @@
         <v>138</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>433</v>
+        <v>361</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>434</v>
+        <v>362</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="16"/>
@@ -5063,10 +4868,10 @@
         <v>140</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>447</v>
+        <v>375</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>444</v>
+        <v>372</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="16"/>
@@ -5081,10 +4886,10 @@
         <v>143</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>457</v>
+        <v>385</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>534</v>
+        <v>458</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -5099,10 +4904,10 @@
         <v>144</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>456</v>
+        <v>384</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>455</v>
+        <v>383</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -5117,10 +4922,10 @@
         <v>145</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>471</v>
+        <v>399</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>470</v>
+        <v>398</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -5135,10 +4940,10 @@
         <v>146</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>499</v>
+        <v>423</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>498</v>
+        <v>422</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -5153,10 +4958,10 @@
         <v>147</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>524</v>
+        <v>448</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>525</v>
+        <v>449</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="16"/>
@@ -5171,10 +4976,10 @@
         <v>148</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>535</v>
+        <v>459</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>454</v>
+        <v>382</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="16"/>
@@ -5394,7 +5199,7 @@
         <v>166</v>
       </c>
       <c r="G1" s="54" t="s">
-        <v>406</v>
+        <v>334</v>
       </c>
       <c r="H1" s="54" t="s">
         <v>167</v>
@@ -5405,186 +5210,186 @@
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="47" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="B2" s="48" t="s">
-        <v>469</v>
+        <v>397</v>
       </c>
       <c r="C2" s="49" t="s">
+        <v>169</v>
+      </c>
+      <c r="D2" s="50" t="s">
         <v>170</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="E2" s="50" t="s">
         <v>171</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>172</v>
       </c>
-      <c r="F2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>173</v>
       </c>
-      <c r="G2" s="50" t="s">
+      <c r="H2" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="H2" s="50" t="s">
-        <v>175</v>
-      </c>
       <c r="I2" s="50" t="s">
-        <v>487</v>
+        <v>415</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
-        <v>408</v>
+        <v>336</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>407</v>
+        <v>335</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="E3" s="42" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3" s="42" t="s">
         <v>176</v>
       </c>
-      <c r="F3" s="42" t="s">
+      <c r="G3" s="42" t="s">
         <v>177</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="H3" s="42" t="s">
+        <v>288</v>
+      </c>
+      <c r="I3" s="42" t="s">
         <v>178</v>
-      </c>
-      <c r="H3" s="42" t="s">
-        <v>290</v>
-      </c>
-      <c r="I3" s="42" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>180</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="C4" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D4" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D4" s="42" t="s">
+      <c r="E4" s="42" t="s">
         <v>182</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="F4" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="G4" s="42" t="s">
         <v>183</v>
       </c>
-      <c r="F4" s="42" t="s">
-        <v>437</v>
-      </c>
-      <c r="G4" s="42" t="s">
+      <c r="H4" s="42" t="s">
         <v>184</v>
-      </c>
-      <c r="H4" s="42" t="s">
-        <v>185</v>
       </c>
       <c r="I4" s="45"/>
     </row>
     <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>294</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" s="42" t="s">
         <v>186</v>
       </c>
-      <c r="B5" s="35" t="s">
-        <v>296</v>
-      </c>
-      <c r="C5" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D5" s="42" t="s">
+      <c r="E5" s="42" t="s">
         <v>187</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="F5" s="42" t="s">
         <v>188</v>
       </c>
-      <c r="F5" s="42" t="s">
-        <v>189</v>
-      </c>
       <c r="G5" s="42" t="s">
-        <v>404</v>
+        <v>332</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I5" s="45"/>
     </row>
     <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" s="36" t="s">
         <v>190</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="C6" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D6" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="C6" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" s="42" t="s">
+      <c r="E6" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="F6" s="42" t="s">
         <v>193</v>
       </c>
-      <c r="F6" s="42" t="s">
-        <v>194</v>
-      </c>
       <c r="G6" s="42" t="s">
-        <v>405</v>
+        <v>333</v>
       </c>
       <c r="H6" s="42" t="s">
-        <v>472</v>
+        <v>400</v>
       </c>
       <c r="I6" s="45"/>
     </row>
     <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
+        <v>194</v>
+      </c>
+      <c r="B7" s="36" t="s">
         <v>195</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="C7" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>370</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>292</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>319</v>
+      </c>
+      <c r="G7" s="42" t="s">
         <v>196</v>
-      </c>
-      <c r="C7" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>442</v>
-      </c>
-      <c r="E7" s="42" t="s">
-        <v>294</v>
-      </c>
-      <c r="F7" s="44" t="s">
-        <v>328</v>
-      </c>
-      <c r="G7" s="42" t="s">
-        <v>197</v>
       </c>
       <c r="H7" s="42"/>
       <c r="I7" s="45"/>
     </row>
     <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" s="35" t="s">
         <v>198</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="C8" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D8" s="42" t="s">
+      <c r="E8" s="42" t="s">
+        <v>293</v>
+      </c>
+      <c r="F8" s="42" t="s">
         <v>200</v>
-      </c>
-      <c r="E8" s="42" t="s">
-        <v>295</v>
-      </c>
-      <c r="F8" s="42" t="s">
-        <v>201</v>
       </c>
       <c r="G8" s="42"/>
       <c r="H8" s="42"/>
@@ -5592,22 +5397,22 @@
     </row>
     <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="C9" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9" s="42" t="s">
         <v>203</v>
       </c>
-      <c r="C9" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D9" s="42" t="s">
+      <c r="E9" s="42" t="s">
         <v>204</v>
       </c>
-      <c r="E9" s="42" t="s">
+      <c r="F9" s="42" t="s">
         <v>205</v>
-      </c>
-      <c r="F9" s="42" t="s">
-        <v>206</v>
       </c>
       <c r="G9" s="42"/>
       <c r="H9" s="42"/>
@@ -5615,19 +5420,19 @@
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>377</v>
+      </c>
+      <c r="E10" s="42" t="s">
         <v>208</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D10" s="42" t="s">
-        <v>449</v>
-      </c>
-      <c r="E10" s="42" t="s">
-        <v>209</v>
       </c>
       <c r="F10" s="42"/>
       <c r="G10" s="42"/>
@@ -5636,17 +5441,17 @@
     </row>
     <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B11" s="35" t="s">
-        <v>448</v>
+        <v>376</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D11" s="42"/>
       <c r="E11" s="42" t="s">
-        <v>450</v>
+        <v>378</v>
       </c>
       <c r="F11" s="42"/>
       <c r="G11" s="42"/>
@@ -5655,17 +5460,17 @@
     </row>
     <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="B12" s="35" t="s">
-        <v>212</v>
-      </c>
       <c r="C12" s="38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D12" s="42"/>
       <c r="E12" s="42" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F12" s="44"/>
       <c r="G12" s="42"/>
@@ -5674,17 +5479,17 @@
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
+        <v>213</v>
+      </c>
+      <c r="B13" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="B13" s="35" t="s">
-        <v>215</v>
-      </c>
       <c r="C13" s="38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D13" s="42"/>
       <c r="E13" s="42" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F13" s="44"/>
       <c r="G13" s="42"/>
@@ -5693,17 +5498,17 @@
     </row>
     <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
+        <v>216</v>
+      </c>
+      <c r="B14" s="35" t="s">
         <v>217</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="C14" s="38" t="s">
         <v>218</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>219</v>
       </c>
       <c r="D14" s="42"/>
       <c r="E14" s="42" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F14" s="44"/>
       <c r="G14" s="42"/>
@@ -5712,13 +5517,13 @@
     </row>
     <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="B15" s="35" t="s">
         <v>221</v>
       </c>
-      <c r="B15" s="35" t="s">
-        <v>222</v>
-      </c>
       <c r="C15" s="38" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="42"/>
@@ -5729,13 +5534,13 @@
     </row>
     <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
+        <v>222</v>
+      </c>
+      <c r="B16" s="35" t="s">
         <v>223</v>
       </c>
-      <c r="B16" s="35" t="s">
-        <v>224</v>
-      </c>
       <c r="C16" s="38" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D16" s="42"/>
       <c r="E16" s="42"/>
@@ -5746,13 +5551,13 @@
     </row>
     <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>451</v>
+        <v>379</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>453</v>
+        <v>381</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
@@ -5763,13 +5568,13 @@
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="37" t="s">
+        <v>224</v>
+      </c>
+      <c r="B18" s="35" t="s">
         <v>225</v>
       </c>
-      <c r="B18" s="35" t="s">
+      <c r="C18" s="38" t="s">
         <v>226</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>227</v>
       </c>
       <c r="D18" s="42"/>
       <c r="E18" s="42"/>
@@ -5780,13 +5585,13 @@
     </row>
     <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="B19" s="35" t="s">
         <v>228</v>
       </c>
-      <c r="B19" s="35" t="s">
-        <v>229</v>
-      </c>
       <c r="C19" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D19" s="42"/>
       <c r="E19" s="42"/>
@@ -5797,13 +5602,13 @@
     </row>
     <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
+        <v>229</v>
+      </c>
+      <c r="B20" s="35" t="s">
         <v>230</v>
       </c>
-      <c r="B20" s="35" t="s">
-        <v>231</v>
-      </c>
       <c r="C20" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D20" s="42"/>
       <c r="E20" s="42"/>
@@ -5814,13 +5619,13 @@
     </row>
     <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
-        <v>430</v>
+        <v>358</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>431</v>
+        <v>359</v>
       </c>
       <c r="C21" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D21" s="42"/>
       <c r="E21" s="42"/>
@@ -5831,13 +5636,13 @@
     </row>
     <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="37" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D22" s="42"/>
       <c r="E22" s="42"/>
@@ -5848,13 +5653,13 @@
     </row>
     <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="37" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B23" s="35" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C23" s="38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D23" s="42"/>
       <c r="E23" s="42"/>
@@ -5865,13 +5670,13 @@
     </row>
     <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="39" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C24" s="41" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D24" s="42"/>
       <c r="E24" s="42"/>
@@ -5882,13 +5687,13 @@
     </row>
     <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39" t="s">
-        <v>451</v>
+        <v>379</v>
       </c>
       <c r="B25" s="40" t="s">
-        <v>452</v>
+        <v>380</v>
       </c>
       <c r="C25" s="41" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D25" s="43"/>
       <c r="E25" s="43"/>
@@ -5905,7 +5710,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920DF489-FE6D-4819-BD1A-323DFAE597A3}">
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
@@ -5915,30 +5720,30 @@
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="67"/>
       <c r="B1" s="61" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1" s="61" t="s">
+        <v>235</v>
+      </c>
+      <c r="D1" s="60" t="s">
         <v>236</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="E1" s="60" t="s">
         <v>237</v>
       </c>
-      <c r="D1" s="60" t="s">
+      <c r="F1" s="60" t="s">
         <v>238</v>
       </c>
-      <c r="E1" s="60" t="s">
+      <c r="G1" s="60" t="s">
         <v>239</v>
       </c>
-      <c r="F1" s="60" t="s">
-        <v>240</v>
-      </c>
-      <c r="G1" s="60" t="s">
-        <v>241</v>
-      </c>
       <c r="I1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="69" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B2" s="70" t="s">
         <v>88</v>
@@ -5959,38 +5764,38 @@
         <v>123</v>
       </c>
       <c r="I2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="69" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B3" s="71" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="63" t="s">
-        <v>532</v>
+        <v>456</v>
       </c>
       <c r="D3" s="62" t="s">
-        <v>435</v>
+        <v>363</v>
       </c>
       <c r="E3" s="109" t="s">
         <v>97</v>
       </c>
       <c r="F3" s="59" t="s">
-        <v>402</v>
+        <v>330</v>
       </c>
       <c r="G3" s="63" t="s">
         <v>136</v>
       </c>
       <c r="I3" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="69" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B4" s="63" t="s">
         <v>61</v>
@@ -6011,12 +5816,12 @@
         <v>116</v>
       </c>
       <c r="I4" t="s">
-        <v>428</v>
+        <v>356</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="69" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B5" s="68" t="s">
         <v>141</v>
@@ -6028,21 +5833,21 @@
         <v>17</v>
       </c>
       <c r="E5" s="110" t="s">
-        <v>446</v>
+        <v>374</v>
       </c>
       <c r="F5" s="113" t="s">
         <v>83</v>
       </c>
       <c r="G5" s="111" t="s">
-        <v>456</v>
+        <v>384</v>
       </c>
       <c r="I5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="92" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B6" s="93" t="s">
         <v>104</v>
@@ -6063,951 +5868,561 @@
         <v>121</v>
       </c>
       <c r="I6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="72" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="72" t="s">
+        <v>246</v>
+      </c>
+      <c r="C7" s="69" t="s">
+        <v>322</v>
+      </c>
+      <c r="D7" t="s">
         <v>247</v>
       </c>
-      <c r="B7" s="72" t="s">
+      <c r="E7" s="69" t="s">
         <v>248</v>
       </c>
-      <c r="C7" s="69" t="s">
-        <v>346</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>249</v>
-      </c>
-      <c r="E7" s="69" t="s">
-        <v>250</v>
-      </c>
-      <c r="F7" t="s">
-        <v>251</v>
       </c>
       <c r="G7" s="69" t="s">
         <v>168</v>
       </c>
       <c r="I7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="90" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B8" s="90" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" s="86" t="s">
+        <v>238</v>
+      </c>
+      <c r="D8" s="90" t="s">
         <v>239</v>
       </c>
-      <c r="C8" s="86" t="s">
-        <v>240</v>
-      </c>
-      <c r="D8" s="90" t="s">
-        <v>241</v>
-      </c>
       <c r="E8" s="86" t="s">
+        <v>234</v>
+      </c>
+      <c r="F8" s="90" t="s">
+        <v>235</v>
+      </c>
+      <c r="G8" s="87" t="s">
         <v>236</v>
       </c>
-      <c r="F8" s="90" t="s">
-        <v>237</v>
-      </c>
-      <c r="G8" s="87" t="s">
-        <v>238</v>
-      </c>
       <c r="I8" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="59" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B9" s="59" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C9" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D9" s="59" t="s">
+        <v>235</v>
+      </c>
+      <c r="E9" t="s">
+        <v>239</v>
+      </c>
+      <c r="F9" s="59" t="s">
+        <v>234</v>
+      </c>
+      <c r="G9" s="71" t="s">
         <v>237</v>
-      </c>
-      <c r="E9" t="s">
-        <v>241</v>
-      </c>
-      <c r="F9" s="59" t="s">
-        <v>236</v>
-      </c>
-      <c r="G9" s="71" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="91" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B10" s="91" t="s">
+        <v>236</v>
+      </c>
+      <c r="C10" s="88" t="s">
+        <v>239</v>
+      </c>
+      <c r="D10" s="91" t="s">
+        <v>234</v>
+      </c>
+      <c r="E10" s="88" t="s">
         <v>238</v>
       </c>
-      <c r="C10" s="88" t="s">
-        <v>241</v>
-      </c>
-      <c r="D10" s="91" t="s">
-        <v>236</v>
-      </c>
-      <c r="E10" s="88" t="s">
-        <v>240</v>
-      </c>
       <c r="F10" s="91" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G10" s="89" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>348</v>
+        <v>461</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="D13" s="2"/>
+        <v>420</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>302</v>
+      </c>
       <c r="E13" s="2" t="s">
-        <v>350</v>
+        <v>462</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>351</v>
+        <v>309</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>340</v>
+        <v>302</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>340</v>
+        <v>464</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>340</v>
+        <v>308</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>340</v>
+        <v>417</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>340</v>
+        <v>465</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>341</v>
+        <v>466</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>341</v>
+        <v>194</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>341</v>
+        <v>304</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>341</v>
+        <v>467</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>341</v>
+        <v>468</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>341</v>
+        <v>303</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>332</v>
+        <v>469</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>332</v>
+        <v>470</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>332</v>
+        <v>189</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>332</v>
+        <v>194</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>332</v>
+        <v>463</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
-      <c r="B17" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>324</v>
+      </c>
       <c r="B18" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>336</v>
+        <v>194</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>326</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>336</v>
+        <v>306</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>336</v>
+        <v>419</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>336</v>
+        <v>305</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+      <c r="I18" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>337</v>
+        <v>206</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>337</v>
+        <v>418</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>337</v>
+        <v>302</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>337</v>
+        <v>302</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>337</v>
+        <v>309</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>304</v>
+      </c>
+      <c r="I19" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>344</v>
+        <v>421</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>334</v>
+        <v>303</v>
+      </c>
+      <c r="E20" t="s">
+        <v>206</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>333</v>
+        <v>358</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
-      <c r="B21" s="2" t="s">
-        <v>342</v>
-      </c>
+      <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>356</v>
+        <v>302</v>
+      </c>
+      <c r="D21" t="s">
+        <v>424</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>345</v>
+        <v>460</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="F22" s="2"/>
+        <v>303</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="2"/>
+      <c r="D22" s="2" t="s">
+        <v>320</v>
+      </c>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:9" ht="225" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="255" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>325</v>
+      </c>
       <c r="B24" s="2" t="s">
-        <v>366</v>
+        <v>314</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>370</v>
+        <v>229</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>315</v>
+        <v>201</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>489</v>
+        <v>310</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>367</v>
+        <v>427</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="345" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+      <c r="I24" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
-        <v>368</v>
+        <v>210</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>369</v>
+        <v>213</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>372</v>
+        <v>314</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>373</v>
+        <v>329</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>398</v>
+        <v>471</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="I25" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
-        <v>374</v>
+        <v>430</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>375</v>
+        <v>227</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>195</v>
+        <v>210</v>
+      </c>
+      <c r="E26" t="s">
+        <v>429</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>377</v>
+        <v>210</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="255" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>381</v>
-      </c>
+        <v>312</v>
+      </c>
+      <c r="I26" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>384</v>
+        <v>313</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>491</v>
+        <v>431</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="I27" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C30" t="s">
-        <v>389</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="I30" t="s">
-        <v>314</v>
-      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="I28" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="3"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="I29" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="E32" t="s">
-        <v>207</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D33" t="s">
-        <v>500</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="2"/>
-      <c r="D34" s="2" t="s">
-        <v>329</v>
-      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="3"/>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>359</v>
-      </c>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
-      <c r="I36" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B37" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="I37" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="3"/>
-      <c r="B38" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="I38" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="3"/>
-      <c r="B39" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="E39" t="s">
-        <v>505</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="I39" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="3"/>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="2"/>
-      <c r="C40" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>323</v>
-      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
       <c r="G40" s="2"/>
-      <c r="I40" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
       <c r="E41" s="2"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
-      <c r="I41" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
-    </row>
-    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B47" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B48" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="49" spans="2:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B49" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="50" spans="2:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B50" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="G50" s="2"/>
-    </row>
-    <row r="52" spans="2:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B52" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B53" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B54" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B55" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-    </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-    </row>
-    <row r="58" spans="2:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B58" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B59" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B60" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B61" s="3"/>
-      <c r="C61" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B48" s="3"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7030,66 +6445,66 @@
   <sheetData>
     <row r="1" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" s="32" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C1" s="33" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D1" s="32" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E1" s="114" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="31" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D2" s="31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E2" s="115"/>
     </row>
     <row r="3" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A3" s="30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>408</v>
+        <v>336</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E3" s="115"/>
     </row>
     <row r="4" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A4" s="34" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C4" s="57" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>451</v>
+        <v>379</v>
       </c>
       <c r="E4" s="58" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -7116,42 +6531,42 @@
   <sheetData>
     <row r="1" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>430</v>
+        <v>358</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E1" s="116" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="56" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B2" s="32" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C2" s="33" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D2" s="104" t="s">
-        <v>451</v>
+        <v>379</v>
       </c>
       <c r="E2" s="117"/>
     </row>
     <row r="3" spans="1:5" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="105" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B3" s="118" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C3" s="119"/>
       <c r="D3" s="119"/>
@@ -7178,209 +6593,189 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="121">
-        <v>0</v>
-      </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="121">
+      <c r="A1" s="139">
+        <v>0</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="139">
         <v>1</v>
       </c>
-      <c r="D1" s="122"/>
-      <c r="E1" s="121">
+      <c r="D1" s="140"/>
+      <c r="E1" s="139">
         <v>2</v>
       </c>
-      <c r="F1" s="122"/>
-      <c r="G1" s="121">
+      <c r="F1" s="140"/>
+      <c r="G1" s="139">
         <v>3</v>
       </c>
-      <c r="H1" s="122"/>
-      <c r="I1" s="121">
+      <c r="H1" s="140"/>
+      <c r="I1" s="139">
         <v>4</v>
       </c>
-      <c r="J1" s="122"/>
-      <c r="K1" s="121">
+      <c r="J1" s="140"/>
+      <c r="K1" s="139">
         <v>5</v>
       </c>
-      <c r="L1" s="122"/>
-      <c r="M1" s="121">
+      <c r="L1" s="140"/>
+      <c r="M1" s="139">
         <v>6</v>
       </c>
-      <c r="N1" s="122"/>
+      <c r="N1" s="140"/>
     </row>
     <row r="2" spans="1:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="123">
+      <c r="A2" s="141">
         <v>19</v>
       </c>
-      <c r="B2" s="134" t="s">
-        <v>254</v>
-      </c>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="135"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="123">
+      <c r="B2" s="130" t="s">
+        <v>252</v>
+      </c>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="131"/>
+      <c r="F2" s="131"/>
+      <c r="G2" s="131"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="131"/>
+      <c r="J2" s="131"/>
+      <c r="K2" s="131"/>
+      <c r="L2" s="131"/>
+      <c r="M2" s="132"/>
+      <c r="N2" s="141">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="124"/>
-      <c r="B3" s="137"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
-      <c r="F3" s="138"/>
-      <c r="G3" s="138"/>
-      <c r="H3" s="138"/>
-      <c r="I3" s="138"/>
-      <c r="J3" s="138"/>
-      <c r="K3" s="138"/>
-      <c r="L3" s="138"/>
-      <c r="M3" s="139"/>
-      <c r="N3" s="124"/>
+      <c r="A3" s="142"/>
+      <c r="B3" s="133"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="134"/>
+      <c r="H3" s="134"/>
+      <c r="I3" s="134"/>
+      <c r="J3" s="134"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="134"/>
+      <c r="M3" s="135"/>
+      <c r="N3" s="142"/>
     </row>
     <row r="4" spans="1:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="123">
+      <c r="A4" s="141">
         <v>18</v>
       </c>
-      <c r="B4" s="140"/>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="141"/>
-      <c r="G4" s="141"/>
-      <c r="H4" s="141"/>
-      <c r="I4" s="141"/>
-      <c r="J4" s="141"/>
-      <c r="K4" s="141"/>
-      <c r="L4" s="141"/>
-      <c r="M4" s="142"/>
-      <c r="N4" s="123">
+      <c r="B4" s="136"/>
+      <c r="C4" s="137"/>
+      <c r="D4" s="137"/>
+      <c r="E4" s="137"/>
+      <c r="F4" s="137"/>
+      <c r="G4" s="137"/>
+      <c r="H4" s="137"/>
+      <c r="I4" s="137"/>
+      <c r="J4" s="137"/>
+      <c r="K4" s="137"/>
+      <c r="L4" s="137"/>
+      <c r="M4" s="138"/>
+      <c r="N4" s="141">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="124"/>
-      <c r="B5" s="125" t="s">
-        <v>255</v>
-      </c>
-      <c r="C5" s="126"/>
-      <c r="D5" s="129" t="s">
-        <v>255</v>
-      </c>
-      <c r="E5" s="130"/>
-      <c r="F5" s="129" t="s">
-        <v>255</v>
-      </c>
-      <c r="G5" s="130"/>
-      <c r="H5" s="129" t="s">
-        <v>255</v>
-      </c>
-      <c r="I5" s="130"/>
-      <c r="J5" s="129" t="s">
-        <v>255</v>
-      </c>
-      <c r="K5" s="130"/>
-      <c r="L5" s="129" t="s">
-        <v>255</v>
-      </c>
-      <c r="M5" s="133"/>
-      <c r="N5" s="124"/>
+      <c r="A5" s="142"/>
+      <c r="B5" s="123" t="s">
+        <v>253</v>
+      </c>
+      <c r="C5" s="128"/>
+      <c r="D5" s="121" t="s">
+        <v>253</v>
+      </c>
+      <c r="E5" s="122"/>
+      <c r="F5" s="121" t="s">
+        <v>253</v>
+      </c>
+      <c r="G5" s="122"/>
+      <c r="H5" s="121" t="s">
+        <v>253</v>
+      </c>
+      <c r="I5" s="122"/>
+      <c r="J5" s="121" t="s">
+        <v>253</v>
+      </c>
+      <c r="K5" s="122"/>
+      <c r="L5" s="121" t="s">
+        <v>253</v>
+      </c>
+      <c r="M5" s="127"/>
+      <c r="N5" s="142"/>
     </row>
     <row r="6" spans="1:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="123">
+      <c r="A6" s="141">
         <v>17</v>
       </c>
-      <c r="B6" s="125"/>
-      <c r="C6" s="126"/>
-      <c r="D6" s="125"/>
-      <c r="E6" s="131"/>
-      <c r="F6" s="125"/>
-      <c r="G6" s="131"/>
-      <c r="H6" s="125"/>
-      <c r="I6" s="131"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="131"/>
-      <c r="L6" s="125"/>
-      <c r="M6" s="126"/>
-      <c r="N6" s="123">
+      <c r="B6" s="123"/>
+      <c r="C6" s="128"/>
+      <c r="D6" s="123"/>
+      <c r="E6" s="124"/>
+      <c r="F6" s="123"/>
+      <c r="G6" s="124"/>
+      <c r="H6" s="123"/>
+      <c r="I6" s="124"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="124"/>
+      <c r="L6" s="123"/>
+      <c r="M6" s="128"/>
+      <c r="N6" s="141">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="124"/>
-      <c r="B7" s="127"/>
-      <c r="C7" s="128"/>
-      <c r="D7" s="127"/>
-      <c r="E7" s="132"/>
-      <c r="F7" s="127"/>
-      <c r="G7" s="132"/>
-      <c r="H7" s="127"/>
-      <c r="I7" s="132"/>
-      <c r="J7" s="127"/>
-      <c r="K7" s="132"/>
-      <c r="L7" s="127"/>
-      <c r="M7" s="128"/>
-      <c r="N7" s="124"/>
+      <c r="A7" s="142"/>
+      <c r="B7" s="125"/>
+      <c r="C7" s="129"/>
+      <c r="D7" s="125"/>
+      <c r="E7" s="126"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="126"/>
+      <c r="H7" s="125"/>
+      <c r="I7" s="126"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="126"/>
+      <c r="L7" s="125"/>
+      <c r="M7" s="129"/>
+      <c r="N7" s="142"/>
     </row>
     <row r="8" spans="1:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="121">
+      <c r="A8" s="139">
         <v>16</v>
       </c>
-      <c r="B8" s="122"/>
-      <c r="C8" s="121">
+      <c r="B8" s="140"/>
+      <c r="C8" s="139">
         <v>15</v>
       </c>
-      <c r="D8" s="122"/>
-      <c r="E8" s="121">
+      <c r="D8" s="140"/>
+      <c r="E8" s="139">
         <v>14</v>
       </c>
-      <c r="F8" s="122"/>
-      <c r="G8" s="121">
+      <c r="F8" s="140"/>
+      <c r="G8" s="139">
         <v>13</v>
       </c>
-      <c r="H8" s="122"/>
-      <c r="I8" s="121">
+      <c r="H8" s="140"/>
+      <c r="I8" s="139">
         <v>12</v>
       </c>
-      <c r="J8" s="122"/>
-      <c r="K8" s="121">
+      <c r="J8" s="140"/>
+      <c r="K8" s="139">
         <v>11</v>
       </c>
-      <c r="L8" s="122"/>
-      <c r="M8" s="121">
+      <c r="L8" s="140"/>
+      <c r="M8" s="139">
         <v>10</v>
       </c>
-      <c r="N8" s="122"/>
+      <c r="N8" s="140"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="F5:G7"/>
-    <mergeCell ref="H5:I7"/>
-    <mergeCell ref="J5:K7"/>
-    <mergeCell ref="L5:M7"/>
-    <mergeCell ref="B2:M4"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="E8:F8"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A6:A7"/>
@@ -7388,6 +6783,26 @@
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B5:C7"/>
     <mergeCell ref="D5:E7"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="F5:G7"/>
+    <mergeCell ref="H5:I7"/>
+    <mergeCell ref="J5:K7"/>
+    <mergeCell ref="L5:M7"/>
+    <mergeCell ref="B2:M4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -9178,31 +8593,31 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D1" t="s">
         <v>275</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>276</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>277</v>
-      </c>
-      <c r="E1" t="s">
-        <v>278</v>
-      </c>
-      <c r="F1" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B2">
         <f>30*2</f>
         <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D2">
         <v>27.7</v>
@@ -9210,14 +8625,14 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B3">
         <f>34*2</f>
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D3">
         <v>27.7</v>
@@ -9225,14 +8640,14 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B4">
         <f>18*3</f>
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D4">
         <v>30.75</v>
@@ -9240,222 +8655,222 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B5">
         <f>2*6+6*6</f>
         <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B6">
         <f>1*6+10*6</f>
         <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B7">
         <f>10*6+10</f>
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B8">
         <f>2*8*6</f>
         <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E8" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B9">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B10">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E10" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B11">
         <f>(30*6-B10)/5</f>
         <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E11" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B12">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C12" t="s">
+        <v>279</v>
+      </c>
+      <c r="E12" t="s">
         <v>281</v>
-      </c>
-      <c r="E12" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B13">
         <f>(15*6-B12)/5</f>
         <v>12</v>
       </c>
       <c r="C13" t="s">
+        <v>279</v>
+      </c>
+      <c r="E13" t="s">
         <v>281</v>
-      </c>
-      <c r="E13" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B18">
         <f>10*6</f>
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B19">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B20">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -9487,67 +8902,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>411</v>
+        <v>339</v>
       </c>
       <c r="B1" t="s">
-        <v>412</v>
+        <v>340</v>
       </c>
       <c r="C1" t="s">
-        <v>413</v>
+        <v>341</v>
       </c>
       <c r="D1" t="s">
-        <v>414</v>
+        <v>342</v>
       </c>
       <c r="E1" t="s">
-        <v>415</v>
+        <v>343</v>
       </c>
       <c r="F1" t="s">
-        <v>441</v>
+        <v>369</v>
       </c>
       <c r="G1" t="s">
-        <v>440</v>
+        <v>368</v>
       </c>
       <c r="H1" t="s">
-        <v>416</v>
+        <v>344</v>
       </c>
       <c r="I1" t="s">
-        <v>417</v>
+        <v>345</v>
       </c>
       <c r="J1" s="103" t="s">
-        <v>438</v>
+        <v>366</v>
       </c>
       <c r="K1" t="s">
-        <v>418</v>
+        <v>346</v>
       </c>
       <c r="L1" t="s">
-        <v>419</v>
+        <v>347</v>
       </c>
       <c r="M1" t="s">
-        <v>420</v>
+        <v>348</v>
       </c>
       <c r="N1" t="s">
-        <v>421</v>
+        <v>349</v>
       </c>
       <c r="O1" t="s">
-        <v>422</v>
+        <v>350</v>
       </c>
       <c r="P1" t="s">
-        <v>423</v>
+        <v>351</v>
       </c>
       <c r="Q1" t="s">
-        <v>424</v>
+        <v>352</v>
       </c>
       <c r="R1" t="s">
-        <v>425</v>
+        <v>353</v>
       </c>
       <c r="S1" t="s">
-        <v>426</v>
+        <v>354</v>
       </c>
       <c r="T1" t="s">
-        <v>427</v>
+        <v>355</v>
       </c>
       <c r="U1" t="s">
-        <v>439</v>
+        <v>367</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Modified cards after playtest session
Removed Investment to give up to 3 automatic hits during Trial
Removed Investment to provide private Donate action
Swapped Investment conditions of repeating Provincial and Court actions
Clarified Laws not quite in sync with current state of game
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4260" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E9160F4-F4CF-4F20-B7DC-ADF9830D065B}"/>
+  <xr:revisionPtr revIDLastSave="4334" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7FF52B8-417B-4081-8740-AA1E8D3555A0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7755" yWindow="3660" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="469">
   <si>
     <t>Standard Card</t>
   </si>
@@ -272,9 +272,6 @@
     <t>Heavy Overtme</t>
   </si>
   <si>
-    <t>You may repeat $L3 Provincial Actions per round</t>
-  </si>
-  <si>
     <t>Realistic Priorities</t>
   </si>
   <si>
@@ -407,9 +404,6 @@
     <t>Contingency Plans</t>
   </si>
   <si>
-    <t>Each Player must have at least $L6 Cards in hand or they will suffer sanctions on Monetize</t>
-  </si>
-  <si>
     <t>4D</t>
   </si>
   <si>
@@ -422,9 +416,6 @@
     <t>Worthless Procrastinators</t>
   </si>
   <si>
-    <t>No Player may have more than $L6 Cards in their hand or they will suffer sanctions on Monetize</t>
-  </si>
-  <si>
     <t>5D</t>
   </si>
   <si>
@@ -1016,9 +1007,6 @@
     <t>Desperate Attorneys</t>
   </si>
   <si>
-    <t>Mock Trials</t>
-  </si>
-  <si>
     <t>Players return one held Favor for each of their leader levels to each other if they have one</t>
   </si>
   <si>
@@ -1142,9 +1130,6 @@
     <t>Trade for up to $L3 additional Coins when Monetizing in the Court</t>
   </si>
   <si>
-    <t>Heavy Overtime</t>
-  </si>
-  <si>
     <t>Courtroom Gambling</t>
   </si>
   <si>
@@ -1178,15 +1163,6 @@
     <t>Abusive Power</t>
   </si>
   <si>
-    <t>Soup Kitchens</t>
-  </si>
-  <si>
-    <t>At least $L6 Players must use Deploy or all Players suffer sanctions on Donate</t>
-  </si>
-  <si>
-    <t>No more than $L6 Players may use Deploy or all Players suffer sanctions on Donate</t>
-  </si>
-  <si>
     <t>Stalled Front</t>
   </si>
   <si>
@@ -1211,9 +1187,6 @@
     <t>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
   </si>
   <si>
-    <t xml:space="preserve">You may repeat Court Actions with level 7 - $L6 (or higher) Leaders </t>
-  </si>
-  <si>
     <t>Send Troops up to Leader's Level to the Battlefield and gain half Troops in Coins</t>
   </si>
   <si>
@@ -1376,9 +1349,6 @@
     <t>Honorable Accountability</t>
   </si>
   <si>
-    <t>Add $L3 Hits to each Roll during a Trial</t>
-  </si>
-  <si>
     <t>Add $L6 additional dice to each Roll during a Trial</t>
   </si>
   <si>
@@ -1452,13 +1422,34 @@
   </si>
   <si>
     <t>Collect 4 Commodities</t>
-  </si>
-  <si>
-    <t>Provides Private Donate action with no penalty and convert $L3 additional Coins.</t>
   </si>
   <si>
     <t>Persian
 Troops</t>
+  </si>
+  <si>
+    <t>Each Player must Deploy at least $L6 Troops or they will suffer sanctions on Donate</t>
+  </si>
+  <si>
+    <t>No Player may Deploy more than $L6 Troops or they will suffer sanctions on Donate</t>
+  </si>
+  <si>
+    <t>Each Player must have at least $L6 Cards of each type in hand or they will suffer sanctions on Monetize</t>
+  </si>
+  <si>
+    <t>No Player may have more than $L6 Cards of each type in their hand or they will suffer sanctions on Monetize</t>
+  </si>
+  <si>
+    <t>Mock Trials</t>
+  </si>
+  <si>
+    <t>You may repeat $L3 Court Actions per round</t>
+  </si>
+  <si>
+    <t>Inspiring Command</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You may repeat Provincial Actions with level 7 - $L6 (or higher) Leaders </t>
   </si>
 </sst>
 </file>
@@ -2741,6 +2732,45 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2750,42 +2780,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2794,9 +2788,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4156,7 +4147,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="2"/>
@@ -4167,10 +4158,10 @@
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>14</v>
@@ -4179,10 +4170,10 @@
         <v>15</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>439</v>
+        <v>430</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="2"/>
@@ -4196,19 +4187,19 @@
         <v>17</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="3"/>
@@ -4228,13 +4219,13 @@
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="2"/>
@@ -4257,10 +4248,10 @@
         <v>29</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="3"/>
@@ -4283,10 +4274,10 @@
         <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="3"/>
@@ -4300,19 +4291,19 @@
         <v>41</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="2"/>
@@ -4323,7 +4314,7 @@
         <v>38</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>449</v>
+        <v>439</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>44</v>
@@ -4332,13 +4323,13 @@
         <v>39</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
@@ -4355,16 +4346,16 @@
         <v>49</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>443</v>
+        <v>434</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>447</v>
+        <v>437</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="2"/>
@@ -4375,22 +4366,22 @@
         <v>43</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>438</v>
+        <v>429</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>437</v>
+        <v>428</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="2"/>
@@ -4404,7 +4395,7 @@
         <v>57</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>50</v>
@@ -4416,7 +4407,7 @@
         <v>46</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="2"/>
@@ -4442,7 +4433,7 @@
         <v>52</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
@@ -4468,7 +4459,7 @@
         <v>42</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
@@ -4479,10 +4470,10 @@
         <v>60</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>71</v>
+        <v>467</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>389</v>
+        <v>468</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>63</v>
@@ -4494,7 +4485,7 @@
         <v>65</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="3"/>
@@ -4505,22 +4496,22 @@
         <v>66</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>366</v>
+        <v>71</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>76</v>
+        <v>466</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>69</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="2"/>
@@ -4531,10 +4522,10 @@
         <v>70</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>80</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>72</v>
@@ -4543,10 +4534,10 @@
         <v>73</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="2"/>
@@ -4557,22 +4548,22 @@
         <v>74</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="15" t="s">
-        <v>84</v>
-      </c>
       <c r="D18" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>36</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
@@ -4580,25 +4571,25 @@
     </row>
     <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="15" t="s">
-        <v>88</v>
-      </c>
       <c r="D19" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
@@ -4606,25 +4597,25 @@
     </row>
     <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>92</v>
-      </c>
       <c r="D20" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
@@ -4632,25 +4623,25 @@
     </row>
     <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="C21" s="15" t="s">
-        <v>96</v>
-      </c>
       <c r="D21" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="3"/>
@@ -4658,25 +4649,25 @@
     </row>
     <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C22" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>101</v>
-      </c>
       <c r="D22" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="3"/>
@@ -4684,19 +4675,19 @@
     </row>
     <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>444</v>
+        <v>441</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>370</v>
       </c>
       <c r="D23" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="15" t="s">
         <v>97</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>98</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="7"/>
@@ -4706,19 +4697,19 @@
     </row>
     <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>323</v>
+        <v>465</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>466</v>
+        <v>456</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="9"/>
@@ -4728,19 +4719,19 @@
     </row>
     <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>467</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>104</v>
-      </c>
       <c r="E25" s="15" t="s">
-        <v>468</v>
+        <v>458</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="7"/>
@@ -4750,19 +4741,19 @@
     </row>
     <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>400</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>409</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="E26" s="15" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4772,19 +4763,19 @@
     </row>
     <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="C27" s="16" t="s">
-        <v>115</v>
-      </c>
       <c r="D27" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4794,19 +4785,19 @@
     </row>
     <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>119</v>
-      </c>
       <c r="D28" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4816,19 +4807,19 @@
     </row>
     <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -4838,19 +4829,19 @@
     </row>
     <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>121</v>
+        <v>463</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="7"/>
@@ -4860,19 +4851,19 @@
     </row>
     <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>126</v>
+        <v>464</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="7"/>
@@ -4880,21 +4871,21 @@
       <c r="I31" s="3"/>
       <c r="J31" s="4"/>
     </row>
-    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>379</v>
+        <v>461</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -4904,19 +4895,19 @@
     </row>
     <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>380</v>
+        <v>462</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -4926,13 +4917,13 @@
     </row>
     <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="16"/>
@@ -4944,13 +4935,13 @@
     </row>
     <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="16"/>
@@ -4960,15 +4951,15 @@
       <c r="I35" s="3"/>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>378</v>
+        <v>432</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>470</v>
+        <v>433</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -4980,13 +4971,13 @@
     </row>
     <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -4998,13 +4989,13 @@
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -5016,13 +5007,13 @@
     </row>
     <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -5032,16 +5023,12 @@
       <c r="I39" s="3"/>
       <c r="J39" s="4"/>
     </row>
-    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>441</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>442</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="15"/>
       <c r="D40" s="6"/>
       <c r="E40" s="16"/>
       <c r="F40" s="6"/>
@@ -5050,16 +5037,12 @@
       <c r="I40" s="3"/>
       <c r="J40" s="4"/>
     </row>
-    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="C41" s="15" t="s">
-        <v>375</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="B41" s="6"/>
+      <c r="C41" s="15"/>
       <c r="D41" s="6"/>
       <c r="E41" s="16"/>
       <c r="F41" s="6"/>
@@ -5070,7 +5053,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="16"/>
@@ -5084,7 +5067,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="16"/>
@@ -5098,7 +5081,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="16"/>
@@ -5112,7 +5095,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="16"/>
@@ -5126,7 +5109,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="16"/>
@@ -5140,7 +5123,7 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="16"/>
@@ -5154,7 +5137,7 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="16"/>
@@ -5168,7 +5151,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="16"/>
@@ -5182,7 +5165,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="16"/>
@@ -5196,7 +5179,7 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B51" s="99"/>
       <c r="C51" s="100"/>
@@ -5210,7 +5193,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B52" s="99"/>
       <c r="C52" s="100"/>
@@ -5224,7 +5207,7 @@
     </row>
     <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="17"/>
@@ -5260,215 +5243,215 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1" s="49" t="s">
+        <v>155</v>
+      </c>
+      <c r="D1" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="E1" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="F1" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="G1" s="50" t="s">
+        <v>323</v>
+      </c>
+      <c r="H1" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="I1" s="51" t="s">
         <v>160</v>
-      </c>
-      <c r="F1" s="50" t="s">
-        <v>161</v>
-      </c>
-      <c r="G1" s="50" t="s">
-        <v>327</v>
-      </c>
-      <c r="H1" s="50" t="s">
-        <v>162</v>
-      </c>
-      <c r="I1" s="51" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="43" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="C2" s="45" t="s">
+        <v>161</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="E2" s="46" t="s">
+        <v>163</v>
+      </c>
+      <c r="F2" s="46" t="s">
         <v>164</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="G2" s="46" t="s">
         <v>165</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="H2" s="46" t="s">
         <v>166</v>
       </c>
-      <c r="F2" s="46" t="s">
-        <v>167</v>
-      </c>
-      <c r="G2" s="46" t="s">
-        <v>168</v>
-      </c>
-      <c r="H2" s="46" t="s">
-        <v>169</v>
-      </c>
       <c r="I2" s="46" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D3" s="38" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E3" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>168</v>
+      </c>
+      <c r="G3" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="H3" s="38" t="s">
+        <v>278</v>
+      </c>
+      <c r="I3" s="38" t="s">
         <v>170</v>
-      </c>
-      <c r="F3" s="38" t="s">
-        <v>171</v>
-      </c>
-      <c r="G3" s="38" t="s">
-        <v>172</v>
-      </c>
-      <c r="H3" s="38" t="s">
-        <v>281</v>
-      </c>
-      <c r="I3" s="38" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>173</v>
+      </c>
+      <c r="E4" s="38" t="s">
         <v>174</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="F4" s="38" t="s">
+        <v>354</v>
+      </c>
+      <c r="G4" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="C4" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="D4" s="38" t="s">
+      <c r="H4" s="38" t="s">
         <v>176</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="F4" s="38" t="s">
-        <v>358</v>
-      </c>
-      <c r="G4" s="38" t="s">
-        <v>178</v>
-      </c>
-      <c r="H4" s="38" t="s">
-        <v>179</v>
       </c>
       <c r="I4" s="41"/>
     </row>
     <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="F5" s="38" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="31" t="s">
-        <v>287</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>182</v>
-      </c>
-      <c r="F5" s="38" t="s">
-        <v>183</v>
-      </c>
       <c r="G5" s="38" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="H5" s="38" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="I5" s="41"/>
     </row>
     <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>183</v>
+      </c>
+      <c r="E6" s="38" t="s">
         <v>184</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="F6" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="C6" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>187</v>
-      </c>
-      <c r="F6" s="38" t="s">
-        <v>188</v>
-      </c>
       <c r="G6" s="38" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="I6" s="41"/>
     </row>
     <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F7" s="40" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="H7" s="38"/>
       <c r="I7" s="41"/>
     </row>
     <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>190</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>283</v>
+      </c>
+      <c r="F8" s="38" t="s">
         <v>192</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>193</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="D8" s="38" t="s">
-        <v>194</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>286</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>195</v>
       </c>
       <c r="G8" s="38"/>
       <c r="H8" s="38"/>
@@ -5476,22 +5459,22 @@
     </row>
     <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>195</v>
+      </c>
+      <c r="E9" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="F9" s="38" t="s">
         <v>197</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="D9" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>199</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>200</v>
       </c>
       <c r="G9" s="38"/>
       <c r="H9" s="38"/>
@@ -5499,19 +5482,19 @@
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
@@ -5520,17 +5503,17 @@
     </row>
     <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D11" s="38"/>
       <c r="E11" s="38" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
@@ -5539,17 +5522,17 @@
     </row>
     <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D12" s="38"/>
       <c r="E12" s="38" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F12" s="40"/>
       <c r="G12" s="38"/>
@@ -5558,17 +5541,17 @@
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D13" s="38"/>
       <c r="E13" s="38" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F13" s="40"/>
       <c r="G13" s="38"/>
@@ -5577,17 +5560,17 @@
     </row>
     <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D14" s="38"/>
       <c r="E14" s="38" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="F14" s="40"/>
       <c r="G14" s="38"/>
@@ -5596,13 +5579,13 @@
     </row>
     <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C15" s="34" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D15" s="38"/>
       <c r="E15" s="38"/>
@@ -5613,13 +5596,13 @@
     </row>
     <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D16" s="38"/>
       <c r="E16" s="38"/>
@@ -5630,13 +5613,13 @@
     </row>
     <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="33" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D17" s="38"/>
       <c r="E17" s="38"/>
@@ -5647,13 +5630,13 @@
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D18" s="38"/>
       <c r="E18" s="38"/>
@@ -5664,13 +5647,13 @@
     </row>
     <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C19" s="34" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D19" s="38"/>
       <c r="E19" s="38"/>
@@ -5681,13 +5664,13 @@
     </row>
     <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D20" s="38"/>
       <c r="E20" s="38"/>
@@ -5698,13 +5681,13 @@
     </row>
     <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="33" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="C21" s="34" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D21" s="38"/>
       <c r="E21" s="38"/>
@@ -5715,13 +5698,13 @@
     </row>
     <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="33" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D22" s="38"/>
       <c r="E22" s="38"/>
@@ -5732,13 +5715,13 @@
     </row>
     <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="33" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C23" s="34" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D23" s="38"/>
       <c r="E23" s="38"/>
@@ -5749,13 +5732,13 @@
     </row>
     <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="35" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B24" s="36" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D24" s="38"/>
       <c r="E24" s="38"/>
@@ -5766,13 +5749,13 @@
     </row>
     <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="35" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B25" s="36" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C25" s="37" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D25" s="39"/>
       <c r="E25" s="39"/>
@@ -5799,33 +5782,33 @@
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="61"/>
       <c r="B1" s="55" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" s="55" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" s="54" t="s">
+        <v>227</v>
+      </c>
+      <c r="E1" s="103" t="s">
         <v>228</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="F1" s="102" t="s">
         <v>229</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="G1" s="55" t="s">
         <v>230</v>
       </c>
-      <c r="E1" s="103" t="s">
-        <v>231</v>
-      </c>
-      <c r="F1" s="102" t="s">
-        <v>232</v>
-      </c>
-      <c r="G1" s="55" t="s">
-        <v>233</v>
-      </c>
       <c r="I1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="63" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C2" s="58" t="s">
         <v>67</v>
@@ -5834,47 +5817,47 @@
         <v>71</v>
       </c>
       <c r="E2" s="101" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F2" s="107" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G2" s="58" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B3" s="65" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="57" t="s">
-        <v>449</v>
+        <v>439</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="E3" s="104" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F3" s="53" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="G3" s="57" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I3" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B4" s="57" t="s">
         <v>61</v>
@@ -5883,27 +5866,27 @@
         <v>21</v>
       </c>
       <c r="D4" s="56" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E4" s="104" t="s">
         <v>75</v>
       </c>
       <c r="F4" s="56" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G4" s="57" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I4" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="63" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B5" s="62" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C5" s="62" t="s">
         <v>57</v>
@@ -5912,24 +5895,24 @@
         <v>17</v>
       </c>
       <c r="E5" s="105" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F5" s="108" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G5" s="106" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="I5" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="86" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B6" s="87" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C6" s="88" t="s">
         <v>34</v>
@@ -5938,205 +5921,205 @@
         <v>69</v>
       </c>
       <c r="E6" s="90" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F6" s="82" t="s">
         <v>58</v>
       </c>
       <c r="G6" s="91" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I6" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="66" t="s">
+        <v>236</v>
+      </c>
+      <c r="B7" s="66" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>312</v>
+      </c>
+      <c r="D7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E7" s="63" t="s">
         <v>239</v>
       </c>
-      <c r="B7" s="66" t="s">
+      <c r="F7" t="s">
         <v>240</v>
       </c>
-      <c r="C7" s="63" t="s">
-        <v>315</v>
-      </c>
-      <c r="D7" t="s">
-        <v>241</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>242</v>
-      </c>
-      <c r="F7" t="s">
-        <v>243</v>
-      </c>
       <c r="G7" s="63" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I7" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="84" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B8" s="84" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C8" s="80" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D8" s="84" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E8" s="80" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F8" s="84" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="G8" s="81" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I8" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="53" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C9" t="s">
+        <v>227</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>226</v>
+      </c>
+      <c r="E9" t="s">
         <v>230</v>
       </c>
-      <c r="D9" s="53" t="s">
-        <v>229</v>
-      </c>
-      <c r="E9" t="s">
-        <v>233</v>
-      </c>
       <c r="F9" s="53" t="s">
+        <v>225</v>
+      </c>
+      <c r="G9" s="65" t="s">
         <v>228</v>
-      </c>
-      <c r="G9" s="65" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="85" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B10" s="85" t="s">
+        <v>227</v>
+      </c>
+      <c r="C10" s="82" t="s">
         <v>230</v>
       </c>
-      <c r="C10" s="82" t="s">
-        <v>233</v>
-      </c>
       <c r="D10" s="85" t="s">
+        <v>225</v>
+      </c>
+      <c r="E10" s="82" t="s">
+        <v>229</v>
+      </c>
+      <c r="F10" s="85" t="s">
         <v>228</v>
       </c>
-      <c r="E10" s="82" t="s">
-        <v>232</v>
-      </c>
-      <c r="F10" s="85" t="s">
-        <v>231</v>
-      </c>
       <c r="G10" s="83" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>469</v>
+        <v>459</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>301</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>459</v>
+        <v>449</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>469</v>
+        <v>459</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -6150,99 +6133,99 @@
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="I18" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="I19" t="s">
         <v>297</v>
-      </c>
-      <c r="I19" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="E20" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D21" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="G22" s="2"/>
     </row>
@@ -6256,93 +6239,93 @@
     </row>
     <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="I24" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>207</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="I25" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E26" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="I26" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G27" s="2"/>
       <c r="I27" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -6354,7 +6337,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="I28" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -6366,7 +6349,7 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="I29" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -6519,208 +6502,208 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="126" t="s">
-        <v>246</v>
-      </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="128"/>
+      <c r="A1" s="127" t="s">
+        <v>243</v>
+      </c>
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="128"/>
+      <c r="F1" s="129"/>
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="129" t="s">
-        <v>471</v>
-      </c>
-      <c r="B2" s="129" t="s">
-        <v>471</v>
-      </c>
-      <c r="C2" s="129" t="s">
-        <v>471</v>
-      </c>
-      <c r="D2" s="129" t="s">
-        <v>471</v>
-      </c>
-      <c r="E2" s="129" t="s">
-        <v>471</v>
-      </c>
-      <c r="F2" s="129" t="s">
-        <v>471</v>
+      <c r="A2" s="123" t="s">
+        <v>460</v>
+      </c>
+      <c r="B2" s="123" t="s">
+        <v>460</v>
+      </c>
+      <c r="C2" s="123" t="s">
+        <v>460</v>
+      </c>
+      <c r="D2" s="123" t="s">
+        <v>460</v>
+      </c>
+      <c r="E2" s="123" t="s">
+        <v>460</v>
+      </c>
+      <c r="F2" s="123" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="118">
-        <v>0</v>
-      </c>
-      <c r="B3" s="119">
+      <c r="A3" s="115">
+        <v>0</v>
+      </c>
+      <c r="B3" s="116">
         <v>1</v>
       </c>
-      <c r="C3" s="119">
+      <c r="C3" s="116">
         <v>2</v>
       </c>
-      <c r="D3" s="118">
+      <c r="D3" s="115">
         <v>3</v>
       </c>
-      <c r="E3" s="119">
+      <c r="E3" s="116">
         <v>4</v>
       </c>
-      <c r="F3" s="118">
+      <c r="F3" s="115">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="120">
+      <c r="A4" s="117">
         <v>25</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>307</v>
-      </c>
-      <c r="F4" s="120">
+        <v>304</v>
+      </c>
+      <c r="F4" s="117">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="121">
+      <c r="A5" s="118">
         <v>24</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="114" t="s">
-        <v>184</v>
+        <v>177</v>
+      </c>
+      <c r="D5" s="111" t="s">
+        <v>181</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>189</v>
-      </c>
-      <c r="F5" s="120">
+        <v>186</v>
+      </c>
+      <c r="F5" s="117">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="120">
+      <c r="A6" s="117">
         <v>23</v>
       </c>
       <c r="B6" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="C6" s="28" t="s">
         <v>204</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="D6" s="29" t="s">
+        <v>325</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="F6" s="120">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="118">
+        <v>22</v>
+      </c>
+      <c r="B7" s="30" t="s">
         <v>207</v>
       </c>
-      <c r="D6" s="29" t="s">
-        <v>329</v>
-      </c>
-      <c r="E6" s="28" t="s">
-        <v>203</v>
-      </c>
-      <c r="F6" s="123">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="121">
-        <v>22</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>210</v>
-      </c>
       <c r="C7" s="30" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>372</v>
-      </c>
-      <c r="F7" s="120">
+        <v>367</v>
+      </c>
+      <c r="F7" s="117">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="120">
+      <c r="A8" s="117">
         <v>21</v>
       </c>
       <c r="B8" s="98" t="s">
-        <v>244</v>
-      </c>
-      <c r="C8" s="111" t="s">
-        <v>245</v>
-      </c>
-      <c r="D8" s="112"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="123">
+        <v>241</v>
+      </c>
+      <c r="C8" s="124" t="s">
+        <v>242</v>
+      </c>
+      <c r="D8" s="125"/>
+      <c r="E8" s="126"/>
+      <c r="F8" s="120">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="121">
+      <c r="A9" s="118">
         <v>20</v>
       </c>
       <c r="B9" s="109" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E9" s="110" t="s">
-        <v>372</v>
-      </c>
-      <c r="F9" s="120">
+        <v>367</v>
+      </c>
+      <c r="F9" s="117">
         <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="120">
+      <c r="A10" s="117">
         <v>19</v>
       </c>
-      <c r="B10" s="115" t="s">
+      <c r="B10" s="112" t="s">
+        <v>215</v>
+      </c>
+      <c r="C10" s="113" t="s">
         <v>218</v>
       </c>
-      <c r="C10" s="116" t="s">
-        <v>221</v>
-      </c>
-      <c r="D10" s="117" t="s">
-        <v>351</v>
-      </c>
-      <c r="E10" s="116" t="s">
-        <v>223</v>
-      </c>
-      <c r="F10" s="123">
+      <c r="D10" s="114" t="s">
+        <v>347</v>
+      </c>
+      <c r="E10" s="113" t="s">
+        <v>220</v>
+      </c>
+      <c r="F10" s="120">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="122">
+      <c r="A11" s="119">
         <v>18</v>
       </c>
-      <c r="B11" s="124">
+      <c r="B11" s="121">
         <v>17</v>
       </c>
-      <c r="C11" s="125">
+      <c r="C11" s="122">
         <v>16</v>
       </c>
-      <c r="D11" s="124">
+      <c r="D11" s="121">
         <v>15</v>
       </c>
-      <c r="E11" s="125">
+      <c r="E11" s="122">
         <v>14</v>
       </c>
-      <c r="F11" s="120">
+      <c r="F11" s="117">
         <v>13</v>
       </c>
     </row>
@@ -6860,11 +6843,11 @@
       </c>
       <c r="P1" s="67" t="str">
         <f>Cards!B15</f>
-        <v>Undeniable Advisors</v>
+        <v>Inspiring Command</v>
       </c>
       <c r="Q1" s="69" t="str">
         <f>Cards!B16</f>
-        <v>Heavy Overtime</v>
+        <v>Undeniable Advisors</v>
       </c>
       <c r="R1" s="67" t="str">
         <f>Cards!B17</f>
@@ -6892,11 +6875,11 @@
       </c>
       <c r="X1" s="67" t="str">
         <f>Cards!B23</f>
-        <v>Mock Trials</v>
+        <v>Boasting Propaganda</v>
       </c>
       <c r="Y1" s="69" t="str">
         <f>Cards!B24</f>
-        <v>Desperate Attorneys</v>
+        <v>Mock Trials</v>
       </c>
       <c r="Z1" s="67" t="str">
         <f>Cards!B25</f>
@@ -6944,7 +6927,7 @@
       </c>
       <c r="AK1" s="69" t="str">
         <f>Cards!B36</f>
-        <v>Soup Kitchens</v>
+        <v>One Man's Trash</v>
       </c>
       <c r="AL1" s="67" t="str">
         <f>Cards!B37</f>
@@ -7020,11 +7003,11 @@
       </c>
       <c r="BD1" s="69" t="str">
         <f t="shared" si="1"/>
-        <v>Undeniable Advisors</v>
+        <v>Inspiring Command</v>
       </c>
       <c r="BE1" s="67" t="str">
         <f t="shared" si="1"/>
-        <v>Heavy Overtime</v>
+        <v>Undeniable Advisors</v>
       </c>
       <c r="BF1" s="69" t="str">
         <f t="shared" si="1"/>
@@ -7052,11 +7035,11 @@
       </c>
       <c r="BL1" s="69" t="str">
         <f t="shared" si="2"/>
-        <v>Mock Trials</v>
+        <v>Boasting Propaganda</v>
       </c>
       <c r="BM1" s="67" t="str">
         <f t="shared" si="2"/>
-        <v>Desperate Attorneys</v>
+        <v>Mock Trials</v>
       </c>
       <c r="BN1" s="69" t="str">
         <f t="shared" si="2"/>
@@ -7147,11 +7130,11 @@
       </c>
       <c r="P2" s="93" t="str">
         <f>Cards!C15</f>
-        <v xml:space="preserve">You may repeat Court Actions with level 7 - $L6 (or higher) Leaders </v>
+        <v xml:space="preserve">You may repeat Provincial Actions with level 7 - $L6 (or higher) Leaders </v>
       </c>
       <c r="Q2" s="92" t="str">
         <f>Cards!C16</f>
-        <v>You may repeat $L3 Provincial Actions per round</v>
+        <v>You may repeat $L3 Court Actions per round</v>
       </c>
       <c r="R2" s="93" t="str">
         <f>Cards!C17</f>
@@ -7179,7 +7162,7 @@
       </c>
       <c r="X2" s="93" t="str">
         <f>Cards!C23</f>
-        <v>Add $L3 Hits to each Roll during a Trial</v>
+        <v>Convert $L3 additional Coins during Court Donate</v>
       </c>
       <c r="Y2" s="92" t="str">
         <f>Cards!C24</f>
@@ -7231,7 +7214,7 @@
       </c>
       <c r="AK2" s="92" t="str">
         <f>Cards!C36</f>
-        <v>Provides Private Donate action with no penalty and convert $L3 additional Coins.</v>
+        <v>Draw $L6 additional cards from the top of any discard pile during Brainstorm</v>
       </c>
       <c r="AL2" s="93" t="str">
         <f>Cards!C37</f>
@@ -7307,11 +7290,11 @@
       </c>
       <c r="BD2" s="92" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">You may repeat Court Actions with level 7 - $L6 (or higher) Leaders </v>
+        <v xml:space="preserve">You may repeat Provincial Actions with level 7 - $L6 (or higher) Leaders </v>
       </c>
       <c r="BE2" s="93" t="str">
         <f t="shared" si="1"/>
-        <v>You may repeat $L3 Provincial Actions per round</v>
+        <v>You may repeat $L3 Court Actions per round</v>
       </c>
       <c r="BF2" s="92" t="str">
         <f t="shared" si="1"/>
@@ -7339,7 +7322,7 @@
       </c>
       <c r="BL2" s="92" t="str">
         <f t="shared" si="2"/>
-        <v>Add $L3 Hits to each Roll during a Trial</v>
+        <v>Convert $L3 additional Coins during Court Donate</v>
       </c>
       <c r="BM2" s="93" t="str">
         <f t="shared" si="2"/>
@@ -7635,7 +7618,7 @@
       </c>
       <c r="BO3" s="67" t="str">
         <f t="shared" si="4"/>
-        <v>Soup Kitchens</v>
+        <v>One Man's Trash</v>
       </c>
       <c r="BP3" s="69" t="str">
         <f t="shared" si="4"/>
@@ -7770,19 +7753,19 @@
       </c>
       <c r="AC4" s="74" t="str">
         <f>Cards!E30</f>
-        <v>Each Player must have at least $L6 Cards in hand or they will suffer sanctions on Monetize</v>
+        <v>Each Player must have at least $L6 Cards of each type in hand or they will suffer sanctions on Monetize</v>
       </c>
       <c r="AD4" s="75" t="str">
         <f>Cards!E31</f>
-        <v>No Player may have more than $L6 Cards in their hand or they will suffer sanctions on Monetize</v>
+        <v>No Player may have more than $L6 Cards of each type in their hand or they will suffer sanctions on Monetize</v>
       </c>
       <c r="AE4" s="72" t="str">
         <f>Cards!E32</f>
-        <v>At least $L6 Players must use Deploy or all Players suffer sanctions on Donate</v>
+        <v>Each Player must Deploy at least $L6 Troops or they will suffer sanctions on Donate</v>
       </c>
       <c r="AF4" s="72" t="str">
         <f>Cards!E33</f>
-        <v>No more than $L6 Players may use Deploy or all Players suffer sanctions on Donate</v>
+        <v>No Player may Deploy more than $L6 Troops or they will suffer sanctions on Donate</v>
       </c>
       <c r="AG4" s="74" t="str">
         <f t="shared" ref="AG4:BL4" si="5">A4</f>
@@ -7898,19 +7881,19 @@
       </c>
       <c r="BI4" s="72" t="str">
         <f t="shared" si="5"/>
-        <v>Each Player must have at least $L6 Cards in hand or they will suffer sanctions on Monetize</v>
+        <v>Each Player must have at least $L6 Cards of each type in hand or they will suffer sanctions on Monetize</v>
       </c>
       <c r="BJ4" s="74" t="str">
         <f t="shared" si="5"/>
-        <v>No Player may have more than $L6 Cards in their hand or they will suffer sanctions on Monetize</v>
+        <v>No Player may have more than $L6 Cards of each type in their hand or they will suffer sanctions on Monetize</v>
       </c>
       <c r="BK4" s="72" t="str">
         <f t="shared" si="5"/>
-        <v>At least $L6 Players must use Deploy or all Players suffer sanctions on Donate</v>
+        <v>Each Player must Deploy at least $L6 Troops or they will suffer sanctions on Donate</v>
       </c>
       <c r="BL4" s="74" t="str">
         <f t="shared" si="5"/>
-        <v>No more than $L6 Players may use Deploy or all Players suffer sanctions on Donate</v>
+        <v>No Player may Deploy more than $L6 Troops or they will suffer sanctions on Donate</v>
       </c>
       <c r="BM4" s="72"/>
       <c r="BN4" s="92" t="str">
@@ -7919,7 +7902,7 @@
       </c>
       <c r="BO4" s="93" t="str">
         <f t="shared" si="4"/>
-        <v>Provides Private Donate action with no penalty and convert $L3 additional Coins.</v>
+        <v>Draw $L6 additional cards from the top of any discard pile during Brainstorm</v>
       </c>
       <c r="BP4" s="92" t="str">
         <f t="shared" si="4"/>
@@ -8519,31 +8502,31 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E1" t="s">
         <v>266</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>267</v>
-      </c>
-      <c r="D1" t="s">
-        <v>268</v>
-      </c>
-      <c r="E1" t="s">
-        <v>269</v>
-      </c>
-      <c r="F1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B2">
         <f>30*2</f>
         <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D2">
         <v>27.7</v>
@@ -8551,14 +8534,14 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B3">
         <f>34*2</f>
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D3">
         <v>27.7</v>
@@ -8566,14 +8549,14 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B4">
         <f>18*3</f>
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D4">
         <v>30.75</v>
@@ -8581,222 +8564,222 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B5">
         <f>2*6+6*6</f>
         <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B6">
         <f>1*6+10*6</f>
         <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E6" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B7">
         <f>10*6+10</f>
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E7" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B8">
         <f>2*8*6</f>
         <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E8" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B9">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B10">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E10" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B11">
         <f>(30*6-B10)/5</f>
         <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E11" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B12">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E12" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B13">
         <f>(15*6-B12)/5</f>
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E13" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B18">
         <f>10*6</f>
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B19">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B20">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -8817,8 +8800,7 @@
     <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" style="97" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.28515625" style="97" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
     <col min="12" max="19" width="11.85546875" style="97" bestFit="1" customWidth="1"/>
@@ -8828,67 +8810,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C1" t="s">
+        <v>330</v>
+      </c>
+      <c r="D1" t="s">
+        <v>331</v>
+      </c>
+      <c r="E1" t="s">
         <v>332</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F1" t="s">
+        <v>358</v>
+      </c>
+      <c r="G1" t="s">
+        <v>357</v>
+      </c>
+      <c r="H1" t="s">
         <v>333</v>
       </c>
-      <c r="C1" t="s">
+      <c r="I1" t="s">
         <v>334</v>
       </c>
-      <c r="D1" t="s">
+      <c r="J1" s="97" t="s">
+        <v>355</v>
+      </c>
+      <c r="K1" t="s">
         <v>335</v>
       </c>
-      <c r="E1" t="s">
+      <c r="L1" t="s">
         <v>336</v>
       </c>
-      <c r="F1" t="s">
-        <v>362</v>
-      </c>
-      <c r="G1" t="s">
-        <v>361</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="M1" t="s">
         <v>337</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
         <v>338</v>
       </c>
-      <c r="J1" s="97" t="s">
-        <v>359</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>339</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>340</v>
       </c>
-      <c r="M1" t="s">
+      <c r="Q1" t="s">
         <v>341</v>
       </c>
-      <c r="N1" t="s">
+      <c r="R1" t="s">
         <v>342</v>
       </c>
-      <c r="O1" t="s">
+      <c r="S1" t="s">
         <v>343</v>
       </c>
-      <c r="P1" t="s">
+      <c r="T1" t="s">
         <v>344</v>
       </c>
-      <c r="Q1" t="s">
-        <v>345</v>
-      </c>
-      <c r="R1" t="s">
-        <v>346</v>
-      </c>
-      <c r="S1" t="s">
-        <v>347</v>
-      </c>
-      <c r="T1" t="s">
-        <v>348</v>
-      </c>
       <c r="U1" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
@@ -9195,27 +9177,150 @@
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8" s="95">
+        <v>46138</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
       <c r="C8" s="96" t="b">
         <v>0</v>
       </c>
       <c r="D8" s="96" t="b">
         <v>0</v>
       </c>
+      <c r="E8">
+        <v>8</v>
+      </c>
+      <c r="F8">
+        <v>8</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" s="97">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="I8" s="97">
+        <v>0.69513888888888886</v>
+      </c>
+      <c r="J8" s="97">
+        <v>0.64444444444444449</v>
+      </c>
+      <c r="K8" s="97">
+        <v>0.65416666666666667</v>
+      </c>
+      <c r="L8" s="97">
+        <v>0.67013888888888884</v>
+      </c>
+      <c r="M8" s="97">
+        <v>0.69166666666666665</v>
+      </c>
+      <c r="U8" s="97">
+        <v>0.69513888888888886</v>
+      </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A9" s="95">
+        <v>46145</v>
+      </c>
+      <c r="B9">
+        <v>6</v>
+      </c>
       <c r="C9" s="96" t="b">
         <v>0</v>
       </c>
       <c r="D9" s="96" t="b">
         <v>0</v>
       </c>
+      <c r="E9">
+        <v>12</v>
+      </c>
+      <c r="F9">
+        <v>30</v>
+      </c>
+      <c r="G9">
+        <v>18</v>
+      </c>
+      <c r="H9" s="97">
+        <v>0.60624999999999996</v>
+      </c>
+      <c r="I9" s="97">
+        <v>0.71666666666666667</v>
+      </c>
+      <c r="J9" s="97">
+        <v>0.61250000000000004</v>
+      </c>
+      <c r="K9" s="97">
+        <v>0.62222222222222223</v>
+      </c>
+      <c r="L9" s="97">
+        <v>0.64027777777777772</v>
+      </c>
+      <c r="M9" s="97">
+        <v>0.65833333333333333</v>
+      </c>
+      <c r="N9" s="97">
+        <v>0.6791666666666667</v>
+      </c>
+      <c r="O9" s="97">
+        <v>0.69722222222222219</v>
+      </c>
+      <c r="P9" s="97">
+        <v>0.71250000000000002</v>
+      </c>
+      <c r="U9" s="97">
+        <v>0.71666666666666667</v>
+      </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10" s="95">
+        <v>46152</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
       <c r="C10" s="96" t="b">
         <v>0</v>
       </c>
       <c r="D10" s="96" t="b">
         <v>0</v>
+      </c>
+      <c r="E10">
+        <v>12</v>
+      </c>
+      <c r="F10">
+        <v>21</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" s="97">
+        <v>0.54791666666666672</v>
+      </c>
+      <c r="I10" s="97">
+        <v>0.625</v>
+      </c>
+      <c r="J10" s="97">
+        <v>0.55347222222222225</v>
+      </c>
+      <c r="K10" s="97">
+        <v>0.56180555555555556</v>
+      </c>
+      <c r="L10" s="97">
+        <v>0.57361111111111107</v>
+      </c>
+      <c r="M10" s="97">
+        <v>0.58611111111111114</v>
+      </c>
+      <c r="N10" s="97">
+        <v>0.60486111111111107</v>
+      </c>
+      <c r="O10" s="97">
+        <v>0.61875000000000002</v>
+      </c>
+      <c r="U10" s="97">
+        <v>0.625</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added some playtest records
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4334" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7FF52B8-417B-4081-8740-AA1E8D3555A0}"/>
+  <xr:revisionPtr revIDLastSave="4349" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09ACA5EE-1C52-ED4B-B3FE-21E376819C86}"/>
   <bookViews>
-    <workbookView xWindow="7755" yWindow="3660" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -2732,7 +2732,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4085,23 +4085,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5390625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5078125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.18359375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.01171875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -4127,7 +4127,7 @@
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>7</v>
       </c>
@@ -4153,7 +4153,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>13</v>
       </c>
@@ -4179,7 +4179,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="4"/>
     </row>
-    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>16</v>
       </c>
@@ -4205,7 +4205,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="4"/>
     </row>
-    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>20</v>
       </c>
@@ -4231,7 +4231,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="4"/>
     </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>25</v>
       </c>
@@ -4257,7 +4257,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
@@ -4283,7 +4283,7 @@
       <c r="I7" s="3"/>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>37</v>
       </c>
@@ -4309,7 +4309,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>38</v>
       </c>
@@ -4335,7 +4335,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>40</v>
       </c>
@@ -4361,7 +4361,7 @@
       <c r="I10" s="2"/>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>43</v>
       </c>
@@ -4387,7 +4387,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>47</v>
       </c>
@@ -4413,7 +4413,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>53</v>
       </c>
@@ -4439,7 +4439,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>56</v>
       </c>
@@ -4465,7 +4465,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>60</v>
       </c>
@@ -4491,7 +4491,7 @@
       <c r="I15" s="3"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>66</v>
       </c>
@@ -4517,7 +4517,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="4"/>
     </row>
-    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>70</v>
       </c>
@@ -4543,7 +4543,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>74</v>
       </c>
@@ -4569,7 +4569,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>77</v>
       </c>
@@ -4595,7 +4595,7 @@
       <c r="I19" s="2"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>81</v>
       </c>
@@ -4621,7 +4621,7 @@
       <c r="I20" s="3"/>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>85</v>
       </c>
@@ -4647,7 +4647,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>89</v>
       </c>
@@ -4673,7 +4673,7 @@
       <c r="I22" s="3"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>93</v>
       </c>
@@ -4695,7 +4695,7 @@
       <c r="I23" s="3"/>
       <c r="J23" s="4"/>
     </row>
-    <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>98</v>
       </c>
@@ -4717,7 +4717,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>102</v>
       </c>
@@ -4739,7 +4739,7 @@
       <c r="I25" s="3"/>
       <c r="J25" s="4"/>
     </row>
-    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>104</v>
       </c>
@@ -4761,7 +4761,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="4"/>
     </row>
-    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>106</v>
       </c>
@@ -4783,7 +4783,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="4"/>
     </row>
-    <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>109</v>
       </c>
@@ -4805,7 +4805,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="4"/>
     </row>
-    <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>112</v>
       </c>
@@ -4827,7 +4827,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="4"/>
     </row>
-    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
         <v>116</v>
       </c>
@@ -4849,7 +4849,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="4"/>
     </row>
-    <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
         <v>120</v>
       </c>
@@ -4871,7 +4871,7 @@
       <c r="I31" s="3"/>
       <c r="J31" s="4"/>
     </row>
-    <row r="32" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
         <v>124</v>
       </c>
@@ -4893,7 +4893,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="4"/>
     </row>
-    <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
         <v>127</v>
       </c>
@@ -4915,7 +4915,7 @@
       <c r="I33" s="3"/>
       <c r="J33" s="4"/>
     </row>
-    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A34" s="11" t="s">
         <v>130</v>
       </c>
@@ -4933,7 +4933,7 @@
       <c r="I34" s="3"/>
       <c r="J34" s="4"/>
     </row>
-    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
         <v>132</v>
       </c>
@@ -4951,7 +4951,7 @@
       <c r="I35" s="3"/>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
         <v>135</v>
       </c>
@@ -4969,7 +4969,7 @@
       <c r="I36" s="3"/>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
         <v>136</v>
       </c>
@@ -4987,7 +4987,7 @@
       <c r="I37" s="3"/>
       <c r="J37" s="4"/>
     </row>
-    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
         <v>137</v>
       </c>
@@ -5005,7 +5005,7 @@
       <c r="I38" s="3"/>
       <c r="J38" s="4"/>
     </row>
-    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
         <v>138</v>
       </c>
@@ -5023,7 +5023,7 @@
       <c r="I39" s="3"/>
       <c r="J39" s="4"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
         <v>139</v>
       </c>
@@ -5037,7 +5037,7 @@
       <c r="I40" s="3"/>
       <c r="J40" s="4"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>140</v>
       </c>
@@ -5051,7 +5051,7 @@
       <c r="I41" s="3"/>
       <c r="J41" s="4"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>141</v>
       </c>
@@ -5065,7 +5065,7 @@
       <c r="I42" s="3"/>
       <c r="J42" s="4"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
         <v>142</v>
       </c>
@@ -5079,7 +5079,7 @@
       <c r="I43" s="3"/>
       <c r="J43" s="4"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
         <v>143</v>
       </c>
@@ -5093,7 +5093,7 @@
       <c r="I44" s="3"/>
       <c r="J44" s="4"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
         <v>144</v>
       </c>
@@ -5107,7 +5107,7 @@
       <c r="I45" s="3"/>
       <c r="J45" s="4"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
         <v>145</v>
       </c>
@@ -5121,7 +5121,7 @@
       <c r="I46" s="3"/>
       <c r="J46" s="4"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
         <v>146</v>
       </c>
@@ -5135,7 +5135,7 @@
       <c r="I47" s="3"/>
       <c r="J47" s="4"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
         <v>147</v>
       </c>
@@ -5149,7 +5149,7 @@
       <c r="I48" s="3"/>
       <c r="J48" s="4"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
         <v>148</v>
       </c>
@@ -5163,7 +5163,7 @@
       <c r="I49" s="3"/>
       <c r="J49" s="4"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
         <v>149</v>
       </c>
@@ -5177,7 +5177,7 @@
       <c r="I50" s="3"/>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
         <v>150</v>
       </c>
@@ -5191,7 +5191,7 @@
       <c r="I51" s="3"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>151</v>
       </c>
@@ -5205,7 +5205,7 @@
       <c r="I52" s="3"/>
       <c r="J52" s="4"/>
     </row>
-    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>152</v>
       </c>
@@ -5228,20 +5228,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D195C1D-DB02-1743-BBD2-99104C1FFD33}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="37.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="39.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="40.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.71875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.86328125" customWidth="1"/>
+    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.55859375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.26171875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7890625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="39.546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="34.16796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="40.0859375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="47" t="s">
         <v>153</v>
       </c>
@@ -5270,7 +5270,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A2" s="43" t="s">
         <v>304</v>
       </c>
@@ -5299,7 +5299,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A3" s="33" t="s">
         <v>325</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="81" x14ac:dyDescent="0.2">
       <c r="A4" s="33" t="s">
         <v>171</v>
       </c>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="I4" s="41"/>
     </row>
-    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
         <v>177</v>
       </c>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="I5" s="41"/>
     </row>
-    <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A6" s="33" t="s">
         <v>181</v>
       </c>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="I6" s="41"/>
     </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
         <v>186</v>
       </c>
@@ -5434,7 +5434,7 @@
       <c r="H7" s="38"/>
       <c r="I7" s="41"/>
     </row>
-    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
         <v>189</v>
       </c>
@@ -5457,7 +5457,7 @@
       <c r="H8" s="38"/>
       <c r="I8" s="41"/>
     </row>
-    <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
         <v>193</v>
       </c>
@@ -5480,7 +5480,7 @@
       <c r="H9" s="38"/>
       <c r="I9" s="41"/>
     </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
         <v>453</v>
       </c>
@@ -5501,7 +5501,7 @@
       <c r="H10" s="38"/>
       <c r="I10" s="41"/>
     </row>
-    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
         <v>200</v>
       </c>
@@ -5520,7 +5520,7 @@
       <c r="H11" s="38"/>
       <c r="I11" s="41"/>
     </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
         <v>201</v>
       </c>
@@ -5539,7 +5539,7 @@
       <c r="H12" s="38"/>
       <c r="I12" s="41"/>
     </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
         <v>204</v>
       </c>
@@ -5558,7 +5558,7 @@
       <c r="H13" s="38"/>
       <c r="I13" s="41"/>
     </row>
-    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
         <v>207</v>
       </c>
@@ -5577,7 +5577,7 @@
       <c r="H14" s="38"/>
       <c r="I14" s="41"/>
     </row>
-    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
         <v>211</v>
       </c>
@@ -5594,7 +5594,7 @@
       <c r="H15" s="38"/>
       <c r="I15" s="41"/>
     </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
         <v>213</v>
       </c>
@@ -5611,7 +5611,7 @@
       <c r="H16" s="38"/>
       <c r="I16" s="41"/>
     </row>
-    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
         <v>367</v>
       </c>
@@ -5628,7 +5628,7 @@
       <c r="H17" s="38"/>
       <c r="I17" s="41"/>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
         <v>215</v>
       </c>
@@ -5645,7 +5645,7 @@
       <c r="H18" s="38"/>
       <c r="I18" s="41"/>
     </row>
-    <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
         <v>218</v>
       </c>
@@ -5662,7 +5662,7 @@
       <c r="H19" s="38"/>
       <c r="I19" s="41"/>
     </row>
-    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
         <v>220</v>
       </c>
@@ -5679,7 +5679,7 @@
       <c r="H20" s="38"/>
       <c r="I20" s="41"/>
     </row>
-    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
         <v>347</v>
       </c>
@@ -5696,7 +5696,7 @@
       <c r="H21" s="38"/>
       <c r="I21" s="41"/>
     </row>
-    <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
         <v>207</v>
       </c>
@@ -5713,7 +5713,7 @@
       <c r="H22" s="38"/>
       <c r="I22" s="41"/>
     </row>
-    <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
         <v>211</v>
       </c>
@@ -5730,7 +5730,7 @@
       <c r="H23" s="38"/>
       <c r="I23" s="41"/>
     </row>
-    <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="35" t="s">
         <v>213</v>
       </c>
@@ -5747,7 +5747,7 @@
       <c r="H24" s="38"/>
       <c r="I24" s="41"/>
     </row>
-    <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="35" t="s">
         <v>367</v>
       </c>
@@ -5773,13 +5773,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920DF489-FE6D-4819-BD1A-323DFAE597A3}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="30.66796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="61"/>
       <c r="B1" s="55" t="s">
         <v>225</v>
@@ -5803,7 +5803,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="63" t="s">
         <v>231</v>
       </c>
@@ -5829,7 +5829,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="63" t="s">
         <v>232</v>
       </c>
@@ -5855,7 +5855,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
         <v>233</v>
       </c>
@@ -5881,7 +5881,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="63" t="s">
         <v>234</v>
       </c>
@@ -5907,7 +5907,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="86" t="s">
         <v>235</v>
       </c>
@@ -5933,7 +5933,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="66" t="s">
         <v>236</v>
       </c>
@@ -5959,7 +5959,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="84" t="s">
         <v>287</v>
       </c>
@@ -5985,7 +5985,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="53" t="s">
         <v>288</v>
       </c>
@@ -6008,7 +6008,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="85" t="s">
         <v>289</v>
       </c>
@@ -6031,12 +6031,12 @@
         <v>226</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>313</v>
       </c>
@@ -6059,7 +6059,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
         <v>292</v>
@@ -6080,7 +6080,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
         <v>447</v>
@@ -6101,7 +6101,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
         <v>450</v>
@@ -6122,7 +6122,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -6131,7 +6131,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>314</v>
       </c>
@@ -6157,7 +6157,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
         <v>453</v>
@@ -6181,7 +6181,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
         <v>292</v>
@@ -6202,7 +6202,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
@@ -6221,7 +6221,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="D22" s="2" t="s">
@@ -6229,7 +6229,7 @@
       </c>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="D23" s="2"/>
@@ -6237,7 +6237,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>315</v>
       </c>
@@ -6263,7 +6263,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
         <v>201</v>
@@ -6287,7 +6287,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
         <v>414</v>
@@ -6311,7 +6311,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
@@ -6328,7 +6328,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -6340,7 +6340,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -6352,7 +6352,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -6361,7 +6361,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -6369,7 +6369,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -6377,7 +6377,7 @@
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -6385,7 +6385,7 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -6393,7 +6393,7 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -6401,7 +6401,7 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -6409,7 +6409,7 @@
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -6417,7 +6417,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -6425,7 +6425,7 @@
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -6433,7 +6433,7 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -6441,7 +6441,7 @@
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -6449,7 +6449,7 @@
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -6457,7 +6457,7 @@
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -6465,7 +6465,7 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -6473,7 +6473,7 @@
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48" s="3"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -6481,7 +6481,7 @@
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -6495,10 +6495,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4430D7D8-35BC-4E32-9DE8-E2E435ADAAA0}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="36" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="37.5" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="6" width="30.7109375" style="26" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="26"/>
+    <col min="1" max="6" width="30.66796875" style="26" customWidth="1"/>
+    <col min="7" max="16384" width="9.14453125" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
@@ -6721,66 +6721,66 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CEB427C-0CB4-4E8D-8367-36F6DD891282}">
   <dimension ref="A1:CA6"/>
-  <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="19.7734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" style="53"/>
-    <col min="2" max="2" width="19.7109375" style="65"/>
-    <col min="4" max="4" width="19.7109375" style="53"/>
-    <col min="6" max="6" width="19.7109375" style="53"/>
-    <col min="8" max="8" width="19.7109375" style="53"/>
-    <col min="10" max="10" width="19.7109375" style="53"/>
-    <col min="12" max="12" width="19.7109375" style="53"/>
-    <col min="14" max="14" width="19.7109375" style="53"/>
-    <col min="16" max="16" width="19.7109375" style="53"/>
-    <col min="18" max="18" width="19.7109375" style="53"/>
-    <col min="20" max="20" width="19.7109375" style="53"/>
-    <col min="22" max="22" width="19.7109375" style="53"/>
-    <col min="24" max="24" width="19.7109375" style="53"/>
-    <col min="26" max="26" width="19.7109375" style="53"/>
-    <col min="28" max="28" width="19.7109375" style="53"/>
-    <col min="30" max="30" width="19.7109375" style="71"/>
-    <col min="31" max="32" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.7109375" customWidth="1"/>
-    <col min="42" max="42" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="19.7109375" style="71" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="19.7109375" style="71" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="19.7109375" style="53"/>
-    <col min="63" max="63" width="19.7109375" style="53"/>
-    <col min="65" max="65" width="19.7109375" style="53"/>
-    <col min="67" max="67" width="19.7109375" style="53"/>
-    <col min="69" max="70" width="19.7109375" style="53"/>
-    <col min="71" max="71" width="19.7109375" style="65"/>
-    <col min="73" max="73" width="19.7109375" style="53"/>
-    <col min="75" max="75" width="19.7109375" style="53"/>
-    <col min="77" max="77" width="19.7109375" style="53"/>
-    <col min="79" max="79" width="19.7109375" style="53"/>
+    <col min="1" max="1" width="19.7734375" style="53"/>
+    <col min="2" max="2" width="19.7734375" style="65"/>
+    <col min="4" max="4" width="19.7734375" style="53"/>
+    <col min="6" max="6" width="19.7734375" style="53"/>
+    <col min="8" max="8" width="19.7734375" style="53"/>
+    <col min="10" max="10" width="19.7734375" style="53"/>
+    <col min="12" max="12" width="19.7734375" style="53"/>
+    <col min="14" max="14" width="19.7734375" style="53"/>
+    <col min="16" max="16" width="19.7734375" style="53"/>
+    <col min="18" max="18" width="19.7734375" style="53"/>
+    <col min="20" max="20" width="19.7734375" style="53"/>
+    <col min="22" max="22" width="19.7734375" style="53"/>
+    <col min="24" max="24" width="19.7734375" style="53"/>
+    <col min="26" max="26" width="19.7734375" style="53"/>
+    <col min="28" max="28" width="19.7734375" style="53"/>
+    <col min="30" max="30" width="19.7734375" style="71"/>
+    <col min="31" max="32" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.7734375" customWidth="1"/>
+    <col min="42" max="42" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="19.7734375" style="71" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="19.7734375" style="71" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="19.7734375" style="53"/>
+    <col min="63" max="63" width="19.7734375" style="53"/>
+    <col min="65" max="65" width="19.7734375" style="53"/>
+    <col min="67" max="67" width="19.7734375" style="53"/>
+    <col min="69" max="70" width="19.7734375" style="53"/>
+    <col min="71" max="71" width="19.7734375" style="65"/>
+    <col min="73" max="73" width="19.7734375" style="53"/>
+    <col min="75" max="75" width="19.7734375" style="53"/>
+    <col min="77" max="77" width="19.7734375" style="53"/>
+    <col min="79" max="79" width="19.7734375" style="53"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="67" t="str">
         <f>Cards!B2</f>
         <v>Fillibuster</v>
@@ -7067,7 +7067,7 @@
       <c r="BY1" s="67"/>
       <c r="CA1" s="67"/>
     </row>
-    <row r="2" spans="1:79" s="92" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:79" s="92" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="93" t="str">
         <f>Cards!C2</f>
         <v>Move the deliberated Law $L6 additional places back in the queue during Postpone</v>
@@ -7354,7 +7354,7 @@
       <c r="BY2" s="93"/>
       <c r="CA2" s="93"/>
     </row>
-    <row r="3" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="67" t="str">
         <f>Cards!D2</f>
         <v>Full Coffers</v>
@@ -7638,7 +7638,7 @@
       <c r="BY3" s="67"/>
       <c r="CA3" s="67"/>
     </row>
-    <row r="4" spans="1:79" s="74" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:79" s="74" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="72" t="str">
         <f>Cards!E2</f>
         <v>The Royal Bank must have at least $L6 Coins or all Players suffer sanctions on Undermarket Actions</v>
@@ -7922,7 +7922,7 @@
       <c r="BY4" s="72"/>
       <c r="CA4" s="72"/>
     </row>
-    <row r="5" spans="1:79" s="78" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:79" s="78" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="76" t="str">
         <f>Cards!F2</f>
         <v>Fickle Mercenaries</v>
@@ -8202,7 +8202,7 @@
       <c r="BY5" s="76"/>
       <c r="CA5" s="76"/>
     </row>
-    <row r="6" spans="1:79" s="74" customFormat="1" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:79" s="74" customFormat="1" ht="81.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="72" t="str">
         <f>Cards!G2</f>
         <v>Give $2D6 Troops to $R</v>
@@ -8491,16 +8491,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BDA35E-BFC3-134A-A064-89D65A8B31CF}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.50390625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.22265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>263</v>
       </c>
@@ -8517,7 +8517,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>244</v>
       </c>
@@ -8532,7 +8532,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>245</v>
       </c>
@@ -8547,7 +8547,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>246</v>
       </c>
@@ -8562,7 +8562,7 @@
         <v>30.75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>247</v>
       </c>
@@ -8574,7 +8574,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>259</v>
       </c>
@@ -8589,7 +8589,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>248</v>
       </c>
@@ -8604,7 +8604,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>249</v>
       </c>
@@ -8619,7 +8619,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>250</v>
       </c>
@@ -8631,7 +8631,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>251</v>
       </c>
@@ -8646,7 +8646,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>252</v>
       </c>
@@ -8661,7 +8661,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>253</v>
       </c>
@@ -8676,7 +8676,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>254</v>
       </c>
@@ -8691,7 +8691,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>255</v>
       </c>
@@ -8702,7 +8702,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>256</v>
       </c>
@@ -8713,7 +8713,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>257</v>
       </c>
@@ -8724,7 +8724,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>258</v>
       </c>
@@ -8735,7 +8735,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>262</v>
       </c>
@@ -8747,7 +8747,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>261</v>
       </c>
@@ -8759,7 +8759,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>260</v>
       </c>
@@ -8771,7 +8771,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>275</v>
       </c>
@@ -8791,24 +8791,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC83F89-2724-CA43-A519-59213A612B31}">
   <dimension ref="A1:U55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24" style="95" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" style="97" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
-    <col min="12" max="19" width="11.85546875" style="97" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" style="97" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.9453125" style="95" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.72265625" customWidth="1"/>
+    <col min="4" max="4" width="8.33984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.27734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5078125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.97265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.43359375" style="97" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.22265625" style="97" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.43359375" style="97" bestFit="1" customWidth="1"/>
+    <col min="12" max="19" width="11.8359375" style="97" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.9140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.5078125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>328</v>
       </c>
@@ -8873,7 +8873,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="95">
         <v>46075</v>
       </c>
@@ -8917,7 +8917,7 @@
         <v>0.92638888888888893</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="95">
         <v>46089</v>
       </c>
@@ -8973,7 +8973,7 @@
         <v>0.86527777777777781</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="95">
         <v>46105</v>
       </c>
@@ -9026,7 +9026,7 @@
         <v>0.92777777777777781</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="95">
         <v>46118</v>
       </c>
@@ -9079,7 +9079,7 @@
         <v>0.9194444444444444</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="95">
         <v>46124</v>
       </c>
@@ -9123,7 +9123,7 @@
         <v>0.74583333333333335</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="95">
         <v>46131</v>
       </c>
@@ -9176,7 +9176,7 @@
         <v>0.70277777777777772</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="95">
         <v>46138</v>
       </c>
@@ -9220,7 +9220,7 @@
         <v>0.69513888888888886</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="95">
         <v>46145</v>
       </c>
@@ -9273,7 +9273,7 @@
         <v>0.71666666666666667</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="95">
         <v>46152</v>
       </c>
@@ -9323,15 +9323,60 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A11" s="95">
+        <v>46158</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
       <c r="C11" s="96" t="b">
         <v>0</v>
       </c>
       <c r="D11" s="96" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="E11">
+        <v>12</v>
+      </c>
+      <c r="F11">
+        <v>24</v>
+      </c>
+      <c r="G11">
+        <v>12</v>
+      </c>
+      <c r="H11" s="97">
+        <v>0.84236111111111112</v>
+      </c>
+      <c r="I11" s="97">
+        <v>0.99236111111111114</v>
+      </c>
+      <c r="J11" s="97">
+        <v>0.85902777777777772</v>
+      </c>
+      <c r="K11" s="97">
+        <v>0.87222222222222223</v>
+      </c>
+      <c r="L11" s="97">
+        <v>0.88958333333333328</v>
+      </c>
+      <c r="M11" s="97">
+        <v>0.90625</v>
+      </c>
+      <c r="N11" s="97">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="O11" s="97">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="P11" s="97">
+        <v>0.98888888888888893</v>
+      </c>
+      <c r="U11" s="97">
+        <v>0.99236111111111114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C12" s="96" t="b">
         <v>0</v>
       </c>
@@ -9339,7 +9384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C13" s="96" t="b">
         <v>0</v>
       </c>
@@ -9347,7 +9392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C14" s="96" t="b">
         <v>0</v>
       </c>
@@ -9355,7 +9400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C15" s="96" t="b">
         <v>0</v>
       </c>
@@ -9363,7 +9408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C16" s="96" t="b">
         <v>0</v>
       </c>
@@ -9371,7 +9416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C17" s="96" t="b">
         <v>0</v>
       </c>
@@ -9379,7 +9424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C18" s="96" t="b">
         <v>0</v>
       </c>
@@ -9387,7 +9432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C19" s="96" t="b">
         <v>0</v>
       </c>
@@ -9395,7 +9440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C20" s="96" t="b">
         <v>0</v>
       </c>
@@ -9403,7 +9448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C21" s="96" t="b">
         <v>0</v>
       </c>
@@ -9411,7 +9456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C22" s="96" t="b">
         <v>0</v>
       </c>
@@ -9419,7 +9464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C23" s="96" t="b">
         <v>0</v>
       </c>
@@ -9427,7 +9472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C24" s="96" t="b">
         <v>0</v>
       </c>
@@ -9435,7 +9480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C25" s="96" t="b">
         <v>0</v>
       </c>
@@ -9443,7 +9488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C26" s="96" t="b">
         <v>0</v>
       </c>
@@ -9451,7 +9496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C27" s="96" t="b">
         <v>0</v>
       </c>
@@ -9459,7 +9504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C28" s="96" t="b">
         <v>0</v>
       </c>
@@ -9467,7 +9512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C29" s="96" t="b">
         <v>0</v>
       </c>
@@ -9475,7 +9520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C30" s="96" t="b">
         <v>0</v>
       </c>
@@ -9483,7 +9528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C31" s="96" t="b">
         <v>0</v>
       </c>
@@ -9491,7 +9536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C32" s="96" t="b">
         <v>0</v>
       </c>
@@ -9499,7 +9544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C33" s="96" t="b">
         <v>0</v>
       </c>
@@ -9507,7 +9552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C34" s="96" t="b">
         <v>0</v>
       </c>
@@ -9515,7 +9560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C35" s="96" t="b">
         <v>0</v>
       </c>
@@ -9523,7 +9568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C36" s="96" t="b">
         <v>0</v>
       </c>
@@ -9531,7 +9576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C37" s="96" t="b">
         <v>0</v>
       </c>
@@ -9539,7 +9584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C38" s="96" t="b">
         <v>0</v>
       </c>
@@ -9547,7 +9592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C39" s="96" t="b">
         <v>0</v>
       </c>
@@ -9555,7 +9600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C40" s="96" t="b">
         <v>0</v>
       </c>
@@ -9563,7 +9608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C41" s="96" t="b">
         <v>0</v>
       </c>
@@ -9571,7 +9616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C42" s="96" t="b">
         <v>0</v>
       </c>
@@ -9579,7 +9624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C43" s="96" t="b">
         <v>0</v>
       </c>
@@ -9587,7 +9632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C44" s="96" t="b">
         <v>0</v>
       </c>
@@ -9595,7 +9640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C45" s="96" t="b">
         <v>0</v>
       </c>
@@ -9603,7 +9648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C46" s="96" t="b">
         <v>0</v>
       </c>
@@ -9611,7 +9656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C47" s="96" t="b">
         <v>0</v>
       </c>
@@ -9619,7 +9664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C48" s="96" t="b">
         <v>0</v>
       </c>
@@ -9627,7 +9672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C49" s="96" t="b">
         <v>0</v>
       </c>
@@ -9635,7 +9680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C50" s="96" t="b">
         <v>0</v>
       </c>
@@ -9643,7 +9688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C51" s="96" t="b">
         <v>0</v>
       </c>
@@ -9651,7 +9696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C52" s="96" t="b">
         <v>0</v>
       </c>
@@ -9659,7 +9704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C53" s="96" t="b">
         <v>0</v>
       </c>
@@ -9667,7 +9712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C54" s="96" t="b">
         <v>0</v>
       </c>
@@ -9675,7 +9720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C55" s="96" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Cleaned up training manuals
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4360" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A30327A-1BCC-0146-A681-773EE6088D85}"/>
+  <xr:revisionPtr revIDLastSave="4361" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{814644E0-E163-4C0A-B310-8877049B5630}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="472">
   <si>
     <t>Standard Card</t>
   </si>
@@ -993,9 +993,6 @@
   </si>
   <si>
     <t>Accuse Veteran</t>
-  </si>
-  <si>
-    <t>Desperate Attorneys</t>
   </si>
   <si>
     <t>Players return one held Favor for each of their leader levels to each other if they have one</t>
@@ -2744,7 +2741,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4097,23 +4094,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.6171875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.58984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5390625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.58984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.58984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.58984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5078125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.18359375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39.01171875" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -4139,7 +4136,7 @@
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
-    <row r="2" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>7</v>
       </c>
@@ -4159,21 +4156,21 @@
         <v>12</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="2"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C3" s="24" t="s">
         <v>349</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>350</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>14</v>
@@ -4182,16 +4179,16 @@
         <v>15</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="2"/>
       <c r="J3" s="4"/>
     </row>
-    <row r="4" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>16</v>
       </c>
@@ -4199,7 +4196,7 @@
         <v>17</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
@@ -4211,13 +4208,13 @@
         <v>19</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="3"/>
       <c r="J4" s="4"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>20</v>
       </c>
@@ -4237,13 +4234,13 @@
         <v>24</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="2"/>
       <c r="J5" s="4"/>
     </row>
-    <row r="6" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>25</v>
       </c>
@@ -4260,16 +4257,16 @@
         <v>29</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="3"/>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
@@ -4286,16 +4283,16 @@
         <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>416</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>417</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="3"/>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>37</v>
       </c>
@@ -4303,7 +4300,7 @@
         <v>41</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>315</v>
@@ -4312,21 +4309,21 @@
         <v>314</v>
       </c>
       <c r="F8" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>418</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>419</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="2"/>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>38</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>44</v>
@@ -4338,16 +4335,16 @@
         <v>314</v>
       </c>
       <c r="F9" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>420</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>421</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>40</v>
       </c>
@@ -4358,48 +4355,48 @@
         <v>49</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F10" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>422</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>423</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="2"/>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>43</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="2"/>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>47</v>
       </c>
@@ -4407,7 +4404,7 @@
         <v>57</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>50</v>
@@ -4419,13 +4416,13 @@
         <v>46</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="2"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>53</v>
       </c>
@@ -4445,13 +4442,13 @@
         <v>52</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>56</v>
       </c>
@@ -4465,45 +4462,45 @@
         <v>58</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>42</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>59</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>464</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>465</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>62</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>63</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="3"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>64</v>
       </c>
@@ -4511,25 +4508,25 @@
         <v>69</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>67</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="2"/>
       <c r="J16" s="4"/>
     </row>
-    <row r="17" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>68</v>
       </c>
@@ -4546,16 +4543,16 @@
         <v>71</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="2"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>72</v>
       </c>
@@ -4569,19 +4566,19 @@
         <v>74</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>36</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>75</v>
       </c>
@@ -4595,19 +4592,19 @@
         <v>78</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>79</v>
       </c>
@@ -4621,19 +4618,19 @@
         <v>82</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>83</v>
       </c>
@@ -4647,19 +4644,19 @@
         <v>86</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="3"/>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>87</v>
       </c>
@@ -4673,33 +4670,33 @@
         <v>90</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="3"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>91</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>94</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="7"/>
@@ -4707,21 +4704,21 @@
       <c r="I23" s="3"/>
       <c r="J23" s="4"/>
     </row>
-    <row r="24" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>95</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>98</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="9"/>
@@ -4729,7 +4726,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>99</v>
       </c>
@@ -4737,13 +4734,13 @@
         <v>104</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="7"/>
@@ -4751,7 +4748,7 @@
       <c r="I25" s="3"/>
       <c r="J25" s="4"/>
     </row>
-    <row r="26" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>101</v>
       </c>
@@ -4759,13 +4756,13 @@
         <v>107</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4773,7 +4770,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="4"/>
     </row>
-    <row r="27" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>103</v>
       </c>
@@ -4787,7 +4784,7 @@
         <v>105</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4795,7 +4792,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="4"/>
     </row>
-    <row r="28" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>106</v>
       </c>
@@ -4809,7 +4806,7 @@
         <v>108</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4817,7 +4814,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="4"/>
     </row>
-    <row r="29" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>109</v>
       </c>
@@ -4831,7 +4828,7 @@
         <v>112</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -4839,7 +4836,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="4"/>
     </row>
-    <row r="30" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>113</v>
       </c>
@@ -4853,7 +4850,7 @@
         <v>116</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="7"/>
@@ -4861,7 +4858,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="4"/>
     </row>
-    <row r="31" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>117</v>
       </c>
@@ -4875,7 +4872,7 @@
         <v>120</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="7"/>
@@ -4883,7 +4880,7 @@
       <c r="I31" s="3"/>
       <c r="J31" s="4"/>
     </row>
-    <row r="32" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>121</v>
       </c>
@@ -4891,13 +4888,13 @@
         <v>128</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -4905,7 +4902,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="4"/>
     </row>
-    <row r="33" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>124</v>
       </c>
@@ -4916,10 +4913,10 @@
         <v>131</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -4927,21 +4924,21 @@
       <c r="I33" s="3"/>
       <c r="J33" s="4"/>
     </row>
-    <row r="34" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>127</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C34" s="15" t="s">
         <v>347</v>
       </c>
-      <c r="C34" s="15" t="s">
-        <v>348</v>
-      </c>
       <c r="D34" s="6" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="7"/>
@@ -4949,21 +4946,21 @@
       <c r="I34" s="3"/>
       <c r="J34" s="4"/>
     </row>
-    <row r="35" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>129</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="7"/>
@@ -4971,15 +4968,15 @@
       <c r="I35" s="3"/>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>132</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="C36" s="15" t="s">
         <v>429</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>430</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -4989,15 +4986,15 @@
       <c r="I36" s="3"/>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>133</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -5007,15 +5004,15 @@
       <c r="I37" s="3"/>
       <c r="J37" s="4"/>
     </row>
-    <row r="38" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>134</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -5025,15 +5022,15 @@
       <c r="I38" s="3"/>
       <c r="J38" s="4"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>135</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -5043,7 +5040,7 @@
       <c r="I39" s="3"/>
       <c r="J39" s="4"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>136</v>
       </c>
@@ -5057,7 +5054,7 @@
       <c r="I40" s="3"/>
       <c r="J40" s="4"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>137</v>
       </c>
@@ -5071,7 +5068,7 @@
       <c r="I41" s="3"/>
       <c r="J41" s="4"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>138</v>
       </c>
@@ -5085,7 +5082,7 @@
       <c r="I42" s="3"/>
       <c r="J42" s="4"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>139</v>
       </c>
@@ -5099,7 +5096,7 @@
       <c r="I43" s="3"/>
       <c r="J43" s="4"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>140</v>
       </c>
@@ -5113,7 +5110,7 @@
       <c r="I44" s="3"/>
       <c r="J44" s="4"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>141</v>
       </c>
@@ -5127,7 +5124,7 @@
       <c r="I45" s="3"/>
       <c r="J45" s="4"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>142</v>
       </c>
@@ -5141,7 +5138,7 @@
       <c r="I46" s="3"/>
       <c r="J46" s="4"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>143</v>
       </c>
@@ -5155,7 +5152,7 @@
       <c r="I47" s="3"/>
       <c r="J47" s="4"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>144</v>
       </c>
@@ -5169,7 +5166,7 @@
       <c r="I48" s="3"/>
       <c r="J48" s="4"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>145</v>
       </c>
@@ -5183,7 +5180,7 @@
       <c r="I49" s="3"/>
       <c r="J49" s="4"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>146</v>
       </c>
@@ -5197,7 +5194,7 @@
       <c r="I50" s="3"/>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
         <v>147</v>
       </c>
@@ -5211,7 +5208,7 @@
       <c r="I51" s="3"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
         <v>148</v>
       </c>
@@ -5225,7 +5222,7 @@
       <c r="I52" s="3"/>
       <c r="J52" s="4"/>
     </row>
-    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
         <v>149</v>
       </c>
@@ -5248,20 +5245,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D195C1D-DB02-1743-BBD2-99104C1FFD33}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.71875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.86328125" customWidth="1"/>
-    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.55859375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="37.26171875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.7890625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="39.546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="34.16796875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="40.0859375" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="39.5703125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="34.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="40.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="47" t="s">
         <v>150</v>
       </c>
@@ -5281,7 +5278,7 @@
         <v>155</v>
       </c>
       <c r="G1" s="50" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H1" s="50" t="s">
         <v>156</v>
@@ -5290,12 +5287,12 @@
         <v>157</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="43" t="s">
         <v>301</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C2" s="45" t="s">
         <v>158</v>
@@ -5316,15 +5313,15 @@
         <v>163</v>
       </c>
       <c r="I2" s="46" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C3" s="34" t="s">
         <v>158</v>
@@ -5348,7 +5345,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="81" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>168</v>
       </c>
@@ -5365,7 +5362,7 @@
         <v>171</v>
       </c>
       <c r="F4" s="38" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G4" s="38" t="s">
         <v>172</v>
@@ -5375,7 +5372,7 @@
       </c>
       <c r="I4" s="41"/>
     </row>
-    <row r="5" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>174</v>
       </c>
@@ -5395,14 +5392,14 @@
         <v>177</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H5" s="38" t="s">
         <v>274</v>
       </c>
       <c r="I5" s="41"/>
     </row>
-    <row r="6" spans="1:9" ht="108" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>178</v>
       </c>
@@ -5422,14 +5419,14 @@
         <v>182</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I6" s="41"/>
     </row>
-    <row r="7" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>183</v>
       </c>
@@ -5440,7 +5437,7 @@
         <v>158</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E7" s="38" t="s">
         <v>279</v>
@@ -5454,7 +5451,7 @@
       <c r="H7" s="38"/>
       <c r="I7" s="41"/>
     </row>
-    <row r="8" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
         <v>186</v>
       </c>
@@ -5477,7 +5474,7 @@
       <c r="H8" s="38"/>
       <c r="I8" s="41"/>
     </row>
-    <row r="9" spans="1:9" ht="108" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>190</v>
       </c>
@@ -5500,9 +5497,9 @@
       <c r="H9" s="38"/>
       <c r="I9" s="41"/>
     </row>
-    <row r="10" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B10" s="31" t="s">
         <v>195</v>
@@ -5511,7 +5508,7 @@
         <v>158</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E10" s="38" t="s">
         <v>196</v>
@@ -5521,26 +5518,26 @@
       <c r="H10" s="38"/>
       <c r="I10" s="41"/>
     </row>
-    <row r="11" spans="1:9" ht="68.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
         <v>197</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C11" s="34" t="s">
         <v>158</v>
       </c>
       <c r="D11" s="38"/>
       <c r="E11" s="38" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
       <c r="H11" s="38"/>
       <c r="I11" s="41"/>
     </row>
-    <row r="12" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>198</v>
       </c>
@@ -5559,7 +5556,7 @@
       <c r="H12" s="38"/>
       <c r="I12" s="41"/>
     </row>
-    <row r="13" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
         <v>201</v>
       </c>
@@ -5578,7 +5575,7 @@
       <c r="H13" s="38"/>
       <c r="I13" s="41"/>
     </row>
-    <row r="14" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
         <v>204</v>
       </c>
@@ -5597,7 +5594,7 @@
       <c r="H14" s="38"/>
       <c r="I14" s="41"/>
     </row>
-    <row r="15" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>208</v>
       </c>
@@ -5614,7 +5611,7 @@
       <c r="H15" s="38"/>
       <c r="I15" s="41"/>
     </row>
-    <row r="16" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>210</v>
       </c>
@@ -5631,12 +5628,12 @@
       <c r="H16" s="38"/>
       <c r="I16" s="41"/>
     </row>
-    <row r="17" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="33" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C17" s="34" t="s">
         <v>206</v>
@@ -5648,7 +5645,7 @@
       <c r="H17" s="38"/>
       <c r="I17" s="41"/>
     </row>
-    <row r="18" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
         <v>212</v>
       </c>
@@ -5665,7 +5662,7 @@
       <c r="H18" s="38"/>
       <c r="I18" s="41"/>
     </row>
-    <row r="19" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
         <v>215</v>
       </c>
@@ -5682,7 +5679,7 @@
       <c r="H19" s="38"/>
       <c r="I19" s="41"/>
     </row>
-    <row r="20" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
         <v>217</v>
       </c>
@@ -5699,12 +5696,12 @@
       <c r="H20" s="38"/>
       <c r="I20" s="41"/>
     </row>
-    <row r="21" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="B21" s="31" t="s">
         <v>344</v>
-      </c>
-      <c r="B21" s="31" t="s">
-        <v>345</v>
       </c>
       <c r="C21" s="34" t="s">
         <v>214</v>
@@ -5716,7 +5713,7 @@
       <c r="H21" s="38"/>
       <c r="I21" s="41"/>
     </row>
-    <row r="22" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="33" t="s">
         <v>204</v>
       </c>
@@ -5733,7 +5730,7 @@
       <c r="H22" s="38"/>
       <c r="I22" s="41"/>
     </row>
-    <row r="23" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="33" t="s">
         <v>208</v>
       </c>
@@ -5750,7 +5747,7 @@
       <c r="H23" s="38"/>
       <c r="I23" s="41"/>
     </row>
-    <row r="24" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="35" t="s">
         <v>210</v>
       </c>
@@ -5767,12 +5764,12 @@
       <c r="H24" s="38"/>
       <c r="I24" s="41"/>
     </row>
-    <row r="25" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="35" t="s">
+        <v>363</v>
+      </c>
+      <c r="B25" s="36" t="s">
         <v>364</v>
-      </c>
-      <c r="B25" s="36" t="s">
-        <v>365</v>
       </c>
       <c r="C25" s="37" t="s">
         <v>214</v>
@@ -5793,13 +5790,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920DF489-FE6D-4819-BD1A-323DFAE597A3}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.1015625" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="30.66796875" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="61"/>
       <c r="B1" s="55" t="s">
         <v>222</v>
@@ -5823,7 +5820,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="63" t="s">
         <v>228</v>
       </c>
@@ -5849,7 +5846,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
         <v>229</v>
       </c>
@@ -5857,16 +5854,16 @@
         <v>41</v>
       </c>
       <c r="C3" s="57" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E3" s="104" t="s">
         <v>92</v>
       </c>
       <c r="F3" s="53" t="s">
-        <v>317</v>
+        <v>461</v>
       </c>
       <c r="G3" s="57" t="s">
         <v>125</v>
@@ -5875,7 +5872,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
         <v>230</v>
       </c>
@@ -5898,10 +5895,10 @@
         <v>107</v>
       </c>
       <c r="I4" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="63" t="s">
         <v>231</v>
       </c>
@@ -5915,19 +5912,19 @@
         <v>17</v>
       </c>
       <c r="E5" s="105" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F5" s="108" t="s">
         <v>80</v>
       </c>
       <c r="G5" s="106" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="I5" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="86" t="s">
         <v>232</v>
       </c>
@@ -5953,7 +5950,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="66" t="s">
         <v>233</v>
       </c>
@@ -5979,7 +5976,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="84" t="s">
         <v>284</v>
       </c>
@@ -6005,7 +6002,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="53" t="s">
         <v>285</v>
       </c>
@@ -6028,7 +6025,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="85" t="s">
         <v>286</v>
       </c>
@@ -6051,59 +6048,59 @@
         <v>223</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>310</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>289</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>296</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
         <v>289</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>295</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>183</v>
@@ -6112,22 +6109,22 @@
         <v>291</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>445</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>446</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>178</v>
@@ -6136,13 +6133,13 @@
         <v>183</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -6151,7 +6148,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>311</v>
       </c>
@@ -6165,25 +6162,25 @@
         <v>293</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>292</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I18" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>289</v>
@@ -6201,38 +6198,38 @@
         <v>294</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
         <v>289</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>290</v>
       </c>
       <c r="E20" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
         <v>289</v>
       </c>
       <c r="D21" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>290</v>
@@ -6241,7 +6238,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="D22" s="2" t="s">
@@ -6249,7 +6246,7 @@
       </c>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="D23" s="2"/>
@@ -6257,7 +6254,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>312</v>
       </c>
@@ -6274,16 +6271,16 @@
         <v>297</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>305</v>
       </c>
       <c r="I24" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
         <v>198</v>
@@ -6298,19 +6295,19 @@
         <v>316</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I25" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>215</v>
@@ -6319,7 +6316,7 @@
         <v>198</v>
       </c>
       <c r="E26" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>198</v>
@@ -6331,14 +6328,14 @@
         <v>303</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
         <v>300</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>301</v>
@@ -6348,7 +6345,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -6357,10 +6354,10 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="I28" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -6369,10 +6366,10 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="I29" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -6381,7 +6378,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -6389,7 +6386,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -6397,7 +6394,7 @@
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -6405,7 +6402,7 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -6413,7 +6410,7 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -6421,7 +6418,7 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -6429,7 +6426,7 @@
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -6437,7 +6434,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -6445,7 +6442,7 @@
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -6453,7 +6450,7 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -6461,7 +6458,7 @@
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -6469,7 +6466,7 @@
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -6477,7 +6474,7 @@
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -6485,7 +6482,7 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -6493,7 +6490,7 @@
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B48" s="3"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -6501,7 +6498,7 @@
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -6515,10 +6512,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4430D7D8-35BC-4E32-9DE8-E2E435ADAAA0}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="37.5" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="36" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="6" width="30.66796875" style="26" customWidth="1"/>
-    <col min="7" max="16384" width="9.14453125" style="26"/>
+    <col min="1" max="6" width="30.7109375" style="26" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
@@ -6533,22 +6530,22 @@
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="123" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B2" s="123" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C2" s="123" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D2" s="123" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="E2" s="123" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F2" s="123" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
@@ -6576,7 +6573,7 @@
         <v>25</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C4" s="28" t="s">
         <v>186</v>
@@ -6622,7 +6619,7 @@
         <v>201</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E6" s="28" t="s">
         <v>197</v>
@@ -6645,7 +6642,7 @@
         <v>210</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F7" s="117">
         <v>9</v>
@@ -6681,7 +6678,7 @@
         <v>210</v>
       </c>
       <c r="E9" s="110" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F9" s="117">
         <v>11</v>
@@ -6698,7 +6695,7 @@
         <v>215</v>
       </c>
       <c r="D10" s="114" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E10" s="113" t="s">
         <v>217</v>
@@ -6741,66 +6738,66 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CEB427C-0CB4-4E8D-8367-36F6DD891282}">
   <dimension ref="A1:CA6"/>
-  <sheetFormatPr defaultColWidth="19.7734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.7734375" style="53"/>
-    <col min="2" max="2" width="19.7734375" style="65"/>
-    <col min="4" max="4" width="19.7734375" style="53"/>
-    <col min="6" max="6" width="19.7734375" style="53"/>
-    <col min="8" max="8" width="19.7734375" style="53"/>
-    <col min="10" max="10" width="19.7734375" style="53"/>
-    <col min="12" max="12" width="19.7734375" style="53"/>
-    <col min="14" max="14" width="19.7734375" style="53"/>
-    <col min="16" max="16" width="19.7734375" style="53"/>
-    <col min="18" max="18" width="19.7734375" style="53"/>
-    <col min="20" max="20" width="19.7734375" style="53"/>
-    <col min="22" max="22" width="19.7734375" style="53"/>
-    <col min="24" max="24" width="19.7734375" style="53"/>
-    <col min="26" max="26" width="19.7734375" style="53"/>
-    <col min="28" max="28" width="19.7734375" style="53"/>
-    <col min="30" max="30" width="19.7734375" style="71"/>
-    <col min="31" max="32" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.7734375" customWidth="1"/>
-    <col min="42" max="42" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="19.7734375" style="71" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="19.7734375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="19.7734375" style="71" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="19.7734375" style="53"/>
-    <col min="63" max="63" width="19.7734375" style="53"/>
-    <col min="65" max="65" width="19.7734375" style="53"/>
-    <col min="67" max="67" width="19.7734375" style="53"/>
-    <col min="69" max="70" width="19.7734375" style="53"/>
-    <col min="71" max="71" width="19.7734375" style="65"/>
-    <col min="73" max="73" width="19.7734375" style="53"/>
-    <col min="75" max="75" width="19.7734375" style="53"/>
-    <col min="77" max="77" width="19.7734375" style="53"/>
-    <col min="79" max="79" width="19.7734375" style="53"/>
+    <col min="1" max="1" width="19.7109375" style="53"/>
+    <col min="2" max="2" width="19.7109375" style="65"/>
+    <col min="4" max="4" width="19.7109375" style="53"/>
+    <col min="6" max="6" width="19.7109375" style="53"/>
+    <col min="8" max="8" width="19.7109375" style="53"/>
+    <col min="10" max="10" width="19.7109375" style="53"/>
+    <col min="12" max="12" width="19.7109375" style="53"/>
+    <col min="14" max="14" width="19.7109375" style="53"/>
+    <col min="16" max="16" width="19.7109375" style="53"/>
+    <col min="18" max="18" width="19.7109375" style="53"/>
+    <col min="20" max="20" width="19.7109375" style="53"/>
+    <col min="22" max="22" width="19.7109375" style="53"/>
+    <col min="24" max="24" width="19.7109375" style="53"/>
+    <col min="26" max="26" width="19.7109375" style="53"/>
+    <col min="28" max="28" width="19.7109375" style="53"/>
+    <col min="30" max="30" width="19.7109375" style="71"/>
+    <col min="31" max="32" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.7109375" customWidth="1"/>
+    <col min="42" max="42" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="19.7109375" style="71" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="19.7109375" style="71" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="19.7109375" style="53"/>
+    <col min="63" max="63" width="19.7109375" style="53"/>
+    <col min="65" max="65" width="19.7109375" style="53"/>
+    <col min="67" max="67" width="19.7109375" style="53"/>
+    <col min="69" max="70" width="19.7109375" style="53"/>
+    <col min="71" max="71" width="19.7109375" style="65"/>
+    <col min="73" max="73" width="19.7109375" style="53"/>
+    <col min="75" max="75" width="19.7109375" style="53"/>
+    <col min="77" max="77" width="19.7109375" style="53"/>
+    <col min="79" max="79" width="19.7109375" style="53"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="str">
         <f>Cards!B2</f>
         <v>Fillibuster</v>
@@ -7087,7 +7084,7 @@
       <c r="BY1" s="67"/>
       <c r="CA1" s="67"/>
     </row>
-    <row r="2" spans="1:79" s="92" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:79" s="92" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="93" t="str">
         <f>Cards!C2</f>
         <v>Move the deliberated Law $L6 additional places back in the queue during Postpone</v>
@@ -7374,7 +7371,7 @@
       <c r="BY2" s="93"/>
       <c r="CA2" s="93"/>
     </row>
-    <row r="3" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="67" t="str">
         <f>Cards!D2</f>
         <v>Full Coffers</v>
@@ -7658,7 +7655,7 @@
       <c r="BY3" s="67"/>
       <c r="CA3" s="67"/>
     </row>
-    <row r="4" spans="1:79" s="74" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:79" s="74" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="72" t="str">
         <f>Cards!E2</f>
         <v>The Royal Bank must have at least $L6 Coins or all Players suffer sanctions on Undermarket Actions</v>
@@ -7942,7 +7939,7 @@
       <c r="BY4" s="72"/>
       <c r="CA4" s="72"/>
     </row>
-    <row r="5" spans="1:79" s="78" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:79" s="78" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="76" t="str">
         <f>Cards!F2</f>
         <v>Fickle Mercenaries</v>
@@ -8222,7 +8219,7 @@
       <c r="BY5" s="76"/>
       <c r="CA5" s="76"/>
     </row>
-    <row r="6" spans="1:79" s="74" customFormat="1" ht="81.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:79" s="74" customFormat="1" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="72" t="str">
         <f>Cards!G2</f>
         <v>Give $2D6 Troops to $R</v>
@@ -8511,16 +8508,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BDA35E-BFC3-134A-A064-89D65A8B31CF}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.50390625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.22265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>260</v>
       </c>
@@ -8537,7 +8534,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>241</v>
       </c>
@@ -8552,7 +8549,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>242</v>
       </c>
@@ -8567,7 +8564,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>243</v>
       </c>
@@ -8582,7 +8579,7 @@
         <v>30.75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>244</v>
       </c>
@@ -8594,7 +8591,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>256</v>
       </c>
@@ -8609,7 +8606,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>245</v>
       </c>
@@ -8624,7 +8621,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>246</v>
       </c>
@@ -8639,7 +8636,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>247</v>
       </c>
@@ -8651,7 +8648,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>248</v>
       </c>
@@ -8666,7 +8663,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>249</v>
       </c>
@@ -8681,7 +8678,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>250</v>
       </c>
@@ -8696,7 +8693,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>251</v>
       </c>
@@ -8711,7 +8708,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>252</v>
       </c>
@@ -8722,7 +8719,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>253</v>
       </c>
@@ -8733,7 +8730,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>254</v>
       </c>
@@ -8744,7 +8741,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>255</v>
       </c>
@@ -8755,7 +8752,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>259</v>
       </c>
@@ -8767,7 +8764,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>258</v>
       </c>
@@ -8779,7 +8776,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>257</v>
       </c>
@@ -8791,7 +8788,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>272</v>
       </c>
@@ -8811,89 +8808,89 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC83F89-2724-CA43-A519-59213A612B31}">
   <dimension ref="A1:U55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.9453125" style="95" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.72265625" customWidth="1"/>
-    <col min="4" max="4" width="8.33984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.27734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5078125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.97265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="11.43359375" style="97" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.22265625" style="97" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.43359375" style="97" bestFit="1" customWidth="1"/>
-    <col min="12" max="19" width="11.8359375" style="97" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.9140625" style="97" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.5078125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24" style="95" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" style="97" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
+    <col min="12" max="19" width="11.85546875" style="97" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.85546875" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B1" t="s">
         <v>325</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>326</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>327</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>328</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>354</v>
+      </c>
+      <c r="G1" t="s">
+        <v>353</v>
+      </c>
+      <c r="H1" t="s">
         <v>329</v>
       </c>
-      <c r="F1" t="s">
-        <v>355</v>
-      </c>
-      <c r="G1" t="s">
-        <v>354</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>330</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="97" t="s">
+        <v>351</v>
+      </c>
+      <c r="K1" t="s">
         <v>331</v>
       </c>
-      <c r="J1" s="97" t="s">
+      <c r="L1" t="s">
+        <v>332</v>
+      </c>
+      <c r="M1" t="s">
+        <v>333</v>
+      </c>
+      <c r="N1" t="s">
+        <v>334</v>
+      </c>
+      <c r="O1" t="s">
+        <v>335</v>
+      </c>
+      <c r="P1" t="s">
+        <v>336</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>337</v>
+      </c>
+      <c r="R1" t="s">
+        <v>338</v>
+      </c>
+      <c r="S1" t="s">
+        <v>339</v>
+      </c>
+      <c r="T1" t="s">
+        <v>340</v>
+      </c>
+      <c r="U1" t="s">
         <v>352</v>
       </c>
-      <c r="K1" t="s">
-        <v>332</v>
-      </c>
-      <c r="L1" t="s">
-        <v>333</v>
-      </c>
-      <c r="M1" t="s">
-        <v>334</v>
-      </c>
-      <c r="N1" t="s">
-        <v>335</v>
-      </c>
-      <c r="O1" t="s">
-        <v>336</v>
-      </c>
-      <c r="P1" t="s">
-        <v>337</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>338</v>
-      </c>
-      <c r="R1" t="s">
-        <v>339</v>
-      </c>
-      <c r="S1" t="s">
-        <v>340</v>
-      </c>
-      <c r="T1" t="s">
-        <v>341</v>
-      </c>
-      <c r="U1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="95">
         <v>46075</v>
       </c>
@@ -8937,7 +8934,7 @@
         <v>0.92638888888888893</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="95">
         <v>46089</v>
       </c>
@@ -8993,7 +8990,7 @@
         <v>0.86527777777777781</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="95">
         <v>46105</v>
       </c>
@@ -9046,7 +9043,7 @@
         <v>0.92777777777777781</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="95">
         <v>46118</v>
       </c>
@@ -9099,7 +9096,7 @@
         <v>0.9194444444444444</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="95">
         <v>46124</v>
       </c>
@@ -9143,7 +9140,7 @@
         <v>0.74583333333333335</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="95">
         <v>46131</v>
       </c>
@@ -9196,7 +9193,7 @@
         <v>0.70277777777777772</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="95">
         <v>46138</v>
       </c>
@@ -9240,7 +9237,7 @@
         <v>0.69513888888888886</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="95">
         <v>46145</v>
       </c>
@@ -9293,7 +9290,7 @@
         <v>0.71666666666666667</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="95">
         <v>46152</v>
       </c>
@@ -9343,7 +9340,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="95">
         <v>46158</v>
       </c>
@@ -9396,7 +9393,7 @@
         <v>0.99236111111111114</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C12" s="96" t="b">
         <v>0</v>
       </c>
@@ -9404,7 +9401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C13" s="96" t="b">
         <v>0</v>
       </c>
@@ -9412,7 +9409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C14" s="96" t="b">
         <v>0</v>
       </c>
@@ -9420,7 +9417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C15" s="96" t="b">
         <v>0</v>
       </c>
@@ -9428,7 +9425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C16" s="96" t="b">
         <v>0</v>
       </c>
@@ -9436,7 +9433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C17" s="96" t="b">
         <v>0</v>
       </c>
@@ -9444,7 +9441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C18" s="96" t="b">
         <v>0</v>
       </c>
@@ -9452,7 +9449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C19" s="96" t="b">
         <v>0</v>
       </c>
@@ -9460,7 +9457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C20" s="96" t="b">
         <v>0</v>
       </c>
@@ -9468,7 +9465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C21" s="96" t="b">
         <v>0</v>
       </c>
@@ -9476,7 +9473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C22" s="96" t="b">
         <v>0</v>
       </c>
@@ -9484,7 +9481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C23" s="96" t="b">
         <v>0</v>
       </c>
@@ -9492,7 +9489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C24" s="96" t="b">
         <v>0</v>
       </c>
@@ -9500,7 +9497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C25" s="96" t="b">
         <v>0</v>
       </c>
@@ -9508,7 +9505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C26" s="96" t="b">
         <v>0</v>
       </c>
@@ -9516,7 +9513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C27" s="96" t="b">
         <v>0</v>
       </c>
@@ -9524,7 +9521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C28" s="96" t="b">
         <v>0</v>
       </c>
@@ -9532,7 +9529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C29" s="96" t="b">
         <v>0</v>
       </c>
@@ -9540,7 +9537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C30" s="96" t="b">
         <v>0</v>
       </c>
@@ -9548,7 +9545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C31" s="96" t="b">
         <v>0</v>
       </c>
@@ -9556,7 +9553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C32" s="96" t="b">
         <v>0</v>
       </c>
@@ -9564,7 +9561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C33" s="96" t="b">
         <v>0</v>
       </c>
@@ -9572,7 +9569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C34" s="96" t="b">
         <v>0</v>
       </c>
@@ -9580,7 +9577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C35" s="96" t="b">
         <v>0</v>
       </c>
@@ -9588,7 +9585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C36" s="96" t="b">
         <v>0</v>
       </c>
@@ -9596,7 +9593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C37" s="96" t="b">
         <v>0</v>
       </c>
@@ -9604,7 +9601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C38" s="96" t="b">
         <v>0</v>
       </c>
@@ -9612,7 +9609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C39" s="96" t="b">
         <v>0</v>
       </c>
@@ -9620,7 +9617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C40" s="96" t="b">
         <v>0</v>
       </c>
@@ -9628,7 +9625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C41" s="96" t="b">
         <v>0</v>
       </c>
@@ -9636,7 +9633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C42" s="96" t="b">
         <v>0</v>
       </c>
@@ -9644,7 +9641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C43" s="96" t="b">
         <v>0</v>
       </c>
@@ -9652,7 +9649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C44" s="96" t="b">
         <v>0</v>
       </c>
@@ -9660,7 +9657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C45" s="96" t="b">
         <v>0</v>
       </c>
@@ -9668,7 +9665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C46" s="96" t="b">
         <v>0</v>
       </c>
@@ -9676,7 +9673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C47" s="96" t="b">
         <v>0</v>
       </c>
@@ -9684,7 +9681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C48" s="96" t="b">
         <v>0</v>
       </c>
@@ -9692,7 +9689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C49" s="96" t="b">
         <v>0</v>
       </c>
@@ -9700,7 +9697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C50" s="96" t="b">
         <v>0</v>
       </c>
@@ -9708,7 +9705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C51" s="96" t="b">
         <v>0</v>
       </c>
@@ -9716,7 +9713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C52" s="96" t="b">
         <v>0</v>
       </c>
@@ -9724,7 +9721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C53" s="96" t="b">
         <v>0</v>
       </c>
@@ -9732,7 +9729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C54" s="96" t="b">
         <v>0</v>
       </c>
@@ -9740,7 +9737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C55" s="96" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Finished first draft of rulebook
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4361" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{814644E0-E163-4C0A-B310-8877049B5630}"/>
+  <xr:revisionPtr revIDLastSave="4363" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B5A9EBE-F8CB-C648-82A1-9886ADB36BD6}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="474">
   <si>
     <t>Standard Card</t>
   </si>
@@ -377,9 +377,6 @@
     <t>Information Security</t>
   </si>
   <si>
-    <t>Subtract $L3 from Scheme Card rolls</t>
-  </si>
-  <si>
     <t>Suspicious Advisors</t>
   </si>
   <si>
@@ -1230,9 +1227,6 @@
   </si>
   <si>
     <t>Target Player rolls a die. If the result is a 6 or is higher than half their Troops, the Scheme is executed. Otherwise, the Scheme fails. (Scheme Guard Roll)</t>
-  </si>
-  <si>
-    <t>Subtract $L3 from Scheme Guard rolls. An unmodified 6 always succeeds.</t>
   </si>
   <si>
     <t>Deploy 2 Troops for no Coins.</t>
@@ -1459,6 +1453,12 @@
   </si>
   <si>
     <t>Partisan Contributions</t>
+  </si>
+  <si>
+    <t>Subtract $L3 from Scheme Damage rolls</t>
+  </si>
+  <si>
+    <t>Subtract $L3 from Scheme Evasion rolls. An unmodified 6 always succeeds.</t>
   </si>
 </sst>
 </file>
@@ -2741,7 +2741,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4094,23 +4094,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5390625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.58984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5078125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.18359375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.01171875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -4136,7 +4136,7 @@
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>7</v>
       </c>
@@ -4156,21 +4156,21 @@
         <v>12</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="2"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="C3" s="24" t="s">
         <v>348</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>349</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>14</v>
@@ -4179,16 +4179,16 @@
         <v>15</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="2"/>
       <c r="J3" s="4"/>
     </row>
-    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>16</v>
       </c>
@@ -4196,25 +4196,25 @@
         <v>17</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="3"/>
       <c r="J4" s="4"/>
     </row>
-    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>20</v>
       </c>
@@ -4228,19 +4228,19 @@
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="2"/>
       <c r="J5" s="4"/>
     </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>25</v>
       </c>
@@ -4257,16 +4257,16 @@
         <v>29</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="3"/>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
@@ -4283,16 +4283,16 @@
         <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="3"/>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>37</v>
       </c>
@@ -4300,30 +4300,30 @@
         <v>41</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="2"/>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>38</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>44</v>
@@ -4332,19 +4332,19 @@
         <v>39</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>40</v>
       </c>
@@ -4355,48 +4355,48 @@
         <v>49</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="2"/>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>43</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="2"/>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>47</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>57</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>50</v>
@@ -4416,13 +4416,13 @@
         <v>46</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="2"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>53</v>
       </c>
@@ -4442,13 +4442,13 @@
         <v>52</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
       <c r="J13" s="4"/>
     </row>
-    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>56</v>
       </c>
@@ -4462,45 +4462,45 @@
         <v>58</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>42</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>59</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>62</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>63</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="3"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>64</v>
       </c>
@@ -4508,25 +4508,25 @@
         <v>69</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>67</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="2"/>
       <c r="J16" s="4"/>
     </row>
-    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>68</v>
       </c>
@@ -4543,16 +4543,16 @@
         <v>71</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="2"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>72</v>
       </c>
@@ -4566,19 +4566,19 @@
         <v>74</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>36</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
       <c r="J18" s="4"/>
     </row>
-    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>75</v>
       </c>
@@ -4592,19 +4592,19 @@
         <v>78</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
       <c r="J19" s="4"/>
     </row>
-    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>79</v>
       </c>
@@ -4618,19 +4618,19 @@
         <v>82</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>83</v>
       </c>
@@ -4644,19 +4644,19 @@
         <v>86</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="3"/>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>87</v>
       </c>
@@ -4670,33 +4670,33 @@
         <v>90</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>30</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="3"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>91</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>94</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="7"/>
@@ -4704,21 +4704,21 @@
       <c r="I23" s="3"/>
       <c r="J23" s="4"/>
     </row>
-    <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>95</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>98</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="9"/>
@@ -4726,7 +4726,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>99</v>
       </c>
@@ -4734,13 +4734,13 @@
         <v>104</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="7"/>
@@ -4748,7 +4748,7 @@
       <c r="I25" s="3"/>
       <c r="J25" s="4"/>
     </row>
-    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>101</v>
       </c>
@@ -4756,13 +4756,13 @@
         <v>107</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>396</v>
+        <v>471</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>102</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4770,7 +4770,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="4"/>
     </row>
-    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>103</v>
       </c>
@@ -4778,13 +4778,13 @@
         <v>110</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>111</v>
+        <v>470</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>105</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4792,21 +4792,21 @@
       <c r="I27" s="3"/>
       <c r="J27" s="4"/>
     </row>
-    <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>106</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" s="15" t="s">
         <v>114</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>115</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>108</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4814,21 +4814,21 @@
       <c r="I28" s="3"/>
       <c r="J28" s="4"/>
     </row>
-    <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>109</v>
       </c>
       <c r="B29" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="C29" s="15" t="s">
-        <v>119</v>
-      </c>
       <c r="D29" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -4836,21 +4836,21 @@
       <c r="I29" s="3"/>
       <c r="J29" s="4"/>
     </row>
-    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C30" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C30" s="15" t="s">
-        <v>123</v>
-      </c>
       <c r="D30" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="7"/>
@@ -4858,21 +4858,21 @@
       <c r="I30" s="3"/>
       <c r="J30" s="4"/>
     </row>
-    <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C31" s="15" t="s">
-        <v>126</v>
-      </c>
       <c r="D31" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="7"/>
@@ -4880,21 +4880,21 @@
       <c r="I31" s="3"/>
       <c r="J31" s="4"/>
     </row>
-    <row r="32" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -4902,21 +4902,21 @@
       <c r="I32" s="3"/>
       <c r="J32" s="4"/>
     </row>
-    <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="C33" s="15" t="s">
-        <v>131</v>
-      </c>
       <c r="D33" s="6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -4924,21 +4924,21 @@
       <c r="I33" s="3"/>
       <c r="J33" s="4"/>
     </row>
-    <row r="34" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A34" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="C34" s="15" t="s">
         <v>346</v>
       </c>
-      <c r="C34" s="15" t="s">
-        <v>347</v>
-      </c>
       <c r="D34" s="6" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="7"/>
@@ -4946,21 +4946,21 @@
       <c r="I34" s="3"/>
       <c r="J34" s="4"/>
     </row>
-    <row r="35" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="7"/>
@@ -4968,15 +4968,15 @@
       <c r="I35" s="3"/>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -4986,15 +4986,15 @@
       <c r="I36" s="3"/>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -5004,15 +5004,15 @@
       <c r="I37" s="3"/>
       <c r="J37" s="4"/>
     </row>
-    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -5022,15 +5022,15 @@
       <c r="I38" s="3"/>
       <c r="J38" s="4"/>
     </row>
-    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -5040,9 +5040,9 @@
       <c r="I39" s="3"/>
       <c r="J39" s="4"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="15"/>
@@ -5054,9 +5054,9 @@
       <c r="I40" s="3"/>
       <c r="J40" s="4"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="15"/>
@@ -5068,9 +5068,9 @@
       <c r="I41" s="3"/>
       <c r="J41" s="4"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="16"/>
@@ -5082,9 +5082,9 @@
       <c r="I42" s="3"/>
       <c r="J42" s="4"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="16"/>
@@ -5096,9 +5096,9 @@
       <c r="I43" s="3"/>
       <c r="J43" s="4"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="16"/>
@@ -5110,9 +5110,9 @@
       <c r="I44" s="3"/>
       <c r="J44" s="4"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="16"/>
@@ -5124,9 +5124,9 @@
       <c r="I45" s="3"/>
       <c r="J45" s="4"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="16"/>
@@ -5138,9 +5138,9 @@
       <c r="I46" s="3"/>
       <c r="J46" s="4"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="16"/>
@@ -5152,9 +5152,9 @@
       <c r="I47" s="3"/>
       <c r="J47" s="4"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="16"/>
@@ -5166,9 +5166,9 @@
       <c r="I48" s="3"/>
       <c r="J48" s="4"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="16"/>
@@ -5180,9 +5180,9 @@
       <c r="I49" s="3"/>
       <c r="J49" s="4"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="16"/>
@@ -5194,9 +5194,9 @@
       <c r="I50" s="3"/>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B51" s="99"/>
       <c r="C51" s="100"/>
@@ -5208,9 +5208,9 @@
       <c r="I51" s="3"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B52" s="99"/>
       <c r="C52" s="100"/>
@@ -5222,9 +5222,9 @@
       <c r="I52" s="3"/>
       <c r="J52" s="4"/>
     </row>
-    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="17"/>
@@ -5245,364 +5245,364 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D195C1D-DB02-1743-BBD2-99104C1FFD33}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="37.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="39.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="40.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.71875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.86328125" customWidth="1"/>
+    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.55859375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.26171875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7890625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="39.546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="34.16796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="40.0859375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="47" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="48" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="C1" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="D1" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="E1" s="50" t="s">
         <v>153</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="F1" s="50" t="s">
         <v>154</v>
       </c>
-      <c r="F1" s="50" t="s">
+      <c r="G1" s="50" t="s">
+        <v>318</v>
+      </c>
+      <c r="H1" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="G1" s="50" t="s">
+      <c r="I1" s="51" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="43" t="s">
+        <v>300</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>376</v>
+      </c>
+      <c r="C2" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>160</v>
+      </c>
+      <c r="G2" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="H2" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="I2" s="46" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="33" t="s">
+        <v>320</v>
+      </c>
+      <c r="B3" s="31" t="s">
         <v>319</v>
       </c>
-      <c r="H1" s="50" t="s">
-        <v>156</v>
-      </c>
-      <c r="I1" s="51" t="s">
+      <c r="C3" s="34" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
-        <v>301</v>
-      </c>
-      <c r="B2" s="44" t="s">
-        <v>377</v>
-      </c>
-      <c r="C2" s="45" t="s">
-        <v>158</v>
-      </c>
-      <c r="D2" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="E2" s="46" t="s">
-        <v>160</v>
-      </c>
-      <c r="F2" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G2" s="46" t="s">
-        <v>162</v>
-      </c>
-      <c r="H2" s="46" t="s">
+      <c r="D3" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="E3" s="38" t="s">
         <v>163</v>
       </c>
-      <c r="I2" s="46" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
-        <v>321</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>320</v>
-      </c>
-      <c r="C3" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D3" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="E3" s="38" t="s">
+      <c r="F3" s="38" t="s">
         <v>164</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="G3" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="G3" s="38" t="s">
+      <c r="H3" s="38" t="s">
+        <v>274</v>
+      </c>
+      <c r="I3" s="38" t="s">
         <v>166</v>
       </c>
-      <c r="H3" s="38" t="s">
-        <v>275</v>
-      </c>
-      <c r="I3" s="38" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="81" x14ac:dyDescent="0.2">
+      <c r="A4" s="33" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="A4" s="33" t="s">
+      <c r="B4" s="32" t="s">
         <v>168</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="C4" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="C4" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D4" s="38" t="s">
+      <c r="E4" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="F4" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="G4" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="F4" s="38" t="s">
-        <v>350</v>
-      </c>
-      <c r="G4" s="38" t="s">
+      <c r="H4" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="I4" s="41"/>
+    </row>
+    <row r="5" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="33" t="s">
         <v>173</v>
       </c>
-      <c r="I4" s="41"/>
-    </row>
-    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="B5" s="31" t="s">
+        <v>280</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="38" t="s">
         <v>174</v>
       </c>
-      <c r="B5" s="31" t="s">
-        <v>281</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D5" s="38" t="s">
+      <c r="E5" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="E5" s="38" t="s">
+      <c r="F5" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="G5" s="38" t="s">
+        <v>316</v>
+      </c>
+      <c r="H5" s="38" t="s">
+        <v>273</v>
+      </c>
+      <c r="I5" s="41"/>
+    </row>
+    <row r="6" spans="1:9" ht="108" x14ac:dyDescent="0.2">
+      <c r="A6" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="G5" s="38" t="s">
+      <c r="B6" s="32" t="s">
+        <v>178</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>180</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="G6" s="38" t="s">
         <v>317</v>
       </c>
-      <c r="H5" s="38" t="s">
-        <v>274</v>
-      </c>
-      <c r="I5" s="41"/>
-    </row>
-    <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
-        <v>178</v>
-      </c>
-      <c r="B6" s="32" t="s">
-        <v>179</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="F6" s="38" t="s">
+      <c r="H6" s="38" t="s">
+        <v>379</v>
+      </c>
+      <c r="I6" s="41"/>
+    </row>
+    <row r="7" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="G6" s="38" t="s">
-        <v>318</v>
-      </c>
-      <c r="H6" s="38" t="s">
-        <v>380</v>
-      </c>
-      <c r="I6" s="41"/>
-    </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
+      <c r="B7" s="32" t="s">
         <v>183</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="C7" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>354</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>278</v>
+      </c>
+      <c r="F7" s="40" t="s">
+        <v>305</v>
+      </c>
+      <c r="G7" s="38" t="s">
         <v>184</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>355</v>
-      </c>
-      <c r="E7" s="38" t="s">
-        <v>279</v>
-      </c>
-      <c r="F7" s="40" t="s">
-        <v>306</v>
-      </c>
-      <c r="G7" s="38" t="s">
-        <v>185</v>
       </c>
       <c r="H7" s="38"/>
       <c r="I7" s="41"/>
     </row>
-    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" s="31" t="s">
         <v>186</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="C8" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="C8" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" s="38" t="s">
+      <c r="E8" s="38" t="s">
+        <v>279</v>
+      </c>
+      <c r="F8" s="38" t="s">
         <v>188</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>280</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>189</v>
       </c>
       <c r="G8" s="38"/>
       <c r="H8" s="38"/>
       <c r="I8" s="41"/>
     </row>
-    <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="B9" s="31" t="s">
         <v>190</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="C9" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="38" t="s">
         <v>191</v>
       </c>
-      <c r="C9" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D9" s="38" t="s">
+      <c r="E9" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="38" t="s">
+      <c r="F9" s="38" t="s">
         <v>193</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>194</v>
       </c>
       <c r="G9" s="38"/>
       <c r="H9" s="38"/>
       <c r="I9" s="41"/>
     </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B10" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>360</v>
+      </c>
+      <c r="E10" s="38" t="s">
         <v>195</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="D10" s="38" t="s">
-        <v>361</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>196</v>
       </c>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
       <c r="H10" s="38"/>
       <c r="I10" s="41"/>
     </row>
-    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D11" s="38"/>
       <c r="E11" s="38" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
       <c r="H11" s="38"/>
       <c r="I11" s="41"/>
     </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="B12" s="31" t="s">
         <v>198</v>
       </c>
-      <c r="B12" s="31" t="s">
-        <v>199</v>
-      </c>
       <c r="C12" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D12" s="38"/>
       <c r="E12" s="38" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F12" s="40"/>
       <c r="G12" s="38"/>
       <c r="H12" s="38"/>
       <c r="I12" s="41"/>
     </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="B13" s="31" t="s">
         <v>201</v>
       </c>
-      <c r="B13" s="31" t="s">
-        <v>202</v>
-      </c>
       <c r="C13" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D13" s="38"/>
       <c r="E13" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F13" s="40"/>
       <c r="G13" s="38"/>
       <c r="H13" s="38"/>
       <c r="I13" s="41"/>
     </row>
-    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" s="31" t="s">
         <v>204</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="C14" s="34" t="s">
         <v>205</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>206</v>
       </c>
       <c r="D14" s="38"/>
       <c r="E14" s="38" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F14" s="40"/>
       <c r="G14" s="38"/>
       <c r="H14" s="38"/>
       <c r="I14" s="41"/>
     </row>
-    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="31" t="s">
         <v>208</v>
       </c>
-      <c r="B15" s="31" t="s">
-        <v>209</v>
-      </c>
       <c r="C15" s="34" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D15" s="38"/>
       <c r="E15" s="38"/>
@@ -5611,15 +5611,15 @@
       <c r="H15" s="38"/>
       <c r="I15" s="41"/>
     </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="31" t="s">
         <v>210</v>
       </c>
-      <c r="B16" s="31" t="s">
-        <v>211</v>
-      </c>
       <c r="C16" s="34" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D16" s="38"/>
       <c r="E16" s="38"/>
@@ -5628,15 +5628,15 @@
       <c r="H16" s="38"/>
       <c r="I16" s="41"/>
     </row>
-    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D17" s="38"/>
       <c r="E17" s="38"/>
@@ -5645,15 +5645,15 @@
       <c r="H17" s="38"/>
       <c r="I17" s="41"/>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="B18" s="31" t="s">
         <v>212</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="C18" s="34" t="s">
         <v>213</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>214</v>
       </c>
       <c r="D18" s="38"/>
       <c r="E18" s="38"/>
@@ -5662,15 +5662,15 @@
       <c r="H18" s="38"/>
       <c r="I18" s="41"/>
     </row>
-    <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="B19" s="31" t="s">
         <v>215</v>
       </c>
-      <c r="B19" s="31" t="s">
-        <v>216</v>
-      </c>
       <c r="C19" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D19" s="38"/>
       <c r="E19" s="38"/>
@@ -5679,15 +5679,15 @@
       <c r="H19" s="38"/>
       <c r="I19" s="41"/>
     </row>
-    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
+        <v>216</v>
+      </c>
+      <c r="B20" s="31" t="s">
         <v>217</v>
       </c>
-      <c r="B20" s="31" t="s">
-        <v>218</v>
-      </c>
       <c r="C20" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D20" s="38"/>
       <c r="E20" s="38"/>
@@ -5696,15 +5696,15 @@
       <c r="H20" s="38"/>
       <c r="I20" s="41"/>
     </row>
-    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="B21" s="31" t="s">
         <v>343</v>
       </c>
-      <c r="B21" s="31" t="s">
-        <v>344</v>
-      </c>
       <c r="C21" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D21" s="38"/>
       <c r="E21" s="38"/>
@@ -5713,15 +5713,15 @@
       <c r="H21" s="38"/>
       <c r="I21" s="41"/>
     </row>
-    <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D22" s="38"/>
       <c r="E22" s="38"/>
@@ -5730,15 +5730,15 @@
       <c r="H22" s="38"/>
       <c r="I22" s="41"/>
     </row>
-    <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C23" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D23" s="38"/>
       <c r="E23" s="38"/>
@@ -5747,15 +5747,15 @@
       <c r="H23" s="38"/>
       <c r="I23" s="41"/>
     </row>
-    <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="35" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B24" s="36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D24" s="38"/>
       <c r="E24" s="38"/>
@@ -5764,15 +5764,15 @@
       <c r="H24" s="38"/>
       <c r="I24" s="41"/>
     </row>
-    <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="35" t="s">
+        <v>362</v>
+      </c>
+      <c r="B25" s="36" t="s">
         <v>363</v>
       </c>
-      <c r="B25" s="36" t="s">
-        <v>364</v>
-      </c>
       <c r="C25" s="37" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D25" s="39"/>
       <c r="E25" s="39"/>
@@ -5790,39 +5790,39 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920DF489-FE6D-4819-BD1A-323DFAE597A3}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="30.66796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="61"/>
       <c r="B1" s="55" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" s="55" t="s">
         <v>222</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="D1" s="54" t="s">
         <v>223</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="E1" s="103" t="s">
         <v>224</v>
       </c>
-      <c r="E1" s="103" t="s">
+      <c r="F1" s="102" t="s">
         <v>225</v>
       </c>
-      <c r="F1" s="102" t="s">
+      <c r="G1" s="55" t="s">
         <v>226</v>
       </c>
-      <c r="G1" s="55" t="s">
+      <c r="I1" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="63" t="s">
         <v>227</v>
-      </c>
-      <c r="I1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="63" t="s">
-        <v>228</v>
       </c>
       <c r="B2" s="64" t="s">
         <v>84</v>
@@ -5840,41 +5840,41 @@
         <v>96</v>
       </c>
       <c r="G2" s="58" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I2" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="63" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B3" s="65" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="57" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E3" s="104" t="s">
         <v>92</v>
       </c>
       <c r="F3" s="53" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="G3" s="57" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I3" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B4" s="57" t="s">
         <v>60</v>
@@ -5895,15 +5895,15 @@
         <v>107</v>
       </c>
       <c r="I4" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="63" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B5" s="62" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C5" s="62" t="s">
         <v>57</v>
@@ -5912,21 +5912,21 @@
         <v>17</v>
       </c>
       <c r="E5" s="105" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F5" s="108" t="s">
         <v>80</v>
       </c>
       <c r="G5" s="106" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="I5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="86" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B6" s="87" t="s">
         <v>98</v>
@@ -5944,202 +5944,202 @@
         <v>58</v>
       </c>
       <c r="G6" s="91" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I6" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="66" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" s="66" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>308</v>
+      </c>
+      <c r="D7" t="s">
+        <v>234</v>
+      </c>
+      <c r="E7" s="63" t="s">
+        <v>235</v>
+      </c>
+      <c r="F7" t="s">
+        <v>236</v>
+      </c>
+      <c r="G7" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="I7" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="84" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="66" t="s">
-        <v>233</v>
-      </c>
-      <c r="B7" s="66" t="s">
-        <v>234</v>
-      </c>
-      <c r="C7" s="63" t="s">
+      <c r="B8" s="84" t="s">
+        <v>224</v>
+      </c>
+      <c r="C8" s="80" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" s="84" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="80" t="s">
+        <v>221</v>
+      </c>
+      <c r="F8" s="84" t="s">
+        <v>222</v>
+      </c>
+      <c r="G8" s="81" t="s">
+        <v>223</v>
+      </c>
+      <c r="I8" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="53" t="s">
+        <v>284</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>225</v>
+      </c>
+      <c r="C9" t="s">
+        <v>223</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="E9" t="s">
+        <v>226</v>
+      </c>
+      <c r="F9" s="53" t="s">
+        <v>221</v>
+      </c>
+      <c r="G9" s="65" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="85" t="s">
+        <v>285</v>
+      </c>
+      <c r="B10" s="85" t="s">
+        <v>223</v>
+      </c>
+      <c r="C10" s="82" t="s">
+        <v>226</v>
+      </c>
+      <c r="D10" s="85" t="s">
+        <v>221</v>
+      </c>
+      <c r="E10" s="82" t="s">
+        <v>225</v>
+      </c>
+      <c r="F10" s="85" t="s">
+        <v>224</v>
+      </c>
+      <c r="G10" s="83" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="D7" t="s">
-        <v>235</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>236</v>
-      </c>
-      <c r="F7" t="s">
-        <v>237</v>
-      </c>
-      <c r="G7" s="63" t="s">
-        <v>157</v>
-      </c>
-      <c r="I7" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="84" t="s">
-        <v>284</v>
-      </c>
-      <c r="B8" s="84" t="s">
-        <v>225</v>
-      </c>
-      <c r="C8" s="80" t="s">
-        <v>226</v>
-      </c>
-      <c r="D8" s="84" t="s">
-        <v>227</v>
-      </c>
-      <c r="E8" s="80" t="s">
-        <v>222</v>
-      </c>
-      <c r="F8" s="84" t="s">
-        <v>223</v>
-      </c>
-      <c r="G8" s="81" t="s">
-        <v>224</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="B13" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="53" t="s">
-        <v>285</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>226</v>
-      </c>
-      <c r="C9" t="s">
-        <v>224</v>
-      </c>
-      <c r="D9" s="53" t="s">
-        <v>223</v>
-      </c>
-      <c r="E9" t="s">
-        <v>227</v>
-      </c>
-      <c r="F9" s="53" t="s">
-        <v>222</v>
-      </c>
-      <c r="G9" s="65" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="85" t="s">
-        <v>286</v>
-      </c>
-      <c r="B10" s="85" t="s">
-        <v>224</v>
-      </c>
-      <c r="C10" s="82" t="s">
-        <v>227</v>
-      </c>
-      <c r="D10" s="85" t="s">
-        <v>222</v>
-      </c>
-      <c r="E10" s="82" t="s">
-        <v>226</v>
-      </c>
-      <c r="F10" s="85" t="s">
-        <v>225</v>
-      </c>
-      <c r="G10" s="83" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>289</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>445</v>
-      </c>
       <c r="G15" s="2" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -6148,105 +6148,105 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="I18" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I19" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>290</v>
-      </c>
       <c r="E20" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D21" t="s">
+        <v>402</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D21" t="s">
-        <v>404</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>290</v>
-      </c>
       <c r="G21" s="2" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="D23" s="2"/>
@@ -6254,98 +6254,98 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I24" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="I25" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E26" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I26" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>300</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>301</v>
       </c>
       <c r="G27" s="2"/>
       <c r="I27" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -6354,10 +6354,10 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="I28" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -6366,10 +6366,10 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="I29" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -6378,7 +6378,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -6386,7 +6386,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -6394,7 +6394,7 @@
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -6402,7 +6402,7 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -6410,7 +6410,7 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -6418,7 +6418,7 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -6426,7 +6426,7 @@
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -6434,7 +6434,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -6442,7 +6442,7 @@
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -6450,7 +6450,7 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -6458,7 +6458,7 @@
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -6466,7 +6466,7 @@
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -6474,7 +6474,7 @@
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -6482,7 +6482,7 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -6490,7 +6490,7 @@
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48" s="3"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -6498,7 +6498,7 @@
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -6512,15 +6512,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4430D7D8-35BC-4E32-9DE8-E2E435ADAAA0}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="36" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="37.5" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="6" width="30.7109375" style="26" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="26"/>
+    <col min="1" max="6" width="30.66796875" style="26" customWidth="1"/>
+    <col min="7" max="16384" width="9.14453125" style="26"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" s="127" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B1" s="128"/>
       <c r="C1" s="128"/>
@@ -6530,22 +6530,22 @@
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="123" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B2" s="123" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C2" s="123" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="D2" s="123" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="E2" s="123" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="F2" s="123" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
@@ -6573,16 +6573,16 @@
         <v>25</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F4" s="117">
         <v>6</v>
@@ -6593,16 +6593,16 @@
         <v>24</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D5" s="111" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F5" s="117">
         <v>7</v>
@@ -6613,16 +6613,16 @@
         <v>23</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F6" s="120">
         <v>8</v>
@@ -6633,16 +6633,16 @@
         <v>22</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F7" s="117">
         <v>9</v>
@@ -6653,10 +6653,10 @@
         <v>21</v>
       </c>
       <c r="B8" s="98" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" s="124" t="s">
         <v>238</v>
-      </c>
-      <c r="C8" s="124" t="s">
-        <v>239</v>
       </c>
       <c r="D8" s="125"/>
       <c r="E8" s="126"/>
@@ -6669,16 +6669,16 @@
         <v>20</v>
       </c>
       <c r="B9" s="109" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E9" s="110" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F9" s="117">
         <v>11</v>
@@ -6689,16 +6689,16 @@
         <v>19</v>
       </c>
       <c r="B10" s="112" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C10" s="113" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D10" s="114" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E10" s="113" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F10" s="120">
         <v>12</v>
@@ -6738,66 +6738,66 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CEB427C-0CB4-4E8D-8367-36F6DD891282}">
   <dimension ref="A1:CA6"/>
-  <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="19.7734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" style="53"/>
-    <col min="2" max="2" width="19.7109375" style="65"/>
-    <col min="4" max="4" width="19.7109375" style="53"/>
-    <col min="6" max="6" width="19.7109375" style="53"/>
-    <col min="8" max="8" width="19.7109375" style="53"/>
-    <col min="10" max="10" width="19.7109375" style="53"/>
-    <col min="12" max="12" width="19.7109375" style="53"/>
-    <col min="14" max="14" width="19.7109375" style="53"/>
-    <col min="16" max="16" width="19.7109375" style="53"/>
-    <col min="18" max="18" width="19.7109375" style="53"/>
-    <col min="20" max="20" width="19.7109375" style="53"/>
-    <col min="22" max="22" width="19.7109375" style="53"/>
-    <col min="24" max="24" width="19.7109375" style="53"/>
-    <col min="26" max="26" width="19.7109375" style="53"/>
-    <col min="28" max="28" width="19.7109375" style="53"/>
-    <col min="30" max="30" width="19.7109375" style="71"/>
-    <col min="31" max="32" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.7109375" customWidth="1"/>
-    <col min="42" max="42" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="19.7109375" style="71" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.7109375" style="53" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="19.7109375" style="71" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="19.7109375" style="53"/>
-    <col min="63" max="63" width="19.7109375" style="53"/>
-    <col min="65" max="65" width="19.7109375" style="53"/>
-    <col min="67" max="67" width="19.7109375" style="53"/>
-    <col min="69" max="70" width="19.7109375" style="53"/>
-    <col min="71" max="71" width="19.7109375" style="65"/>
-    <col min="73" max="73" width="19.7109375" style="53"/>
-    <col min="75" max="75" width="19.7109375" style="53"/>
-    <col min="77" max="77" width="19.7109375" style="53"/>
-    <col min="79" max="79" width="19.7109375" style="53"/>
+    <col min="1" max="1" width="19.7734375" style="53"/>
+    <col min="2" max="2" width="19.7734375" style="65"/>
+    <col min="4" max="4" width="19.7734375" style="53"/>
+    <col min="6" max="6" width="19.7734375" style="53"/>
+    <col min="8" max="8" width="19.7734375" style="53"/>
+    <col min="10" max="10" width="19.7734375" style="53"/>
+    <col min="12" max="12" width="19.7734375" style="53"/>
+    <col min="14" max="14" width="19.7734375" style="53"/>
+    <col min="16" max="16" width="19.7734375" style="53"/>
+    <col min="18" max="18" width="19.7734375" style="53"/>
+    <col min="20" max="20" width="19.7734375" style="53"/>
+    <col min="22" max="22" width="19.7734375" style="53"/>
+    <col min="24" max="24" width="19.7734375" style="53"/>
+    <col min="26" max="26" width="19.7734375" style="53"/>
+    <col min="28" max="28" width="19.7734375" style="53"/>
+    <col min="30" max="30" width="19.7734375" style="71"/>
+    <col min="31" max="32" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.7734375" customWidth="1"/>
+    <col min="42" max="42" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="19.7734375" style="71" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.7734375" style="53" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="19.7734375" style="71" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="19.7734375" style="53"/>
+    <col min="63" max="63" width="19.7734375" style="53"/>
+    <col min="65" max="65" width="19.7734375" style="53"/>
+    <col min="67" max="67" width="19.7734375" style="53"/>
+    <col min="69" max="70" width="19.7734375" style="53"/>
+    <col min="71" max="71" width="19.7734375" style="65"/>
+    <col min="73" max="73" width="19.7734375" style="53"/>
+    <col min="75" max="75" width="19.7734375" style="53"/>
+    <col min="77" max="77" width="19.7734375" style="53"/>
+    <col min="79" max="79" width="19.7734375" style="53"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="67" t="str">
         <f>Cards!B2</f>
         <v>Fillibuster</v>
@@ -7084,7 +7084,7 @@
       <c r="BY1" s="67"/>
       <c r="CA1" s="67"/>
     </row>
-    <row r="2" spans="1:79" s="92" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:79" s="92" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="93" t="str">
         <f>Cards!C2</f>
         <v>Move the deliberated Law $L6 additional places back in the queue during Postpone</v>
@@ -7191,11 +7191,11 @@
       </c>
       <c r="AA2" s="92" t="str">
         <f>Cards!C26</f>
-        <v>Subtract $L3 from Scheme Guard rolls. An unmodified 6 always succeeds.</v>
+        <v>Subtract $L3 from Scheme Evasion rolls. An unmodified 6 always succeeds.</v>
       </c>
       <c r="AB2" s="93" t="str">
         <f>Cards!C27</f>
-        <v>Subtract $L3 from Scheme Card rolls</v>
+        <v>Subtract $L3 from Scheme Damage rolls</v>
       </c>
       <c r="AC2" s="92" t="str">
         <f>Cards!C28</f>
@@ -7351,11 +7351,11 @@
       </c>
       <c r="BO2" s="93" t="str">
         <f t="shared" si="2"/>
-        <v>Subtract $L3 from Scheme Guard rolls. An unmodified 6 always succeeds.</v>
+        <v>Subtract $L3 from Scheme Evasion rolls. An unmodified 6 always succeeds.</v>
       </c>
       <c r="BP2" s="92" t="str">
         <f t="shared" si="2"/>
-        <v>Subtract $L3 from Scheme Card rolls</v>
+        <v>Subtract $L3 from Scheme Damage rolls</v>
       </c>
       <c r="BQ2" s="72" t="str">
         <f t="shared" si="2"/>
@@ -7371,7 +7371,7 @@
       <c r="BY2" s="93"/>
       <c r="CA2" s="93"/>
     </row>
-    <row r="3" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:79" s="69" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="67" t="str">
         <f>Cards!D2</f>
         <v>Full Coffers</v>
@@ -7655,7 +7655,7 @@
       <c r="BY3" s="67"/>
       <c r="CA3" s="67"/>
     </row>
-    <row r="4" spans="1:79" s="74" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:79" s="74" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="72" t="str">
         <f>Cards!E2</f>
         <v>The Royal Bank must have at least $L6 Coins or all Players suffer sanctions on Undermarket Actions</v>
@@ -7939,7 +7939,7 @@
       <c r="BY4" s="72"/>
       <c r="CA4" s="72"/>
     </row>
-    <row r="5" spans="1:79" s="78" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:79" s="78" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="76" t="str">
         <f>Cards!F2</f>
         <v>Fickle Mercenaries</v>
@@ -8219,7 +8219,7 @@
       <c r="BY5" s="76"/>
       <c r="CA5" s="76"/>
     </row>
-    <row r="6" spans="1:79" s="74" customFormat="1" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:79" s="74" customFormat="1" ht="81.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="72" t="str">
         <f>Cards!G2</f>
         <v>Give $2D6 Troops to $R</v>
@@ -8508,295 +8508,295 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BDA35E-BFC3-134A-A064-89D65A8B31CF}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.50390625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.22265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1" t="s">
         <v>260</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>261</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>262</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>263</v>
       </c>
-      <c r="F1" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B2">
         <f>30*2</f>
         <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D2">
         <v>27.7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B3">
         <f>34*2</f>
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D3">
         <v>27.7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B4">
         <f>18*3</f>
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D4">
         <v>30.75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B5">
         <f>2*6+6*6</f>
         <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B6">
         <f>1*6+10*6</f>
         <v>66</v>
       </c>
       <c r="C6" t="s">
+        <v>265</v>
+      </c>
+      <c r="E6" t="s">
         <v>266</v>
       </c>
-      <c r="E6" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B7">
         <f>10*6+10</f>
         <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B8">
         <f>2*8*6</f>
         <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E8" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B9">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B10">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C10" t="s">
+        <v>265</v>
+      </c>
+      <c r="E10" t="s">
         <v>266</v>
       </c>
-      <c r="E10" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B11">
         <f>(30*6-B10)/5</f>
         <v>30</v>
       </c>
       <c r="C11" t="s">
+        <v>265</v>
+      </c>
+      <c r="E11" t="s">
         <v>266</v>
       </c>
-      <c r="E11" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B12">
         <f>5*6</f>
         <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E12" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B13">
         <f>(15*6-B12)/5</f>
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E13" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B18">
         <f>10*6</f>
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B19">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B20">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -8808,89 +8808,89 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC83F89-2724-CA43-A519-59213A612B31}">
   <dimension ref="A1:U55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24" style="95" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" style="97" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" style="97" bestFit="1" customWidth="1"/>
-    <col min="12" max="19" width="11.85546875" style="97" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" style="97" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.9453125" style="95" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.72265625" customWidth="1"/>
+    <col min="4" max="4" width="8.33984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.27734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5078125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.97265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.43359375" style="97" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.22265625" style="97" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.43359375" style="97" bestFit="1" customWidth="1"/>
+    <col min="12" max="19" width="11.8359375" style="97" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.9140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.5078125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B1" t="s">
         <v>324</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>325</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>326</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>327</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>353</v>
+      </c>
+      <c r="G1" t="s">
+        <v>352</v>
+      </c>
+      <c r="H1" t="s">
         <v>328</v>
       </c>
-      <c r="F1" t="s">
-        <v>354</v>
-      </c>
-      <c r="G1" t="s">
-        <v>353</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>329</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="97" t="s">
+        <v>350</v>
+      </c>
+      <c r="K1" t="s">
         <v>330</v>
       </c>
-      <c r="J1" s="97" t="s">
+      <c r="L1" t="s">
+        <v>331</v>
+      </c>
+      <c r="M1" t="s">
+        <v>332</v>
+      </c>
+      <c r="N1" t="s">
+        <v>333</v>
+      </c>
+      <c r="O1" t="s">
+        <v>334</v>
+      </c>
+      <c r="P1" t="s">
+        <v>335</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>336</v>
+      </c>
+      <c r="R1" t="s">
+        <v>337</v>
+      </c>
+      <c r="S1" t="s">
+        <v>338</v>
+      </c>
+      <c r="T1" t="s">
+        <v>339</v>
+      </c>
+      <c r="U1" t="s">
         <v>351</v>
       </c>
-      <c r="K1" t="s">
-        <v>331</v>
-      </c>
-      <c r="L1" t="s">
-        <v>332</v>
-      </c>
-      <c r="M1" t="s">
-        <v>333</v>
-      </c>
-      <c r="N1" t="s">
-        <v>334</v>
-      </c>
-      <c r="O1" t="s">
-        <v>335</v>
-      </c>
-      <c r="P1" t="s">
-        <v>336</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>337</v>
-      </c>
-      <c r="R1" t="s">
-        <v>338</v>
-      </c>
-      <c r="S1" t="s">
-        <v>339</v>
-      </c>
-      <c r="T1" t="s">
-        <v>340</v>
-      </c>
-      <c r="U1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="95">
         <v>46075</v>
       </c>
@@ -8934,7 +8934,7 @@
         <v>0.92638888888888893</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="95">
         <v>46089</v>
       </c>
@@ -8990,7 +8990,7 @@
         <v>0.86527777777777781</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="95">
         <v>46105</v>
       </c>
@@ -9043,7 +9043,7 @@
         <v>0.92777777777777781</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="95">
         <v>46118</v>
       </c>
@@ -9096,7 +9096,7 @@
         <v>0.9194444444444444</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="95">
         <v>46124</v>
       </c>
@@ -9140,7 +9140,7 @@
         <v>0.74583333333333335</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="95">
         <v>46131</v>
       </c>
@@ -9193,7 +9193,7 @@
         <v>0.70277777777777772</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="95">
         <v>46138</v>
       </c>
@@ -9237,7 +9237,7 @@
         <v>0.69513888888888886</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="95">
         <v>46145</v>
       </c>
@@ -9290,7 +9290,7 @@
         <v>0.71666666666666667</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="95">
         <v>46152</v>
       </c>
@@ -9340,7 +9340,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="95">
         <v>46158</v>
       </c>
@@ -9393,7 +9393,7 @@
         <v>0.99236111111111114</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C12" s="96" t="b">
         <v>0</v>
       </c>
@@ -9401,7 +9401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C13" s="96" t="b">
         <v>0</v>
       </c>
@@ -9409,7 +9409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C14" s="96" t="b">
         <v>0</v>
       </c>
@@ -9417,7 +9417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C15" s="96" t="b">
         <v>0</v>
       </c>
@@ -9425,7 +9425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C16" s="96" t="b">
         <v>0</v>
       </c>
@@ -9433,7 +9433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C17" s="96" t="b">
         <v>0</v>
       </c>
@@ -9441,7 +9441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C18" s="96" t="b">
         <v>0</v>
       </c>
@@ -9449,7 +9449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C19" s="96" t="b">
         <v>0</v>
       </c>
@@ -9457,7 +9457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C20" s="96" t="b">
         <v>0</v>
       </c>
@@ -9465,7 +9465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C21" s="96" t="b">
         <v>0</v>
       </c>
@@ -9473,7 +9473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C22" s="96" t="b">
         <v>0</v>
       </c>
@@ -9481,7 +9481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C23" s="96" t="b">
         <v>0</v>
       </c>
@@ -9489,7 +9489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C24" s="96" t="b">
         <v>0</v>
       </c>
@@ -9497,7 +9497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C25" s="96" t="b">
         <v>0</v>
       </c>
@@ -9505,7 +9505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C26" s="96" t="b">
         <v>0</v>
       </c>
@@ -9513,7 +9513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C27" s="96" t="b">
         <v>0</v>
       </c>
@@ -9521,7 +9521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C28" s="96" t="b">
         <v>0</v>
       </c>
@@ -9529,7 +9529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C29" s="96" t="b">
         <v>0</v>
       </c>
@@ -9537,7 +9537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C30" s="96" t="b">
         <v>0</v>
       </c>
@@ -9545,7 +9545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C31" s="96" t="b">
         <v>0</v>
       </c>
@@ -9553,7 +9553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C32" s="96" t="b">
         <v>0</v>
       </c>
@@ -9561,7 +9561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C33" s="96" t="b">
         <v>0</v>
       </c>
@@ -9569,7 +9569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C34" s="96" t="b">
         <v>0</v>
       </c>
@@ -9577,7 +9577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C35" s="96" t="b">
         <v>0</v>
       </c>
@@ -9585,7 +9585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C36" s="96" t="b">
         <v>0</v>
       </c>
@@ -9593,7 +9593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C37" s="96" t="b">
         <v>0</v>
       </c>
@@ -9601,7 +9601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C38" s="96" t="b">
         <v>0</v>
       </c>
@@ -9609,7 +9609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C39" s="96" t="b">
         <v>0</v>
       </c>
@@ -9617,7 +9617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C40" s="96" t="b">
         <v>0</v>
       </c>
@@ -9625,7 +9625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C41" s="96" t="b">
         <v>0</v>
       </c>
@@ -9633,7 +9633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C42" s="96" t="b">
         <v>0</v>
       </c>
@@ -9641,7 +9641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C43" s="96" t="b">
         <v>0</v>
       </c>
@@ -9649,7 +9649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C44" s="96" t="b">
         <v>0</v>
       </c>
@@ -9657,7 +9657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C45" s="96" t="b">
         <v>0</v>
       </c>
@@ -9665,7 +9665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C46" s="96" t="b">
         <v>0</v>
       </c>
@@ -9673,7 +9673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C47" s="96" t="b">
         <v>0</v>
       </c>
@@ -9681,7 +9681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C48" s="96" t="b">
         <v>0</v>
       </c>
@@ -9689,7 +9689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C49" s="96" t="b">
         <v>0</v>
       </c>
@@ -9697,7 +9697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C50" s="96" t="b">
         <v>0</v>
       </c>
@@ -9705,7 +9705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C51" s="96" t="b">
         <v>0</v>
       </c>
@@ -9713,7 +9713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C52" s="96" t="b">
         <v>0</v>
       </c>
@@ -9721,7 +9721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C53" s="96" t="b">
         <v>0</v>
       </c>
@@ -9729,7 +9729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C54" s="96" t="b">
         <v>0</v>
       </c>
@@ -9737,7 +9737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C55" s="96" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added some playtesting sessions
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4363" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B5A9EBE-F8CB-C648-82A1-9886ADB36BD6}"/>
+  <xr:revisionPtr revIDLastSave="4419" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A93B122E-B6FD-BD44-88EB-0C51F1B2CD6B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="472">
   <si>
     <t>Standard Card</t>
   </si>
@@ -131,9 +131,6 @@
     <t>Stable Economies</t>
   </si>
   <si>
-    <t>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Promote &amp; Commission</t>
-  </si>
-  <si>
     <t>Blackmail</t>
   </si>
   <si>
@@ -149,9 +146,6 @@
     <t>Unreasonable Distractions</t>
   </si>
   <si>
-    <t>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Promote &amp; Commission</t>
-  </si>
-  <si>
     <t>Invalid Paperwork</t>
   </si>
   <si>
@@ -335,9 +329,6 @@
     <t>War Machines</t>
   </si>
   <si>
-    <t>Purchase and immediately add up to $L3 Troops to your force when deploying them</t>
-  </si>
-  <si>
     <t>Police Force</t>
   </si>
   <si>
@@ -839,9 +830,6 @@
     <t>Card</t>
   </si>
   <si>
-    <t>Punchboard</t>
-  </si>
-  <si>
     <t>Wood</t>
   </si>
   <si>
@@ -854,9 +842,6 @@
     <t>Plastic</t>
   </si>
   <si>
-    <t>Mini</t>
-  </si>
-  <si>
     <t>Scheme Envelopes</t>
   </si>
   <si>
@@ -1173,9 +1158,6 @@
   </si>
   <si>
     <t>Send Troops up to Leader's Level to the Battlefield and gain half Troops in Coins</t>
-  </si>
-  <si>
-    <t>You may repeat Undermarket Actions at double the penalty</t>
   </si>
   <si>
     <t>Painful Progress</t>
@@ -1459,6 +1441,24 @@
   </si>
   <si>
     <t>Subtract $L3 from Scheme Evasion rolls. An unmodified 6 always succeeds.</t>
+  </si>
+  <si>
+    <t>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Commission</t>
+  </si>
+  <si>
+    <t>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Commission</t>
+  </si>
+  <si>
+    <t>You may pay 7 - $L6 Commodities to repeat Undermarket Actions</t>
+  </si>
+  <si>
+    <t>After deploying, purchase and immediately deploy up to $L3 Troops, but no more than your deployed Troops.</t>
+  </si>
+  <si>
+    <t>Plastic Magnet</t>
+  </si>
+  <si>
+    <t>Plastic Mini</t>
   </si>
 </sst>
 </file>
@@ -4156,7 +4156,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="2"/>
@@ -4167,10 +4167,10 @@
         <v>13</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>14</v>
@@ -4179,10 +4179,10 @@
         <v>15</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="2"/>
@@ -4196,19 +4196,19 @@
         <v>17</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="3"/>
@@ -4228,13 +4228,13 @@
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="2"/>
@@ -4254,13 +4254,13 @@
         <v>28</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>29</v>
+        <v>466</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="3"/>
@@ -4268,25 +4268,25 @@
     </row>
     <row r="7" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>34</v>
-      </c>
       <c r="E7" s="18" t="s">
-        <v>35</v>
+        <v>467</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="3"/>
@@ -4294,25 +4294,25 @@
     </row>
     <row r="8" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="2"/>
@@ -4320,25 +4320,25 @@
     </row>
     <row r="9" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
@@ -4346,25 +4346,25 @@
     </row>
     <row r="10" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="2"/>
@@ -4372,25 +4372,25 @@
     </row>
     <row r="11" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>424</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>430</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>45</v>
-      </c>
       <c r="E11" s="15" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="2"/>
@@ -4398,25 +4398,25 @@
     </row>
     <row r="12" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="2"/>
@@ -4424,25 +4424,25 @@
     </row>
     <row r="13" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>55</v>
-      </c>
       <c r="F13" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
@@ -4450,25 +4450,25 @@
     </row>
     <row r="14" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>58</v>
-      </c>
       <c r="E14" s="15" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
@@ -4476,25 +4476,25 @@
     </row>
     <row r="15" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="3"/>
@@ -4502,25 +4502,25 @@
     </row>
     <row r="16" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="2"/>
@@ -4528,25 +4528,25 @@
     </row>
     <row r="17" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="E17" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="2"/>
@@ -4554,25 +4554,25 @@
     </row>
     <row r="18" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="E18" s="15" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="2"/>
@@ -4580,25 +4580,25 @@
     </row>
     <row r="19" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="2"/>
@@ -4606,25 +4606,25 @@
     </row>
     <row r="20" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3"/>
@@ -4632,25 +4632,25 @@
     </row>
     <row r="21" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="3"/>
@@ -4658,25 +4658,25 @@
     </row>
     <row r="22" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>97</v>
+        <v>469</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="3"/>
@@ -4684,19 +4684,19 @@
     </row>
     <row r="23" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="7"/>
@@ -4706,19 +4706,19 @@
     </row>
     <row r="24" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>423</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>429</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="E24" s="15" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="9"/>
@@ -4728,19 +4728,19 @@
     </row>
     <row r="25" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="7"/>
@@ -4750,19 +4750,19 @@
     </row>
     <row r="26" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7"/>
@@ -4772,19 +4772,19 @@
     </row>
     <row r="27" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7"/>
@@ -4794,19 +4794,19 @@
     </row>
     <row r="28" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7"/>
@@ -4816,19 +4816,19 @@
     </row>
     <row r="29" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="7"/>
@@ -4838,19 +4838,19 @@
     </row>
     <row r="30" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>115</v>
-      </c>
       <c r="E30" s="15" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="7"/>
@@ -4860,19 +4860,19 @@
     </row>
     <row r="31" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>119</v>
-      </c>
       <c r="E31" s="15" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="7"/>
@@ -4882,19 +4882,19 @@
     </row>
     <row r="32" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="7"/>
@@ -4904,19 +4904,19 @@
     </row>
     <row r="33" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="7"/>
@@ -4926,19 +4926,19 @@
     </row>
     <row r="34" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A34" s="11" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="7"/>
@@ -4948,19 +4948,19 @@
     </row>
     <row r="35" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="7"/>
@@ -4970,13 +4970,13 @@
     </row>
     <row r="36" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="16"/>
@@ -4988,13 +4988,13 @@
     </row>
     <row r="37" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="16"/>
@@ -5006,13 +5006,13 @@
     </row>
     <row r="38" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>377</v>
+        <v>468</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="16"/>
@@ -5024,13 +5024,13 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="16"/>
@@ -5042,7 +5042,7 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="15"/>
@@ -5056,7 +5056,7 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="15"/>
@@ -5070,7 +5070,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="16"/>
@@ -5084,7 +5084,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="16"/>
@@ -5098,7 +5098,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="16"/>
@@ -5112,7 +5112,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="16"/>
@@ -5126,7 +5126,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="16"/>
@@ -5140,7 +5140,7 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="16"/>
@@ -5154,7 +5154,7 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="16"/>
@@ -5168,7 +5168,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="16"/>
@@ -5182,7 +5182,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="16"/>
@@ -5196,7 +5196,7 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B51" s="99"/>
       <c r="C51" s="100"/>
@@ -5210,7 +5210,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B52" s="99"/>
       <c r="C52" s="100"/>
@@ -5224,7 +5224,7 @@
     </row>
     <row r="53" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="17"/>
@@ -5260,215 +5260,215 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="49" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" s="50" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="E1" s="50" t="s">
         <v>150</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="F1" s="50" t="s">
         <v>151</v>
       </c>
-      <c r="D1" s="50" t="s">
+      <c r="G1" s="50" t="s">
+        <v>313</v>
+      </c>
+      <c r="H1" s="50" t="s">
         <v>152</v>
       </c>
-      <c r="E1" s="50" t="s">
+      <c r="I1" s="51" t="s">
         <v>153</v>
-      </c>
-      <c r="F1" s="50" t="s">
-        <v>154</v>
-      </c>
-      <c r="G1" s="50" t="s">
-        <v>318</v>
-      </c>
-      <c r="H1" s="50" t="s">
-        <v>155</v>
-      </c>
-      <c r="I1" s="51" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A2" s="43" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C2" s="45" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="46" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="G2" s="46" t="s">
         <v>158</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="H2" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="F2" s="46" t="s">
-        <v>160</v>
-      </c>
-      <c r="G2" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="H2" s="46" t="s">
-        <v>162</v>
-      </c>
       <c r="I2" s="46" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A3" s="33" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D3" s="38" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="E3" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="H3" s="38" t="s">
+        <v>269</v>
+      </c>
+      <c r="I3" s="38" t="s">
         <v>163</v>
-      </c>
-      <c r="F3" s="38" t="s">
-        <v>164</v>
-      </c>
-      <c r="G3" s="38" t="s">
-        <v>165</v>
-      </c>
-      <c r="H3" s="38" t="s">
-        <v>274</v>
-      </c>
-      <c r="I3" s="38" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="81" x14ac:dyDescent="0.2">
       <c r="A4" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="38" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="F4" s="38" t="s">
+        <v>344</v>
+      </c>
+      <c r="G4" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="C4" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="38" t="s">
+      <c r="H4" s="38" t="s">
         <v>169</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="F4" s="38" t="s">
-        <v>349</v>
-      </c>
-      <c r="G4" s="38" t="s">
-        <v>171</v>
-      </c>
-      <c r="H4" s="38" t="s">
-        <v>172</v>
       </c>
       <c r="I4" s="41"/>
     </row>
     <row r="5" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>275</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>172</v>
+      </c>
+      <c r="F5" s="38" t="s">
         <v>173</v>
       </c>
-      <c r="B5" s="31" t="s">
-        <v>280</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="F5" s="38" t="s">
-        <v>176</v>
-      </c>
       <c r="G5" s="38" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="H5" s="38" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="I5" s="41"/>
     </row>
     <row r="6" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A6" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="F6" s="38" t="s">
         <v>178</v>
       </c>
-      <c r="C6" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="F6" s="38" t="s">
-        <v>181</v>
-      </c>
       <c r="G6" s="38" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="I6" s="41"/>
     </row>
     <row r="7" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="F7" s="40" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="H7" s="38"/>
       <c r="I7" s="41"/>
     </row>
     <row r="8" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A8" s="33" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>274</v>
+      </c>
+      <c r="F8" s="38" t="s">
         <v>185</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" s="38" t="s">
-        <v>187</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>279</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>188</v>
       </c>
       <c r="G8" s="38"/>
       <c r="H8" s="38"/>
@@ -5476,22 +5476,22 @@
     </row>
     <row r="9" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A9" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="E9" s="38" t="s">
         <v>189</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="F9" s="38" t="s">
         <v>190</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="D9" s="38" t="s">
-        <v>191</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>192</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>193</v>
       </c>
       <c r="G9" s="38"/>
       <c r="H9" s="38"/>
@@ -5499,19 +5499,19 @@
     </row>
     <row r="10" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A10" s="33" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
@@ -5520,17 +5520,17 @@
     </row>
     <row r="11" spans="1:9" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A11" s="33" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D11" s="38"/>
       <c r="E11" s="38" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
@@ -5539,17 +5539,17 @@
     </row>
     <row r="12" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A12" s="33" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D12" s="38"/>
       <c r="E12" s="38" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F12" s="40"/>
       <c r="G12" s="38"/>
@@ -5558,17 +5558,17 @@
     </row>
     <row r="13" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A13" s="33" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D13" s="38"/>
       <c r="E13" s="38" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F13" s="40"/>
       <c r="G13" s="38"/>
@@ -5577,17 +5577,17 @@
     </row>
     <row r="14" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A14" s="33" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D14" s="38"/>
       <c r="E14" s="38" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F14" s="40"/>
       <c r="G14" s="38"/>
@@ -5596,13 +5596,13 @@
     </row>
     <row r="15" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C15" s="34" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D15" s="38"/>
       <c r="E15" s="38"/>
@@ -5613,13 +5613,13 @@
     </row>
     <row r="16" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D16" s="38"/>
       <c r="E16" s="38"/>
@@ -5630,13 +5630,13 @@
     </row>
     <row r="17" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D17" s="38"/>
       <c r="E17" s="38"/>
@@ -5647,13 +5647,13 @@
     </row>
     <row r="18" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="33" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D18" s="38"/>
       <c r="E18" s="38"/>
@@ -5664,13 +5664,13 @@
     </row>
     <row r="19" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C19" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D19" s="38"/>
       <c r="E19" s="38"/>
@@ -5681,13 +5681,13 @@
     </row>
     <row r="20" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D20" s="38"/>
       <c r="E20" s="38"/>
@@ -5698,13 +5698,13 @@
     </row>
     <row r="21" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="33" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C21" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D21" s="38"/>
       <c r="E21" s="38"/>
@@ -5715,13 +5715,13 @@
     </row>
     <row r="22" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D22" s="38"/>
       <c r="E22" s="38"/>
@@ -5732,13 +5732,13 @@
     </row>
     <row r="23" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C23" s="34" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D23" s="38"/>
       <c r="E23" s="38"/>
@@ -5749,13 +5749,13 @@
     </row>
     <row r="24" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="35" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B24" s="36" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D24" s="38"/>
       <c r="E24" s="38"/>
@@ -5766,13 +5766,13 @@
     </row>
     <row r="25" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="35" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B25" s="36" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="C25" s="37" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D25" s="39"/>
       <c r="E25" s="39"/>
@@ -5799,344 +5799,344 @@
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="61"/>
       <c r="B1" s="55" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" s="55" t="s">
+        <v>219</v>
+      </c>
+      <c r="D1" s="54" t="s">
+        <v>220</v>
+      </c>
+      <c r="E1" s="103" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="F1" s="102" t="s">
         <v>222</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="G1" s="55" t="s">
         <v>223</v>
       </c>
-      <c r="E1" s="103" t="s">
-        <v>224</v>
-      </c>
-      <c r="F1" s="102" t="s">
-        <v>225</v>
-      </c>
-      <c r="G1" s="55" t="s">
-        <v>226</v>
-      </c>
       <c r="I1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="63" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D2" s="59" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E2" s="101" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F2" s="107" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G2" s="58" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I2" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="63" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C3" s="57" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="E3" s="104" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F3" s="53" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="G3" s="57" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C4" s="57" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="56" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E4" s="104" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F4" s="56" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="G4" s="57" t="s">
-        <v>107</v>
-      </c>
       <c r="I4" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="63" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B5" s="62" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C5" s="62" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D5" s="60" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="105" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="F5" s="108" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G5" s="106" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="I5" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="86" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B6" s="87" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C6" s="88" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D6" s="89" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E6" s="90" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F6" s="82" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G6" s="91" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I6" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="66" t="s">
+        <v>229</v>
+      </c>
+      <c r="B7" s="66" t="s">
+        <v>230</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>303</v>
+      </c>
+      <c r="D7" t="s">
+        <v>231</v>
+      </c>
+      <c r="E7" s="63" t="s">
         <v>232</v>
       </c>
-      <c r="B7" s="66" t="s">
+      <c r="F7" t="s">
         <v>233</v>
       </c>
-      <c r="C7" s="63" t="s">
-        <v>308</v>
-      </c>
-      <c r="D7" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>235</v>
-      </c>
-      <c r="F7" t="s">
-        <v>236</v>
-      </c>
       <c r="G7" s="63" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="I7" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="84" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B8" s="84" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C8" s="80" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D8" s="84" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E8" s="80" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="F8" s="84" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G8" s="81" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I8" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="53" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C9" t="s">
+        <v>220</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="E9" t="s">
         <v>223</v>
       </c>
-      <c r="D9" s="53" t="s">
-        <v>222</v>
-      </c>
-      <c r="E9" t="s">
-        <v>226</v>
-      </c>
       <c r="F9" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="G9" s="65" t="s">
         <v>221</v>
-      </c>
-      <c r="G9" s="65" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="85" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B10" s="85" t="s">
+        <v>220</v>
+      </c>
+      <c r="C10" s="82" t="s">
         <v>223</v>
       </c>
-      <c r="C10" s="82" t="s">
-        <v>226</v>
-      </c>
       <c r="D10" s="85" t="s">
+        <v>218</v>
+      </c>
+      <c r="E10" s="82" t="s">
+        <v>222</v>
+      </c>
+      <c r="F10" s="85" t="s">
         <v>221</v>
       </c>
-      <c r="E10" s="82" t="s">
-        <v>225</v>
-      </c>
-      <c r="F10" s="85" t="s">
-        <v>224</v>
-      </c>
       <c r="G10" s="83" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -6150,99 +6150,99 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="I18" t="s">
         <v>397</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="I18" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I19" t="s">
         <v>288</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="I19" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="E20" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="D21" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="G22" s="2"/>
     </row>
@@ -6256,93 +6256,93 @@
     </row>
     <row r="24" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="I24" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="I25" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E26" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="I26" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="G27" s="2"/>
       <c r="I27" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
@@ -6354,7 +6354,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="I28" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
@@ -6366,7 +6366,7 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="I29" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
@@ -6520,7 +6520,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" s="127" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B1" s="128"/>
       <c r="C1" s="128"/>
@@ -6530,22 +6530,22 @@
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="123" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="B2" s="123" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="C2" s="123" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="D2" s="123" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="E2" s="123" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="F2" s="123" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
@@ -6573,16 +6573,16 @@
         <v>25</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="F4" s="117">
         <v>6</v>
@@ -6593,16 +6593,16 @@
         <v>24</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D5" s="111" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F5" s="117">
         <v>7</v>
@@ -6613,16 +6613,16 @@
         <v>23</v>
       </c>
       <c r="B6" s="28" t="s">
+        <v>194</v>
+      </c>
+      <c r="C6" s="28" t="s">
         <v>197</v>
       </c>
-      <c r="C6" s="28" t="s">
-        <v>200</v>
-      </c>
       <c r="D6" s="29" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F6" s="120">
         <v>8</v>
@@ -6633,16 +6633,16 @@
         <v>22</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="F7" s="117">
         <v>9</v>
@@ -6653,10 +6653,10 @@
         <v>21</v>
       </c>
       <c r="B8" s="98" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C8" s="124" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D8" s="125"/>
       <c r="E8" s="126"/>
@@ -6669,16 +6669,16 @@
         <v>20</v>
       </c>
       <c r="B9" s="109" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E9" s="110" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="F9" s="117">
         <v>11</v>
@@ -6689,16 +6689,16 @@
         <v>19</v>
       </c>
       <c r="B10" s="112" t="s">
+        <v>208</v>
+      </c>
+      <c r="C10" s="113" t="s">
         <v>211</v>
       </c>
-      <c r="C10" s="113" t="s">
-        <v>214</v>
-      </c>
       <c r="D10" s="114" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="E10" s="113" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F10" s="120">
         <v>12</v>
@@ -7175,7 +7175,7 @@
       </c>
       <c r="W2" s="92" t="str">
         <f>Cards!C22</f>
-        <v>Purchase and immediately add up to $L3 Troops to your force when deploying them</v>
+        <v>After deploying, purchase and immediately deploy up to $L3 Troops, but no more than your deployed Troops.</v>
       </c>
       <c r="X2" s="93" t="str">
         <f>Cards!C23</f>
@@ -7239,7 +7239,7 @@
       </c>
       <c r="AM2" s="92" t="str">
         <f>Cards!C38</f>
-        <v>You may repeat Undermarket Actions at double the penalty</v>
+        <v>You may pay 7 - $L6 Commodities to repeat Undermarket Actions</v>
       </c>
       <c r="AN2" s="93" t="str">
         <f>Cards!C39</f>
@@ -7335,7 +7335,7 @@
       </c>
       <c r="BK2" s="93" t="str">
         <f t="shared" si="2"/>
-        <v>Purchase and immediately add up to $L3 Troops to your force when deploying them</v>
+        <v>After deploying, purchase and immediately deploy up to $L3 Troops, but no more than your deployed Troops.</v>
       </c>
       <c r="BL2" s="92" t="str">
         <f t="shared" si="2"/>
@@ -7674,11 +7674,11 @@
       </c>
       <c r="E4" s="74" t="str">
         <f>Cards!E6</f>
-        <v>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Promote &amp; Commission</v>
+        <v>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Commission</v>
       </c>
       <c r="F4" s="72" t="str">
         <f>Cards!E7</f>
-        <v>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Promote &amp; Commission</v>
+        <v>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Commission</v>
       </c>
       <c r="G4" s="74" t="str">
         <f>Cards!E8</f>
@@ -7802,11 +7802,11 @@
       </c>
       <c r="AK4" s="74" t="str">
         <f t="shared" si="5"/>
-        <v>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Promote &amp; Commission</v>
+        <v>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Commission</v>
       </c>
       <c r="AL4" s="72" t="str">
         <f t="shared" si="5"/>
-        <v>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Promote &amp; Commission</v>
+        <v>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Commission</v>
       </c>
       <c r="AM4" s="74" t="str">
         <f t="shared" si="5"/>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="BQ4" s="93" t="str">
         <f t="shared" si="4"/>
-        <v>You may repeat Undermarket Actions at double the penalty</v>
+        <v>You may pay 7 - $L6 Commodities to repeat Undermarket Actions</v>
       </c>
       <c r="BR4" s="72" t="str">
         <f t="shared" si="4"/>
@@ -8519,31 +8519,31 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E1" t="s">
         <v>259</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>260</v>
-      </c>
-      <c r="D1" t="s">
-        <v>261</v>
-      </c>
-      <c r="E1" t="s">
-        <v>262</v>
-      </c>
-      <c r="F1" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B2">
         <f>30*2</f>
         <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D2">
         <v>27.7</v>
@@ -8551,14 +8551,14 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B3">
         <f>34*2</f>
         <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D3">
         <v>27.7</v>
@@ -8566,14 +8566,14 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B4">
         <f>18*3</f>
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D4">
         <v>30.75</v>
@@ -8581,19 +8581,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="B5">
         <f>2*6+6*6</f>
         <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>267</v>
+        <v>470</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B6">
         <f>1*6+10*6</f>
@@ -8603,12 +8603,12 @@
         <v>265</v>
       </c>
       <c r="E6" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B7">
         <f>10*6+10</f>
@@ -8618,12 +8618,12 @@
         <v>265</v>
       </c>
       <c r="E7" t="s">
-        <v>270</v>
+        <v>471</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B8">
         <f>2*8*6</f>
@@ -8633,12 +8633,12 @@
         <v>265</v>
       </c>
       <c r="E8" t="s">
-        <v>270</v>
+        <v>471</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B9">
         <f>5*6</f>
@@ -8647,10 +8647,13 @@
       <c r="C9" t="s">
         <v>265</v>
       </c>
+      <c r="E9" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B10">
         <f>5*6</f>
@@ -8660,12 +8663,12 @@
         <v>265</v>
       </c>
       <c r="E10" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B11">
         <f>(30*6-B10)/5</f>
@@ -8675,12 +8678,12 @@
         <v>265</v>
       </c>
       <c r="E11" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B12">
         <f>5*6</f>
@@ -8690,12 +8693,12 @@
         <v>265</v>
       </c>
       <c r="E12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B13">
         <f>(15*6-B12)/5</f>
@@ -8705,98 +8708,98 @@
         <v>265</v>
       </c>
       <c r="E13" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B18">
         <f>10*6</f>
         <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B19">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B20">
         <f>5*7</f>
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -8827,67 +8830,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C1" t="s">
+        <v>320</v>
+      </c>
+      <c r="D1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E1" t="s">
+        <v>322</v>
+      </c>
+      <c r="F1" t="s">
+        <v>348</v>
+      </c>
+      <c r="G1" t="s">
+        <v>347</v>
+      </c>
+      <c r="H1" t="s">
         <v>323</v>
       </c>
-      <c r="B1" t="s">
+      <c r="I1" t="s">
         <v>324</v>
       </c>
-      <c r="C1" t="s">
+      <c r="J1" s="97" t="s">
+        <v>345</v>
+      </c>
+      <c r="K1" t="s">
         <v>325</v>
       </c>
-      <c r="D1" t="s">
+      <c r="L1" t="s">
         <v>326</v>
       </c>
-      <c r="E1" t="s">
+      <c r="M1" t="s">
         <v>327</v>
       </c>
-      <c r="F1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G1" t="s">
-        <v>352</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="N1" t="s">
         <v>328</v>
       </c>
-      <c r="I1" t="s">
+      <c r="O1" t="s">
         <v>329</v>
       </c>
-      <c r="J1" s="97" t="s">
-        <v>350</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>330</v>
       </c>
-      <c r="L1" t="s">
+      <c r="Q1" t="s">
         <v>331</v>
       </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>332</v>
       </c>
-      <c r="N1" t="s">
+      <c r="S1" t="s">
         <v>333</v>
       </c>
-      <c r="O1" t="s">
+      <c r="T1" t="s">
         <v>334</v>
       </c>
-      <c r="P1" t="s">
-        <v>335</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>336</v>
-      </c>
-      <c r="R1" t="s">
-        <v>337</v>
-      </c>
-      <c r="S1" t="s">
-        <v>338</v>
-      </c>
-      <c r="T1" t="s">
-        <v>339</v>
-      </c>
       <c r="U1" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -9394,19 +9397,115 @@
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A12" s="95">
+        <v>46215</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
       <c r="C12" s="96" t="b">
         <v>0</v>
       </c>
       <c r="D12" s="96" t="b">
         <v>0</v>
       </c>
+      <c r="E12">
+        <v>16</v>
+      </c>
+      <c r="F12">
+        <v>22</v>
+      </c>
+      <c r="G12">
+        <v>16</v>
+      </c>
+      <c r="H12" s="97">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="I12" s="97">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="J12" s="97">
+        <v>0.57638888888888884</v>
+      </c>
+      <c r="K12" s="97">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="L12" s="97">
+        <v>0.59583333333333333</v>
+      </c>
+      <c r="M12" s="97">
+        <v>0.625</v>
+      </c>
+      <c r="N12" s="97">
+        <v>0.6381944444444444</v>
+      </c>
+      <c r="O12" s="97">
+        <v>0.66041666666666665</v>
+      </c>
+      <c r="P12" s="97">
+        <v>0.68402777777777779</v>
+      </c>
+      <c r="Q12" s="97">
+        <v>0.70694444444444449</v>
+      </c>
+      <c r="R12" s="97">
+        <v>0.73402777777777772</v>
+      </c>
+      <c r="U12" s="97">
+        <v>0.73888888888888893</v>
+      </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A13" s="95">
+        <v>46247</v>
+      </c>
+      <c r="B13">
+        <v>6</v>
+      </c>
       <c r="C13" s="96" t="b">
         <v>0</v>
       </c>
       <c r="D13" s="96" t="b">
         <v>0</v>
+      </c>
+      <c r="E13">
+        <v>12</v>
+      </c>
+      <c r="F13">
+        <v>21</v>
+      </c>
+      <c r="G13">
+        <v>7</v>
+      </c>
+      <c r="H13" s="97">
+        <v>0.79097222222222219</v>
+      </c>
+      <c r="I13" s="97">
+        <v>0.9458333333333333</v>
+      </c>
+      <c r="J13" s="97">
+        <v>0.8</v>
+      </c>
+      <c r="K13" s="97">
+        <v>0.81041666666666667</v>
+      </c>
+      <c r="L13" s="97">
+        <v>0.82777777777777772</v>
+      </c>
+      <c r="M13" s="97">
+        <v>0.84722222222222221</v>
+      </c>
+      <c r="N13" s="97">
+        <v>0.87569444444444444</v>
+      </c>
+      <c r="O13" s="97">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="P13" s="97">
+        <v>0.93541666666666667</v>
+      </c>
+      <c r="U13" s="97">
+        <v>0.9458333333333333</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Revised training manuals after some game changes
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4608" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EF046A5-0414-4BBC-B770-C49B65FEC21C}"/>
+  <xr:revisionPtr revIDLastSave="4609" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C967B3DB-A4F0-420C-86C3-EA5A38C1350B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2312,24 +2312,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2357,6 +2339,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3333,10 +3333,6 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3658,897 +3654,897 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" style="107" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" style="107" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" style="107" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.140625" style="107" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39" style="107" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="107"/>
+    <col min="1" max="1" width="24.6171875" style="101" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.58984375" style="101" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.50390625" style="101" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5390625" style="101" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.58984375" style="101" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" style="101" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.58984375" style="101" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.046875" style="101" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.58984375" style="101" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5078125" style="101" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.18359375" style="101" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.01171875" style="101" customWidth="1"/>
+    <col min="13" max="16384" width="9.14453125" style="101"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="106" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="100" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="100" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="106" t="s">
+      <c r="C1" s="100" t="s">
         <v>338</v>
       </c>
-      <c r="D1" s="106" t="s">
+      <c r="D1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="106" t="s">
+      <c r="E1" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="106" t="s">
+      <c r="F1" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="106" t="s">
+      <c r="G1" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="106"/>
-      <c r="I1" s="106"/>
-      <c r="J1" s="106"/>
-    </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="108" t="s">
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+    </row>
+    <row r="2" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A2" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="103" t="s">
         <v>340</v>
       </c>
-      <c r="C2" s="109">
+      <c r="C2" s="103">
         <v>6</v>
       </c>
-      <c r="D2" s="108" t="s">
+      <c r="D2" s="102" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="109" t="s">
+      <c r="E2" s="103" t="s">
         <v>377</v>
       </c>
-      <c r="F2" s="108" t="s">
+      <c r="F2" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="109" t="s">
+      <c r="G2" s="103" t="s">
         <v>408</v>
       </c>
-      <c r="H2" s="110"/>
-      <c r="I2" s="111"/>
-      <c r="J2" s="110"/>
-    </row>
-    <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="108" t="s">
+      <c r="H2" s="104"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="104"/>
+    </row>
+    <row r="3" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="102" t="s">
         <v>260</v>
       </c>
-      <c r="B3" s="109" t="s">
+      <c r="B3" s="103" t="s">
         <v>339</v>
       </c>
-      <c r="C3" s="109">
+      <c r="C3" s="103">
         <v>6</v>
       </c>
-      <c r="D3" s="108" t="s">
+      <c r="D3" s="102" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="109" t="s">
+      <c r="E3" s="103" t="s">
         <v>378</v>
       </c>
-      <c r="F3" s="108" t="s">
+      <c r="F3" s="102" t="s">
         <v>313</v>
       </c>
-      <c r="G3" s="109" t="s">
+      <c r="G3" s="103" t="s">
         <v>409</v>
       </c>
-      <c r="H3" s="110"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="110"/>
-    </row>
-    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="108" t="s">
+      <c r="H3" s="104"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="104"/>
+    </row>
+    <row r="4" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="109" t="s">
+      <c r="B4" s="103" t="s">
         <v>342</v>
       </c>
-      <c r="C4" s="109">
+      <c r="C4" s="103">
         <v>6</v>
       </c>
-      <c r="D4" s="108" t="s">
+      <c r="D4" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="109" t="s">
+      <c r="E4" s="103" t="s">
         <v>379</v>
       </c>
-      <c r="F4" s="108" t="s">
+      <c r="F4" s="102" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="109" t="s">
+      <c r="G4" s="103" t="s">
         <v>410</v>
       </c>
-      <c r="H4" s="110"/>
-      <c r="I4" s="112"/>
-      <c r="J4" s="110"/>
-    </row>
-    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="113" t="s">
+      <c r="H4" s="104"/>
+      <c r="I4" s="106"/>
+      <c r="J4" s="104"/>
+    </row>
+    <row r="5" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="109" t="s">
+      <c r="B5" s="103" t="s">
         <v>341</v>
       </c>
-      <c r="C5" s="109">
+      <c r="C5" s="103">
         <v>3</v>
       </c>
-      <c r="D5" s="108" t="s">
+      <c r="D5" s="102" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="109" t="s">
+      <c r="E5" s="103" t="s">
         <v>379</v>
       </c>
-      <c r="F5" s="108" t="s">
+      <c r="F5" s="102" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="109" t="s">
+      <c r="G5" s="103" t="s">
         <v>418</v>
       </c>
-      <c r="H5" s="110"/>
-      <c r="I5" s="111"/>
-      <c r="J5" s="110"/>
-    </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="108" t="s">
+      <c r="H5" s="104"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="104"/>
+    </row>
+    <row r="6" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A6" s="102" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="109" t="s">
+      <c r="B6" s="103" t="s">
         <v>343</v>
       </c>
-      <c r="C6" s="109">
+      <c r="C6" s="103">
         <v>3</v>
       </c>
-      <c r="D6" s="108" t="s">
+      <c r="D6" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="109" t="s">
+      <c r="E6" s="103" t="s">
         <v>380</v>
       </c>
-      <c r="F6" s="108" t="s">
+      <c r="F6" s="102" t="s">
         <v>310</v>
       </c>
-      <c r="G6" s="109" t="s">
+      <c r="G6" s="103" t="s">
         <v>411</v>
       </c>
-      <c r="H6" s="110"/>
-      <c r="I6" s="112"/>
-      <c r="J6" s="110"/>
-    </row>
-    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="108" t="s">
+      <c r="H6" s="104"/>
+      <c r="I6" s="106"/>
+      <c r="J6" s="104"/>
+    </row>
+    <row r="7" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="102" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="109" t="s">
+      <c r="B7" s="103" t="s">
         <v>344</v>
       </c>
-      <c r="C7" s="109">
+      <c r="C7" s="103">
         <v>3</v>
       </c>
-      <c r="D7" s="108" t="s">
+      <c r="D7" s="102" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="114" t="s">
+      <c r="E7" s="108" t="s">
         <v>381</v>
       </c>
-      <c r="F7" s="108" t="s">
+      <c r="F7" s="102" t="s">
         <v>302</v>
       </c>
-      <c r="G7" s="109" t="s">
+      <c r="G7" s="103" t="s">
         <v>303</v>
       </c>
-      <c r="H7" s="110"/>
-      <c r="I7" s="112"/>
-      <c r="J7" s="110"/>
-    </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="108" t="s">
+      <c r="H7" s="104"/>
+      <c r="I7" s="106"/>
+      <c r="J7" s="104"/>
+    </row>
+    <row r="8" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="102" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="109" t="s">
+      <c r="B8" s="103" t="s">
         <v>351</v>
       </c>
-      <c r="C8" s="109">
+      <c r="C8" s="103">
         <v>6</v>
       </c>
-      <c r="D8" s="108" t="s">
+      <c r="D8" s="102" t="s">
         <v>232</v>
       </c>
-      <c r="E8" s="109" t="s">
+      <c r="E8" s="103" t="s">
         <v>379</v>
       </c>
-      <c r="F8" s="108" t="s">
+      <c r="F8" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="G8" s="115" t="s">
+      <c r="G8" s="109" t="s">
         <v>305</v>
       </c>
-      <c r="H8" s="110"/>
-      <c r="I8" s="111"/>
-      <c r="J8" s="110"/>
-    </row>
-    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="108" t="s">
+      <c r="H8" s="104"/>
+      <c r="I8" s="105"/>
+      <c r="J8" s="104"/>
+    </row>
+    <row r="9" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="102" t="s">
         <v>316</v>
       </c>
-      <c r="B9" s="109" t="s">
+      <c r="B9" s="103" t="s">
         <v>350</v>
       </c>
-      <c r="C9" s="109">
+      <c r="C9" s="103">
         <v>6</v>
       </c>
-      <c r="D9" s="108" t="s">
+      <c r="D9" s="102" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="109" t="s">
+      <c r="E9" s="103" t="s">
         <v>379</v>
       </c>
-      <c r="F9" s="108" t="s">
+      <c r="F9" s="102" t="s">
         <v>306</v>
       </c>
-      <c r="G9" s="109" t="s">
+      <c r="G9" s="103" t="s">
         <v>307</v>
       </c>
-      <c r="H9" s="110"/>
-      <c r="I9" s="112"/>
-      <c r="J9" s="110"/>
-    </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="108" t="s">
+      <c r="H9" s="104"/>
+      <c r="I9" s="106"/>
+      <c r="J9" s="104"/>
+    </row>
+    <row r="10" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="102" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="109" t="s">
+      <c r="B10" s="103" t="s">
         <v>345</v>
       </c>
-      <c r="C10" s="109">
+      <c r="C10" s="103">
         <v>3</v>
       </c>
-      <c r="D10" s="108" t="s">
+      <c r="D10" s="102" t="s">
         <v>315</v>
       </c>
-      <c r="E10" s="109" t="s">
+      <c r="E10" s="103" t="s">
         <v>382</v>
       </c>
-      <c r="F10" s="108" t="s">
+      <c r="F10" s="102" t="s">
         <v>308</v>
       </c>
-      <c r="G10" s="109" t="s">
+      <c r="G10" s="103" t="s">
         <v>309</v>
       </c>
-      <c r="H10" s="110"/>
-      <c r="I10" s="111"/>
-      <c r="J10" s="110"/>
-    </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="108" t="s">
+      <c r="H10" s="104"/>
+      <c r="I10" s="105"/>
+      <c r="J10" s="104"/>
+    </row>
+    <row r="11" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A11" s="102" t="s">
         <v>267</v>
       </c>
-      <c r="B11" s="109" t="s">
+      <c r="B11" s="103" t="s">
         <v>346</v>
       </c>
-      <c r="C11" s="109">
+      <c r="C11" s="103">
         <v>3</v>
       </c>
-      <c r="D11" s="108" t="s">
+      <c r="D11" s="102" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="109" t="s">
+      <c r="E11" s="103" t="s">
         <v>383</v>
       </c>
-      <c r="F11" s="108" t="s">
+      <c r="F11" s="102" t="s">
         <v>312</v>
       </c>
-      <c r="G11" s="109" t="s">
+      <c r="G11" s="103" t="s">
         <v>311</v>
       </c>
-      <c r="H11" s="110"/>
-      <c r="I11" s="111"/>
-      <c r="J11" s="110"/>
-    </row>
-    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="108" t="s">
+      <c r="H11" s="104"/>
+      <c r="I11" s="105"/>
+      <c r="J11" s="104"/>
+    </row>
+    <row r="12" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="109" t="s">
+      <c r="B12" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="C12" s="109">
+      <c r="C12" s="103">
         <v>3</v>
       </c>
-      <c r="D12" s="108" t="s">
+      <c r="D12" s="102" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="109" t="s">
+      <c r="E12" s="103" t="s">
         <v>384</v>
       </c>
-      <c r="F12" s="108" t="s">
+      <c r="F12" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="109" t="s">
+      <c r="G12" s="103" t="s">
         <v>419</v>
       </c>
-      <c r="H12" s="110"/>
-      <c r="I12" s="111"/>
-      <c r="J12" s="110"/>
-    </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="108" t="s">
+      <c r="H12" s="104"/>
+      <c r="I12" s="105"/>
+      <c r="J12" s="104"/>
+    </row>
+    <row r="13" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="102" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="109" t="s">
+      <c r="B13" s="103" t="s">
         <v>348</v>
       </c>
-      <c r="C13" s="109">
+      <c r="C13" s="103">
         <v>6</v>
       </c>
-      <c r="D13" s="108" t="s">
+      <c r="D13" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="109" t="s">
+      <c r="E13" s="103" t="s">
         <v>385</v>
       </c>
-      <c r="F13" s="108" t="s">
+      <c r="F13" s="102" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="109" t="s">
+      <c r="G13" s="103" t="s">
         <v>412</v>
       </c>
-      <c r="H13" s="110"/>
-      <c r="I13" s="111"/>
-      <c r="J13" s="110"/>
-    </row>
-    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="108" t="s">
+      <c r="H13" s="104"/>
+      <c r="I13" s="105"/>
+      <c r="J13" s="104"/>
+    </row>
+    <row r="14" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A14" s="102" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="109" t="s">
+      <c r="B14" s="103" t="s">
         <v>349</v>
       </c>
-      <c r="C14" s="109">
+      <c r="C14" s="103">
         <v>3</v>
       </c>
-      <c r="D14" s="108" t="s">
+      <c r="D14" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="109" t="s">
+      <c r="E14" s="103" t="s">
         <v>386</v>
       </c>
-      <c r="F14" s="108" t="s">
+      <c r="F14" s="102" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="109" t="s">
+      <c r="G14" s="103" t="s">
         <v>412</v>
       </c>
-      <c r="H14" s="110"/>
-      <c r="I14" s="112"/>
-      <c r="J14" s="110"/>
-    </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="108" t="s">
+      <c r="H14" s="104"/>
+      <c r="I14" s="106"/>
+      <c r="J14" s="104"/>
+    </row>
+    <row r="15" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A15" s="102" t="s">
         <v>333</v>
       </c>
-      <c r="B15" s="109" t="s">
+      <c r="B15" s="103" t="s">
         <v>352</v>
       </c>
-      <c r="C15" s="109">
+      <c r="C15" s="103">
         <v>6</v>
       </c>
-      <c r="D15" s="108" t="s">
+      <c r="D15" s="102" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="109" t="s">
+      <c r="E15" s="103" t="s">
         <v>387</v>
       </c>
-      <c r="F15" s="108" t="s">
+      <c r="F15" s="102" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="109" t="s">
+      <c r="G15" s="103" t="s">
         <v>413</v>
       </c>
-      <c r="H15" s="110"/>
-      <c r="I15" s="112"/>
-      <c r="J15" s="110"/>
-    </row>
-    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A16" s="108" t="s">
+      <c r="H15" s="104"/>
+      <c r="I15" s="106"/>
+      <c r="J15" s="104"/>
+    </row>
+    <row r="16" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A16" s="102" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="109" t="s">
+      <c r="B16" s="103" t="s">
         <v>353</v>
       </c>
-      <c r="C16" s="109">
+      <c r="C16" s="103">
         <v>3</v>
       </c>
-      <c r="D16" s="108" t="s">
+      <c r="D16" s="102" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="109" t="s">
+      <c r="E16" s="103" t="s">
         <v>388</v>
       </c>
-      <c r="F16" s="108" t="s">
+      <c r="F16" s="102" t="s">
         <v>301</v>
       </c>
-      <c r="G16" s="109" t="s">
+      <c r="G16" s="103" t="s">
         <v>414</v>
       </c>
-      <c r="H16" s="110"/>
-      <c r="I16" s="111"/>
-      <c r="J16" s="110"/>
-    </row>
-    <row r="17" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="108" t="s">
+      <c r="H16" s="104"/>
+      <c r="I16" s="105"/>
+      <c r="J16" s="104"/>
+    </row>
+    <row r="17" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="102" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="109" t="s">
+      <c r="B17" s="103" t="s">
         <v>354</v>
       </c>
-      <c r="C17" s="109">
+      <c r="C17" s="103">
         <v>3</v>
       </c>
-      <c r="D17" s="108" t="s">
+      <c r="D17" s="102" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="109" t="s">
+      <c r="E17" s="103" t="s">
         <v>389</v>
       </c>
-      <c r="F17" s="108" t="s">
+      <c r="F17" s="102" t="s">
         <v>284</v>
       </c>
-      <c r="G17" s="109" t="s">
+      <c r="G17" s="103" t="s">
         <v>414</v>
       </c>
-      <c r="H17" s="110"/>
-      <c r="I17" s="111"/>
-      <c r="J17" s="110"/>
-    </row>
-    <row r="18" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="108" t="s">
+      <c r="H17" s="104"/>
+      <c r="I17" s="105"/>
+      <c r="J17" s="104"/>
+    </row>
+    <row r="18" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A18" s="102" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="109" t="s">
+      <c r="B18" s="103" t="s">
         <v>355</v>
       </c>
-      <c r="C18" s="109">
+      <c r="C18" s="103">
         <v>3</v>
       </c>
-      <c r="D18" s="108" t="s">
+      <c r="D18" s="102" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="109" t="s">
+      <c r="E18" s="103" t="s">
         <v>390</v>
       </c>
-      <c r="F18" s="108" t="s">
+      <c r="F18" s="102" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="109" t="s">
+      <c r="G18" s="103" t="s">
         <v>283</v>
       </c>
-      <c r="H18" s="110"/>
-      <c r="I18" s="111"/>
-      <c r="J18" s="110"/>
-    </row>
-    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" s="108" t="s">
+      <c r="H18" s="104"/>
+      <c r="I18" s="105"/>
+      <c r="J18" s="104"/>
+    </row>
+    <row r="19" spans="1:10" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="102" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="109" t="s">
+      <c r="B19" s="103" t="s">
         <v>356</v>
       </c>
-      <c r="C19" s="109">
+      <c r="C19" s="103">
         <v>3</v>
       </c>
-      <c r="D19" s="108" t="s">
+      <c r="D19" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="109" t="s">
+      <c r="E19" s="103" t="s">
         <v>391</v>
       </c>
-      <c r="F19" s="108" t="s">
+      <c r="F19" s="102" t="s">
         <v>278</v>
       </c>
-      <c r="G19" s="109" t="s">
+      <c r="G19" s="103" t="s">
         <v>415</v>
       </c>
-      <c r="H19" s="110"/>
-      <c r="I19" s="111"/>
-      <c r="J19" s="110"/>
-    </row>
-    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="108" t="s">
+      <c r="H19" s="104"/>
+      <c r="I19" s="105"/>
+      <c r="J19" s="104"/>
+    </row>
+    <row r="20" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="102" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="109" t="s">
+      <c r="B20" s="103" t="s">
         <v>357</v>
       </c>
-      <c r="C20" s="109">
+      <c r="C20" s="103">
         <v>3</v>
       </c>
-      <c r="D20" s="108" t="s">
+      <c r="D20" s="102" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="109" t="s">
+      <c r="E20" s="103" t="s">
         <v>392</v>
       </c>
-      <c r="F20" s="108" t="s">
+      <c r="F20" s="102" t="s">
         <v>279</v>
       </c>
-      <c r="G20" s="109" t="s">
+      <c r="G20" s="103" t="s">
         <v>416</v>
       </c>
-      <c r="H20" s="110"/>
-      <c r="I20" s="112"/>
-      <c r="J20" s="110"/>
-    </row>
-    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="108" t="s">
+      <c r="H20" s="104"/>
+      <c r="I20" s="106"/>
+      <c r="J20" s="104"/>
+    </row>
+    <row r="21" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="102" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="109" t="s">
+      <c r="B21" s="103" t="s">
         <v>358</v>
       </c>
-      <c r="C21" s="109">
+      <c r="C21" s="103">
         <v>3</v>
       </c>
-      <c r="D21" s="108" t="s">
+      <c r="D21" s="102" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="109" t="s">
+      <c r="E21" s="103" t="s">
         <v>393</v>
       </c>
-      <c r="F21" s="108" t="s">
+      <c r="F21" s="102" t="s">
         <v>285</v>
       </c>
-      <c r="G21" s="109" t="s">
+      <c r="G21" s="103" t="s">
         <v>415</v>
       </c>
-      <c r="H21" s="110"/>
-      <c r="I21" s="112"/>
-      <c r="J21" s="110"/>
-    </row>
-    <row r="22" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A22" s="108" t="s">
+      <c r="H21" s="104"/>
+      <c r="I21" s="106"/>
+      <c r="J21" s="104"/>
+    </row>
+    <row r="22" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A22" s="102" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="109" t="s">
+      <c r="B22" s="103" t="s">
         <v>359</v>
       </c>
-      <c r="C22" s="109">
+      <c r="C22" s="103">
         <v>3</v>
       </c>
-      <c r="D22" s="108" t="s">
+      <c r="D22" s="102" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="109" t="s">
+      <c r="E22" s="103" t="s">
         <v>394</v>
       </c>
-      <c r="F22" s="108" t="s">
+      <c r="F22" s="102" t="s">
         <v>18</v>
       </c>
-      <c r="G22" s="109" t="s">
+      <c r="G22" s="103" t="s">
         <v>417</v>
       </c>
-      <c r="H22" s="110"/>
-      <c r="I22" s="112"/>
-      <c r="J22" s="110"/>
-    </row>
-    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="108" t="s">
+      <c r="H22" s="104"/>
+      <c r="I22" s="106"/>
+      <c r="J22" s="104"/>
+    </row>
+    <row r="23" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="102" t="s">
         <v>317</v>
       </c>
-      <c r="B23" s="109" t="s">
+      <c r="B23" s="103" t="s">
         <v>360</v>
       </c>
-      <c r="C23" s="109">
+      <c r="C23" s="103">
         <v>3</v>
       </c>
-      <c r="D23" s="108" t="s">
+      <c r="D23" s="102" t="s">
         <v>51</v>
       </c>
-      <c r="E23" s="109" t="s">
+      <c r="E23" s="103" t="s">
         <v>395</v>
       </c>
-      <c r="F23" s="110"/>
-      <c r="G23" s="112"/>
-    </row>
-    <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="108" t="s">
+      <c r="F23" s="104"/>
+      <c r="G23" s="106"/>
+    </row>
+    <row r="24" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A24" s="102" t="s">
         <v>332</v>
       </c>
-      <c r="B24" s="109" t="s">
+      <c r="B24" s="103" t="s">
         <v>361</v>
       </c>
-      <c r="C24" s="109">
+      <c r="C24" s="103">
         <v>6</v>
       </c>
-      <c r="D24" s="108" t="s">
+      <c r="D24" s="102" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="109" t="s">
+      <c r="E24" s="103" t="s">
         <v>396</v>
       </c>
-      <c r="F24" s="110"/>
-      <c r="G24" s="112"/>
-    </row>
-    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="108" t="s">
+      <c r="F24" s="104"/>
+      <c r="G24" s="106"/>
+    </row>
+    <row r="25" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="102" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="109" t="s">
+      <c r="B25" s="103" t="s">
         <v>362</v>
       </c>
-      <c r="C25" s="109">
+      <c r="C25" s="103">
         <v>6</v>
       </c>
-      <c r="D25" s="108" t="s">
+      <c r="D25" s="102" t="s">
         <v>54</v>
       </c>
-      <c r="E25" s="109" t="s">
+      <c r="E25" s="103" t="s">
         <v>397</v>
       </c>
-      <c r="F25" s="110"/>
-      <c r="G25" s="112"/>
-    </row>
-    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="108" t="s">
+      <c r="F25" s="104"/>
+      <c r="G25" s="106"/>
+    </row>
+    <row r="26" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A26" s="102" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="109" t="s">
+      <c r="B26" s="103" t="s">
         <v>363</v>
       </c>
-      <c r="C26" s="109">
+      <c r="C26" s="103">
         <v>3</v>
       </c>
-      <c r="D26" s="108" t="s">
+      <c r="D26" s="102" t="s">
         <v>55</v>
       </c>
-      <c r="E26" s="109" t="s">
+      <c r="E26" s="103" t="s">
         <v>398</v>
       </c>
-      <c r="F26" s="110"/>
-      <c r="G26" s="112"/>
-    </row>
-    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="108" t="s">
+      <c r="F26" s="104"/>
+      <c r="G26" s="106"/>
+    </row>
+    <row r="27" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A27" s="102" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="109" t="s">
+      <c r="B27" s="103" t="s">
         <v>364</v>
       </c>
-      <c r="C27" s="115">
+      <c r="C27" s="109">
         <v>3</v>
       </c>
-      <c r="D27" s="108" t="s">
+      <c r="D27" s="102" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="109" t="s">
+      <c r="E27" s="103" t="s">
         <v>399</v>
       </c>
-      <c r="F27" s="110"/>
-      <c r="G27" s="112"/>
-    </row>
-    <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A28" s="108" t="s">
+      <c r="F27" s="104"/>
+      <c r="G27" s="106"/>
+    </row>
+    <row r="28" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="102" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="109" t="s">
+      <c r="B28" s="103" t="s">
         <v>365</v>
       </c>
-      <c r="C28" s="109">
+      <c r="C28" s="103">
         <v>3</v>
       </c>
-      <c r="D28" s="108" t="s">
+      <c r="D28" s="102" t="s">
         <v>59</v>
       </c>
-      <c r="E28" s="109" t="s">
+      <c r="E28" s="103" t="s">
         <v>400</v>
       </c>
-      <c r="F28" s="110"/>
-      <c r="G28" s="112"/>
-    </row>
-    <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A29" s="108" t="s">
+      <c r="F28" s="104"/>
+      <c r="G28" s="106"/>
+    </row>
+    <row r="29" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A29" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="109" t="s">
+      <c r="B29" s="103" t="s">
         <v>366</v>
       </c>
-      <c r="C29" s="109">
+      <c r="C29" s="103">
         <v>3</v>
       </c>
-      <c r="D29" s="108" t="s">
+      <c r="D29" s="102" t="s">
         <v>61</v>
       </c>
-      <c r="E29" s="109" t="s">
+      <c r="E29" s="103" t="s">
         <v>401</v>
       </c>
-      <c r="F29" s="110"/>
-      <c r="G29" s="112"/>
-    </row>
-    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="108" t="s">
+      <c r="F29" s="104"/>
+      <c r="G29" s="106"/>
+    </row>
+    <row r="30" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A30" s="102" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="109" t="s">
+      <c r="B30" s="103" t="s">
         <v>367</v>
       </c>
-      <c r="C30" s="109">
+      <c r="C30" s="103">
         <v>3</v>
       </c>
-      <c r="D30" s="108" t="s">
+      <c r="D30" s="102" t="s">
         <v>63</v>
       </c>
-      <c r="E30" s="109" t="s">
+      <c r="E30" s="103" t="s">
         <v>402</v>
       </c>
-      <c r="F30" s="110"/>
-      <c r="G30" s="112"/>
-    </row>
-    <row r="31" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A31" s="108" t="s">
+      <c r="F30" s="104"/>
+      <c r="G30" s="106"/>
+    </row>
+    <row r="31" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A31" s="102" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="109" t="s">
+      <c r="B31" s="103" t="s">
         <v>368</v>
       </c>
-      <c r="C31" s="109">
+      <c r="C31" s="103">
         <v>3</v>
       </c>
-      <c r="D31" s="108" t="s">
+      <c r="D31" s="102" t="s">
         <v>65</v>
       </c>
-      <c r="E31" s="109" t="s">
+      <c r="E31" s="103" t="s">
         <v>403</v>
       </c>
-      <c r="F31" s="110"/>
-      <c r="G31" s="112"/>
-    </row>
-    <row r="32" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A32" s="108" t="s">
+      <c r="F31" s="104"/>
+      <c r="G31" s="106"/>
+    </row>
+    <row r="32" spans="1:10" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A32" s="102" t="s">
         <v>68</v>
       </c>
-      <c r="B32" s="109" t="s">
+      <c r="B32" s="103" t="s">
         <v>369</v>
       </c>
-      <c r="C32" s="109">
+      <c r="C32" s="103">
         <v>3</v>
       </c>
-      <c r="D32" s="113" t="s">
+      <c r="D32" s="107" t="s">
         <v>276</v>
       </c>
-      <c r="E32" s="109" t="s">
+      <c r="E32" s="103" t="s">
         <v>404</v>
       </c>
-      <c r="F32" s="110"/>
-      <c r="G32" s="112"/>
-    </row>
-    <row r="33" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A33" s="108" t="s">
+      <c r="F32" s="104"/>
+      <c r="G32" s="106"/>
+    </row>
+    <row r="33" spans="1:7" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A33" s="102" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="109" t="s">
+      <c r="B33" s="103" t="s">
         <v>370</v>
       </c>
-      <c r="C33" s="109">
+      <c r="C33" s="103">
         <v>3</v>
       </c>
-      <c r="D33" s="108" t="s">
+      <c r="D33" s="102" t="s">
         <v>277</v>
       </c>
-      <c r="E33" s="109" t="s">
+      <c r="E33" s="103" t="s">
         <v>405</v>
       </c>
-      <c r="F33" s="110"/>
-      <c r="G33" s="112"/>
-    </row>
-    <row r="34" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A34" s="108" t="s">
+      <c r="F33" s="104"/>
+      <c r="G33" s="106"/>
+    </row>
+    <row r="34" spans="1:7" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="102" t="s">
         <v>259</v>
       </c>
-      <c r="B34" s="109" t="s">
+      <c r="B34" s="103" t="s">
         <v>371</v>
       </c>
-      <c r="C34" s="109">
+      <c r="C34" s="103">
         <v>3</v>
       </c>
-      <c r="D34" s="108" t="s">
+      <c r="D34" s="102" t="s">
         <v>334</v>
       </c>
-      <c r="E34" s="109" t="s">
+      <c r="E34" s="103" t="s">
         <v>406</v>
       </c>
-      <c r="F34" s="110"/>
-      <c r="G34" s="112"/>
-    </row>
-    <row r="35" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A35" s="108" t="s">
+      <c r="F34" s="104"/>
+      <c r="G34" s="106"/>
+    </row>
+    <row r="35" spans="1:7" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A35" s="102" t="s">
         <v>268</v>
       </c>
-      <c r="B35" s="109" t="s">
+      <c r="B35" s="103" t="s">
         <v>372</v>
       </c>
-      <c r="C35" s="109">
+      <c r="C35" s="103">
         <v>3</v>
       </c>
-      <c r="D35" s="108" t="s">
+      <c r="D35" s="102" t="s">
         <v>335</v>
       </c>
-      <c r="E35" s="109" t="s">
+      <c r="E35" s="103" t="s">
         <v>407</v>
       </c>
-      <c r="F35" s="110"/>
-      <c r="G35" s="112"/>
-    </row>
-    <row r="36" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A36" s="108" t="s">
+      <c r="F35" s="104"/>
+      <c r="G35" s="106"/>
+    </row>
+    <row r="36" spans="1:7" ht="41.25" x14ac:dyDescent="0.2">
+      <c r="A36" s="102" t="s">
         <v>314</v>
       </c>
-      <c r="B36" s="109" t="s">
+      <c r="B36" s="103" t="s">
         <v>373</v>
       </c>
-      <c r="C36" s="109">
+      <c r="C36" s="103">
         <v>6</v>
       </c>
-      <c r="D36" s="110"/>
-      <c r="E36" s="112"/>
-      <c r="F36" s="110"/>
-    </row>
-    <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="108" t="s">
+      <c r="D36" s="104"/>
+      <c r="E36" s="106"/>
+      <c r="F36" s="104"/>
+    </row>
+    <row r="37" spans="1:7" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A37" s="102" t="s">
         <v>275</v>
       </c>
-      <c r="B37" s="109" t="s">
+      <c r="B37" s="103" t="s">
         <v>374</v>
       </c>
-      <c r="C37" s="109">
+      <c r="C37" s="103">
         <v>3</v>
       </c>
-      <c r="D37" s="110"/>
-      <c r="E37" s="112"/>
-      <c r="F37" s="110"/>
-    </row>
-    <row r="38" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A38" s="108" t="s">
+      <c r="D37" s="104"/>
+      <c r="E37" s="106"/>
+      <c r="F37" s="104"/>
+    </row>
+    <row r="38" spans="1:7" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A38" s="102" t="s">
         <v>281</v>
       </c>
-      <c r="B38" s="109" t="s">
+      <c r="B38" s="103" t="s">
         <v>375</v>
       </c>
-      <c r="C38" s="109">
+      <c r="C38" s="103">
         <v>6</v>
       </c>
-      <c r="D38" s="110"/>
-      <c r="E38" s="112"/>
-      <c r="F38" s="110"/>
-    </row>
-    <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="108" t="s">
+      <c r="D38" s="104"/>
+      <c r="E38" s="106"/>
+      <c r="F38" s="104"/>
+    </row>
+    <row r="39" spans="1:7" ht="27.75" x14ac:dyDescent="0.2">
+      <c r="A39" s="102" t="s">
         <v>292</v>
       </c>
-      <c r="B39" s="109" t="s">
+      <c r="B39" s="103" t="s">
         <v>376</v>
       </c>
-      <c r="C39" s="109">
+      <c r="C39" s="103">
         <v>3</v>
       </c>
-      <c r="D39" s="110"/>
-      <c r="E39" s="112"/>
-      <c r="F39" s="110"/>
+      <c r="D39" s="104"/>
+      <c r="E39" s="106"/>
+      <c r="F39" s="104"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4559,20 +4555,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D195C1D-DB02-1743-BBD2-99104C1FFD33}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="37.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="39.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="40.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.71875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.86328125" customWidth="1"/>
+    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.55859375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="37.26171875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7890625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="39.546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="34.16796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="40.0859375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>70</v>
       </c>
@@ -4601,7 +4597,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
         <v>219</v>
       </c>
@@ -4630,7 +4626,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>238</v>
       </c>
@@ -4659,7 +4655,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="81" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>88</v>
       </c>
@@ -4686,7 +4682,7 @@
       </c>
       <c r="I4" s="19"/>
     </row>
-    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>94</v>
       </c>
@@ -4713,7 +4709,7 @@
       </c>
       <c r="I5" s="19"/>
     </row>
-    <row r="6" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>98</v>
       </c>
@@ -4740,7 +4736,7 @@
       </c>
       <c r="I6" s="19"/>
     </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>103</v>
       </c>
@@ -4765,7 +4761,7 @@
       <c r="H7" s="16"/>
       <c r="I7" s="19"/>
     </row>
-    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>106</v>
       </c>
@@ -4788,7 +4784,7 @@
       <c r="H8" s="16"/>
       <c r="I8" s="19"/>
     </row>
-    <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="108" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>110</v>
       </c>
@@ -4811,7 +4807,7 @@
       <c r="H9" s="16"/>
       <c r="I9" s="19"/>
     </row>
-    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>329</v>
       </c>
@@ -4832,7 +4828,7 @@
       <c r="H10" s="16"/>
       <c r="I10" s="19"/>
     </row>
-    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="68.25" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>117</v>
       </c>
@@ -4851,7 +4847,7 @@
       <c r="H11" s="16"/>
       <c r="I11" s="19"/>
     </row>
-    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>118</v>
       </c>
@@ -4870,7 +4866,7 @@
       <c r="H12" s="16"/>
       <c r="I12" s="19"/>
     </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>121</v>
       </c>
@@ -4889,7 +4885,7 @@
       <c r="H13" s="16"/>
       <c r="I13" s="19"/>
     </row>
-    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>124</v>
       </c>
@@ -4908,7 +4904,7 @@
       <c r="H14" s="16"/>
       <c r="I14" s="19"/>
     </row>
-    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>128</v>
       </c>
@@ -4925,7 +4921,7 @@
       <c r="H15" s="16"/>
       <c r="I15" s="19"/>
     </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>130</v>
       </c>
@@ -4942,7 +4938,7 @@
       <c r="H16" s="16"/>
       <c r="I16" s="19"/>
     </row>
-    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>272</v>
       </c>
@@ -4959,7 +4955,7 @@
       <c r="H17" s="16"/>
       <c r="I17" s="19"/>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>132</v>
       </c>
@@ -4976,7 +4972,7 @@
       <c r="H18" s="16"/>
       <c r="I18" s="19"/>
     </row>
-    <row r="19" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>135</v>
       </c>
@@ -4993,7 +4989,7 @@
       <c r="H19" s="16"/>
       <c r="I19" s="19"/>
     </row>
-    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>137</v>
       </c>
@@ -5010,7 +5006,7 @@
       <c r="H20" s="16"/>
       <c r="I20" s="19"/>
     </row>
-    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="41.25" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>257</v>
       </c>
@@ -5027,7 +5023,7 @@
       <c r="H21" s="16"/>
       <c r="I21" s="19"/>
     </row>
-    <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>124</v>
       </c>
@@ -5044,7 +5040,7 @@
       <c r="H22" s="16"/>
       <c r="I22" s="19"/>
     </row>
-    <row r="23" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="54.75" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>128</v>
       </c>
@@ -5061,7 +5057,7 @@
       <c r="H23" s="16"/>
       <c r="I23" s="19"/>
     </row>
-    <row r="24" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>130</v>
       </c>
@@ -5078,7 +5074,7 @@
       <c r="H24" s="16"/>
       <c r="I24" s="19"/>
     </row>
-    <row r="25" spans="1:9" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="42" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>272</v>
       </c>
@@ -5104,13 +5100,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{920DF489-FE6D-4819-BD1A-323DFAE597A3}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="30.66796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="39"/>
       <c r="B1" s="33" t="s">
         <v>142</v>
@@ -5134,7 +5130,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="41" t="s">
         <v>148</v>
       </c>
@@ -5160,7 +5156,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="41" t="s">
         <v>149</v>
       </c>
@@ -5186,7 +5182,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="41" t="s">
         <v>150</v>
       </c>
@@ -5212,7 +5208,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
         <v>151</v>
       </c>
@@ -5238,7 +5234,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="64" t="s">
         <v>152</v>
       </c>
@@ -5264,7 +5260,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
         <v>153</v>
       </c>
@@ -5290,7 +5286,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="62" t="s">
         <v>202</v>
       </c>
@@ -5316,7 +5312,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="31" t="s">
         <v>203</v>
       </c>
@@ -5339,7 +5335,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="63" t="s">
         <v>204</v>
       </c>
@@ -5362,12 +5358,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>228</v>
       </c>
@@ -5390,7 +5386,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
         <v>207</v>
@@ -5411,7 +5407,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
         <v>323</v>
@@ -5432,7 +5428,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
         <v>326</v>
@@ -5453,7 +5449,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -5462,7 +5458,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>229</v>
       </c>
@@ -5488,7 +5484,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="2" t="s">
         <v>329</v>
@@ -5512,7 +5508,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="2" t="s">
         <v>207</v>
@@ -5533,7 +5529,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="s">
@@ -5552,7 +5548,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="2"/>
       <c r="D22" s="2" t="s">
@@ -5560,7 +5556,7 @@
       </c>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="D23" s="2"/>
@@ -5568,7 +5564,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>230</v>
       </c>
@@ -5594,7 +5590,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="2" t="s">
         <v>118</v>
@@ -5618,7 +5614,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="2" t="s">
         <v>298</v>
@@ -5642,7 +5638,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2" t="s">
@@ -5659,7 +5655,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -5671,7 +5667,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -5683,7 +5679,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -5692,7 +5688,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -5700,7 +5696,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -5708,7 +5704,7 @@
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -5716,7 +5712,7 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -5724,7 +5720,7 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -5732,7 +5728,7 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -5740,7 +5736,7 @@
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -5748,7 +5744,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -5756,7 +5752,7 @@
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -5764,7 +5760,7 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -5772,7 +5768,7 @@
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -5780,7 +5776,7 @@
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -5788,7 +5784,7 @@
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -5796,7 +5792,7 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -5804,7 +5800,7 @@
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48" s="3"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -5812,7 +5808,7 @@
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -5826,21 +5822,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4430D7D8-35BC-4E32-9DE8-E2E435ADAAA0}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="36" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="37.5" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="6" width="30.7109375" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="6" width="30.66796875" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="9.14453125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="113" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="105"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="115"/>
     </row>
     <row r="2" spans="1:6" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="99" t="s">
@@ -5969,11 +5965,11 @@
       <c r="B8" s="76" t="s">
         <v>158</v>
       </c>
-      <c r="C8" s="100" t="s">
+      <c r="C8" s="110" t="s">
         <v>159</v>
       </c>
-      <c r="D8" s="101"/>
-      <c r="E8" s="102"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="112"/>
       <c r="F8" s="96">
         <v>10</v>
       </c>
@@ -6052,66 +6048,66 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CEB427C-0CB4-4E8D-8367-36F6DD891282}">
   <dimension ref="A1:CA6"/>
-  <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="19.7734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" style="31"/>
-    <col min="2" max="2" width="19.7109375" style="43"/>
-    <col min="4" max="4" width="19.7109375" style="31"/>
-    <col min="6" max="6" width="19.7109375" style="31"/>
-    <col min="8" max="8" width="19.7109375" style="31"/>
-    <col min="10" max="10" width="19.7109375" style="31"/>
-    <col min="12" max="12" width="19.7109375" style="31"/>
-    <col min="14" max="14" width="19.7109375" style="31"/>
-    <col min="16" max="16" width="19.7109375" style="31"/>
-    <col min="18" max="18" width="19.7109375" style="31"/>
-    <col min="20" max="20" width="19.7109375" style="31"/>
-    <col min="22" max="22" width="19.7109375" style="31"/>
-    <col min="24" max="24" width="19.7109375" style="31"/>
-    <col min="26" max="26" width="19.7109375" style="31"/>
-    <col min="28" max="28" width="19.7109375" style="31"/>
-    <col min="30" max="30" width="19.7109375" style="49"/>
-    <col min="31" max="32" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.7109375" customWidth="1"/>
-    <col min="42" max="42" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="19.7109375" style="49" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="19.7109375" style="49" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="19.7109375" style="31"/>
-    <col min="63" max="63" width="19.7109375" style="31"/>
-    <col min="65" max="65" width="19.7109375" style="31"/>
-    <col min="67" max="67" width="19.7109375" style="31"/>
-    <col min="69" max="70" width="19.7109375" style="31"/>
-    <col min="71" max="71" width="19.7109375" style="43"/>
-    <col min="73" max="73" width="19.7109375" style="31"/>
-    <col min="75" max="75" width="19.7109375" style="31"/>
-    <col min="77" max="77" width="19.7109375" style="31"/>
-    <col min="79" max="79" width="19.7109375" style="31"/>
+    <col min="1" max="1" width="19.7734375" style="31"/>
+    <col min="2" max="2" width="19.7734375" style="43"/>
+    <col min="4" max="4" width="19.7734375" style="31"/>
+    <col min="6" max="6" width="19.7734375" style="31"/>
+    <col min="8" max="8" width="19.7734375" style="31"/>
+    <col min="10" max="10" width="19.7734375" style="31"/>
+    <col min="12" max="12" width="19.7734375" style="31"/>
+    <col min="14" max="14" width="19.7734375" style="31"/>
+    <col min="16" max="16" width="19.7734375" style="31"/>
+    <col min="18" max="18" width="19.7734375" style="31"/>
+    <col min="20" max="20" width="19.7734375" style="31"/>
+    <col min="22" max="22" width="19.7734375" style="31"/>
+    <col min="24" max="24" width="19.7734375" style="31"/>
+    <col min="26" max="26" width="19.7734375" style="31"/>
+    <col min="28" max="28" width="19.7734375" style="31"/>
+    <col min="30" max="30" width="19.7734375" style="49"/>
+    <col min="31" max="32" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.7734375" customWidth="1"/>
+    <col min="42" max="42" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="19.7734375" style="49" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="19.7734375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.7734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="19.7734375" style="49" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="19.7734375" style="31"/>
+    <col min="63" max="63" width="19.7734375" style="31"/>
+    <col min="65" max="65" width="19.7734375" style="31"/>
+    <col min="67" max="67" width="19.7734375" style="31"/>
+    <col min="69" max="70" width="19.7734375" style="31"/>
+    <col min="71" max="71" width="19.7734375" style="43"/>
+    <col min="73" max="73" width="19.7734375" style="31"/>
+    <col min="75" max="75" width="19.7734375" style="31"/>
+    <col min="77" max="77" width="19.7734375" style="31"/>
+    <col min="79" max="79" width="19.7734375" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" s="47" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:79" s="47" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="45" t="str">
         <f>Cards!A2</f>
         <v>Fillibuster</v>
@@ -6398,7 +6394,7 @@
       <c r="BY1" s="45"/>
       <c r="CA1" s="45"/>
     </row>
-    <row r="2" spans="1:79" s="70" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:79" s="70" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="71" t="str">
         <f>Cards!B2</f>
         <v>Move the deliberated Law one additional place back in the queue for each card level during Postpone</v>
@@ -6685,7 +6681,7 @@
       <c r="BY2" s="71"/>
       <c r="CA2" s="71"/>
     </row>
-    <row r="3" spans="1:79" s="47" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:79" s="47" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="45" t="str">
         <f>Cards!D2</f>
         <v>Full Coffers</v>
@@ -6969,7 +6965,7 @@
       <c r="BY3" s="45"/>
       <c r="CA3" s="45"/>
     </row>
-    <row r="4" spans="1:79" s="52" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:79" s="52" customFormat="1" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="50" t="str">
         <f>Cards!E2</f>
         <v>The Royal Bank must have at least one Coin per card level or all Players suffer sanctions on Undermarket Actions</v>
@@ -7253,7 +7249,7 @@
       <c r="BY4" s="50"/>
       <c r="CA4" s="50"/>
     </row>
-    <row r="5" spans="1:79" s="56" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:79" s="56" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="54" t="str">
         <f>Cards!F2</f>
         <v>Fickle Mercenaries</v>
@@ -7533,7 +7529,7 @@
       <c r="BY5" s="54"/>
       <c r="CA5" s="54"/>
     </row>
-    <row r="6" spans="1:79" s="52" customFormat="1" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:79" s="52" customFormat="1" ht="69" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="e">
         <f>Cards!#REF!</f>
         <v>#REF!</v>
@@ -7822,16 +7818,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BDA35E-BFC3-134A-A064-89D65A8B31CF}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.50390625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.10546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.22265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>180</v>
       </c>
@@ -7848,7 +7844,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>161</v>
       </c>
@@ -7863,7 +7859,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>162</v>
       </c>
@@ -7878,7 +7874,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>163</v>
       </c>
@@ -7893,7 +7889,7 @@
         <v>30.75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>164</v>
       </c>
@@ -7905,7 +7901,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>176</v>
       </c>
@@ -7920,7 +7916,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>165</v>
       </c>
@@ -7935,7 +7931,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>166</v>
       </c>
@@ -7950,7 +7946,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>167</v>
       </c>
@@ -7965,7 +7961,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>168</v>
       </c>
@@ -7980,7 +7976,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>169</v>
       </c>
@@ -7995,7 +7991,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>170</v>
       </c>
@@ -8010,7 +8006,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>171</v>
       </c>
@@ -8025,7 +8021,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>172</v>
       </c>
@@ -8036,7 +8032,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>173</v>
       </c>
@@ -8047,7 +8043,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>174</v>
       </c>
@@ -8058,7 +8054,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>175</v>
       </c>
@@ -8069,7 +8065,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>179</v>
       </c>
@@ -8081,7 +8077,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>178</v>
       </c>
@@ -8093,7 +8089,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>177</v>
       </c>
@@ -8105,7 +8101,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>190</v>
       </c>
@@ -8125,24 +8121,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC83F89-2724-CA43-A519-59213A612B31}">
   <dimension ref="A1:U55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24" style="73" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="11.42578125" style="75" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" style="75" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" style="75" bestFit="1" customWidth="1"/>
-    <col min="12" max="19" width="11.85546875" style="75" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" style="75" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.9453125" style="73" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.72265625" customWidth="1"/>
+    <col min="4" max="4" width="8.33984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.27734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5078125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.97265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.43359375" style="75" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.22265625" style="75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.43359375" style="75" bestFit="1" customWidth="1"/>
+    <col min="12" max="19" width="11.8359375" style="75" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.9140625" style="75" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.5078125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>239</v>
       </c>
@@ -8207,7 +8203,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="73">
         <v>46075</v>
       </c>
@@ -8251,7 +8247,7 @@
         <v>0.92638888888888893</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="73">
         <v>46089</v>
       </c>
@@ -8307,7 +8303,7 @@
         <v>0.86527777777777781</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="73">
         <v>46105</v>
       </c>
@@ -8360,7 +8356,7 @@
         <v>0.92777777777777781</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="73">
         <v>46118</v>
       </c>
@@ -8413,7 +8409,7 @@
         <v>0.9194444444444444</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="73">
         <v>46124</v>
       </c>
@@ -8457,7 +8453,7 @@
         <v>0.74583333333333335</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="73">
         <v>46131</v>
       </c>
@@ -8510,7 +8506,7 @@
         <v>0.70277777777777772</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="73">
         <v>46138</v>
       </c>
@@ -8554,7 +8550,7 @@
         <v>0.69513888888888886</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="73">
         <v>46145</v>
       </c>
@@ -8607,7 +8603,7 @@
         <v>0.71666666666666667</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="73">
         <v>46152</v>
       </c>
@@ -8657,7 +8653,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="73">
         <v>46158</v>
       </c>
@@ -8710,7 +8706,7 @@
         <v>0.99236111111111114</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="73">
         <v>46215</v>
       </c>
@@ -8769,7 +8765,7 @@
         <v>0.73888888888888893</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="73">
         <v>46247</v>
       </c>
@@ -8822,7 +8818,7 @@
         <v>0.9458333333333333</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C14" s="74" t="b">
         <v>0</v>
       </c>
@@ -8830,7 +8826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C15" s="74" t="b">
         <v>0</v>
       </c>
@@ -8838,7 +8834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C16" s="74" t="b">
         <v>0</v>
       </c>
@@ -8846,7 +8842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C17" s="74" t="b">
         <v>0</v>
       </c>
@@ -8854,7 +8850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C18" s="74" t="b">
         <v>0</v>
       </c>
@@ -8862,7 +8858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C19" s="74" t="b">
         <v>0</v>
       </c>
@@ -8870,7 +8866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C20" s="74" t="b">
         <v>0</v>
       </c>
@@ -8878,7 +8874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C21" s="74" t="b">
         <v>0</v>
       </c>
@@ -8886,7 +8882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C22" s="74" t="b">
         <v>0</v>
       </c>
@@ -8894,7 +8890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C23" s="74" t="b">
         <v>0</v>
       </c>
@@ -8902,7 +8898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C24" s="74" t="b">
         <v>0</v>
       </c>
@@ -8910,7 +8906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C25" s="74" t="b">
         <v>0</v>
       </c>
@@ -8918,7 +8914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C26" s="74" t="b">
         <v>0</v>
       </c>
@@ -8926,7 +8922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C27" s="74" t="b">
         <v>0</v>
       </c>
@@ -8934,7 +8930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C28" s="74" t="b">
         <v>0</v>
       </c>
@@ -8942,7 +8938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C29" s="74" t="b">
         <v>0</v>
       </c>
@@ -8950,7 +8946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C30" s="74" t="b">
         <v>0</v>
       </c>
@@ -8958,7 +8954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C31" s="74" t="b">
         <v>0</v>
       </c>
@@ -8966,7 +8962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C32" s="74" t="b">
         <v>0</v>
       </c>
@@ -8974,7 +8970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C33" s="74" t="b">
         <v>0</v>
       </c>
@@ -8982,7 +8978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C34" s="74" t="b">
         <v>0</v>
       </c>
@@ -8990,7 +8986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C35" s="74" t="b">
         <v>0</v>
       </c>
@@ -8998,7 +8994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C36" s="74" t="b">
         <v>0</v>
       </c>
@@ -9006,7 +9002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C37" s="74" t="b">
         <v>0</v>
       </c>
@@ -9014,7 +9010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C38" s="74" t="b">
         <v>0</v>
       </c>
@@ -9022,7 +9018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C39" s="74" t="b">
         <v>0</v>
       </c>
@@ -9030,7 +9026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C40" s="74" t="b">
         <v>0</v>
       </c>
@@ -9038,7 +9034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C41" s="74" t="b">
         <v>0</v>
       </c>
@@ -9046,7 +9042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C42" s="74" t="b">
         <v>0</v>
       </c>
@@ -9054,7 +9050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C43" s="74" t="b">
         <v>0</v>
       </c>
@@ -9062,7 +9058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C44" s="74" t="b">
         <v>0</v>
       </c>
@@ -9070,7 +9066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C45" s="74" t="b">
         <v>0</v>
       </c>
@@ -9078,7 +9074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C46" s="74" t="b">
         <v>0</v>
       </c>
@@ -9086,7 +9082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C47" s="74" t="b">
         <v>0</v>
       </c>
@@ -9094,7 +9090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C48" s="74" t="b">
         <v>0</v>
       </c>
@@ -9102,7 +9098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C49" s="74" t="b">
         <v>0</v>
       </c>
@@ -9110,7 +9106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C50" s="74" t="b">
         <v>0</v>
       </c>
@@ -9118,7 +9114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C51" s="74" t="b">
         <v>0</v>
       </c>
@@ -9126,7 +9122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C52" s="74" t="b">
         <v>0</v>
       </c>
@@ -9134,7 +9130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C53" s="74" t="b">
         <v>0</v>
       </c>
@@ -9142,7 +9138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C54" s="74" t="b">
         <v>0</v>
       </c>
@@ -9150,7 +9146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C55" s="74" t="b">
         <v>0</v>
       </c>

</xml_diff>